<commit_message>
Inicio da implementação dos requests para o get expenses
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -3,12 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Constants" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Assets" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ProcessVariables" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -18,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="119">
   <si>
     <t>Name</t>
   </si>
@@ -109,16 +110,10 @@
     <t>obligationDateStart</t>
   </si>
   <si>
-    <t>20/01/2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">Data inicial do range de datas que deve abranger a data de vencimento da obrigação em questão, se não estiver definida nenhuma data nessa variável, o processo define o primeiro e o ultimo dia do mês como as datas de inicio e fim do range.</t>
   </si>
   <si>
     <t>obligationDateEnd</t>
-  </si>
-  <si>
-    <t>01/02/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Data final do range de datas que deve abranger a data de vencimento da obrigação em questão, se não estiver definida nenhuma data nessa variável, o processo define o primeiro e o ultimo dia do mês como as datas de inicio e fim do range.</t>
@@ -163,6 +158,9 @@
     <t>obligationDebugCompanyId</t>
   </si>
   <si>
+    <t>7a8d0889-71e5-4dab-9ec2-734bf7c46734</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -196,7 +194,7 @@
     <t>discordIntegrationWebhook</t>
   </si>
   <si>
-    <t>https://discord.com/api/webhooks/1480622360888348782/kdyzsfcL0x-dRAhSlVzLWuLgtZVv9F-nG_agjagkrFjNF1RSGt6oi5oVvIyV8dKBl_c7</t>
+    <t>https://discord.com/api/webhooks/1481613724102951093/SGz4BHIRTn3KXmhEQP1AgLaNKWGs4-LvW_bYP8tfs_xuurusg2LunnC13mx0I9LRq07B</t>
   </si>
   <si>
     <t xml:space="preserve">Webhook para integração e envio de mensagens e prints quando a automação falhar.</t>
@@ -214,7 +212,40 @@
     <t xml:space="preserve">O erro ocorreu na seguinte empresa:</t>
   </si>
   <si>
-    <t xml:space="preserve">PROCESS TIMEOUTS</t>
+    <t>MaxRetryNumber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Must be 0 if working with Orchestrator queues. If &gt; 0, the robot will retry the same transaction which failed with a system exception. Must be an integer value.</t>
+  </si>
+  <si>
+    <t>MaxConsecutiveSystemExceptions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The number of consecutive system exceptions allowed. If MaxConsecutiveSystemExceptions is reached, the job is stopped. To disable this feature, set the value to 0. </t>
+  </si>
+  <si>
+    <t>ExScreenshotsFolderPath</t>
+  </si>
+  <si>
+    <t>Exceptions_Screenshots</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Where to save exceptions screenshots - can be a full or a relative path.</t>
+  </si>
+  <si>
+    <t>RetryNumberGetTransactionItem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The number of times Get Transaction Item activity is retried in case of an exception. Must be an integer &gt;= 1.</t>
+  </si>
+  <si>
+    <t>RetryNumberSetTransactionStatus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The number of times Set transaction status activity is retried in case of an exception. Must be an integer &gt;= 1. </t>
+  </si>
+  <si>
+    <t>TIMEOUTS</t>
   </si>
   <si>
     <t>login_at_domonio_timeout</t>
@@ -241,40 +272,7 @@
     <t xml:space="preserve">Delay after padrão das atividades do processo</t>
   </si>
   <si>
-    <t>MaxRetryNumber</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Must be 0 if working with Orchestrator queues. If &gt; 0, the robot will retry the same transaction which failed with a system exception. Must be an integer value.</t>
-  </si>
-  <si>
-    <t>MaxConsecutiveSystemExceptions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The number of consecutive system exceptions allowed. If MaxConsecutiveSystemExceptions is reached, the job is stopped. To disable this feature, set the value to 0. </t>
-  </si>
-  <si>
-    <t>ExScreenshotsFolderPath</t>
-  </si>
-  <si>
-    <t>Exceptions_Screenshots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Where to save exceptions screenshots - can be a full or a relative path.</t>
-  </si>
-  <si>
-    <t>RetryNumberGetTransactionItem</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The number of times Get Transaction Item activity is retried in case of an exception. Must be an integer &gt;= 1.</t>
-  </si>
-  <si>
-    <t>RetryNumberSetTransactionStatus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The number of times Set transaction status activity is retried in case of an exception. Must be an integer &gt;= 1. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Success message</t>
+    <t xml:space="preserve">SUCCESS MESSAGE</t>
   </si>
   <si>
     <t>LogMessage_Success</t>
@@ -361,6 +359,15 @@
     <t xml:space="preserve">Faltam informações para a execução da automação na presente empresa. Favor verificar.</t>
   </si>
   <si>
+    <t>ExceptionMessage_AnyExpense</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não existem despesas na empresa em questão para o periodo determinado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso não existam despesas na empresa em questão.</t>
+  </si>
+  <si>
     <t>Asset</t>
   </si>
   <si>
@@ -404,6 +411,60 @@
   </si>
   <si>
     <t xml:space="preserve">Codigo do contador dentro do domínio</t>
+  </si>
+  <si>
+    <t>mainPath</t>
+  </si>
+  <si>
+    <t xml:space="preserve">\\192.168.8.8\Razonet\18- OPERAÇÃO RAZONET\01- ROTINAS AUTOMATICAS\04- LANÇAMENTOS CONTÁBEIS\AUTOMACAO\LANÇAMENTOS DESPESAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Endereço onde serão alocados os arquivos de importação e relatórios de erros de importação do processo</t>
+  </si>
+  <si>
+    <t>GetExpensesSettings</t>
+  </si>
+  <si>
+    <t>expensesUrl</t>
+  </si>
+  <si>
+    <t>https://app.razonet.com.br/integration/v1/company_expenses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Url para requisição das despesas no backoffice.</t>
+  </si>
+  <si>
+    <t>getExpenses_timeout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Timeout do request.</t>
+  </si>
+  <si>
+    <t>getExpenses_perPage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numero de despesas apresentadas em cada página da paginação do json.</t>
+  </si>
+  <si>
+    <t>getExpenses_contentType</t>
+  </si>
+  <si>
+    <t>application/json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo de conteúdo que será aceitado no request</t>
+  </si>
+  <si>
+    <t>getExpenses_dateStart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inicio do range de datas que abrange a data de vencimento das despesas que irão ser importadas. Deve estar no formato "dd/MM/yyyy" e só deve existir caso o getExpenses_dateEnd existir também.</t>
+  </si>
+  <si>
+    <t>getExpenses_dateEnd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fim do range de datas que abrange a data de vencimento das despesas que irão ser importadas. Deve estar no formato "dd/MM/yyyy" e só deve existir caso o getExpenses_dateStart existir também. Deve ser posterior ao getExpenses_dateStart</t>
   </si>
 </sst>
 </file>
@@ -423,12 +484,12 @@
     </font>
     <font>
       <b/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
@@ -445,12 +506,18 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0"/>
+        <bgColor theme="1" tint="0"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -466,20 +533,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.099978637043366805"/>
+        <bgColor theme="2" tint="-0.099978637043366805"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor theme="8" tint="0.59999389629810485"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor theme="9" tint="0.59999389629810485"/>
+        <fgColor theme="0" tint="0"/>
+        <bgColor theme="0" tint="0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.099978637043366805"/>
-        <bgColor theme="2" tint="-0.099978637043366805"/>
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor theme="9" tint="0.59999389629810485"/>
       </patternFill>
     </fill>
     <fill>
@@ -501,7 +574,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -524,11 +597,20 @@
       </bottom>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="53">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -540,58 +622,50 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="3" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf fontId="3" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="3" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="4" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="2" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="4" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -608,27 +682,71 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="5" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="5" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="5" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
     <xf fontId="5" fillId="9" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
+    <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="5" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="5" fillId="11" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="7" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="4" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1143,7 +1261,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="9.140625"/>
     <col customWidth="1" min="2" max="2" width="45.140625"/>
-    <col customWidth="1" min="3" max="3" style="1" width="43.8515625"/>
+    <col customWidth="1" min="3" max="3" style="1" width="60.7109375"/>
     <col customWidth="1" min="4" max="4" width="84.57421875"/>
     <col customWidth="1" min="5" max="5" width="7.00390625"/>
     <col customWidth="1" min="6" max="27" width="8.7109375"/>
@@ -1194,245 +1312,214 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="28.5">
+    <row r="3" ht="17.399999999999999" customHeight="1">
+      <c r="A3" s="5"/>
       <c r="B3" s="5"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="4"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="7"/>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="11"/>
     </row>
     <row r="5" ht="27" customHeight="1">
-      <c r="A5" s="6"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="9"/>
+      <c r="A5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="11"/>
     </row>
     <row r="6" ht="27" customHeight="1">
-      <c r="A6" s="6"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="9"/>
+      <c r="A6" s="8"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="11"/>
     </row>
     <row r="7" ht="27" customHeight="1">
-      <c r="A7" s="6"/>
-      <c r="B7" s="10" t="s">
+      <c r="A7" s="8"/>
+      <c r="B7" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="8" t="b">
+      <c r="C7" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="8" ht="26.399999999999999" customHeight="1">
+    <row r="8" ht="17.399999999999999" customHeight="1">
+      <c r="A8" s="5"/>
       <c r="B8" s="5"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="4"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="7"/>
     </row>
     <row r="9" ht="31.199999999999999" customHeight="1">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="13" t="s">
+      <c r="C9" s="14"/>
+      <c r="D9" s="15" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" ht="33.600000000000001" customHeight="1">
-      <c r="A10" s="11"/>
-      <c r="B10" s="12" t="s">
+      <c r="A10" s="13"/>
+      <c r="B10" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="14" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="11" ht="43.200000000000003" customHeight="1">
-      <c r="A11" s="11"/>
-      <c r="B11" s="12" t="s">
+      <c r="A11" s="13"/>
+      <c r="B11" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="16"/>
+      <c r="D11" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="13" t="s">
+    </row>
+    <row r="12" ht="61.200000000000003" customHeight="1">
+      <c r="A12" s="13"/>
+      <c r="B12" s="14" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="12" ht="61.200000000000003" customHeight="1">
-      <c r="A12" s="11"/>
-      <c r="B12" s="12" t="s">
+      <c r="C12" s="17"/>
+      <c r="D12" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="15" t="s">
+    </row>
+    <row r="13" ht="28.800000000000001" customHeight="1">
+      <c r="A13" s="13"/>
+      <c r="B13" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="C13" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" s="14"/>
+    </row>
+    <row r="14" ht="28.800000000000001" customHeight="1">
+      <c r="A14" s="13"/>
+      <c r="B14" s="14" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="13" ht="28.800000000000001" customHeight="1">
-      <c r="A13" s="11"/>
-      <c r="B13" s="12" t="s">
+      <c r="C14" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D14" s="14"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="13"/>
+      <c r="B15" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="D13" s="12"/>
-    </row>
-    <row r="14" ht="28.800000000000001" customHeight="1">
-      <c r="A14" s="11"/>
-      <c r="B14" s="12" t="s">
+      <c r="C15" s="19"/>
+      <c r="D15" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="12" t="b">
-        <v>0</v>
-      </c>
-      <c r="D14" s="12"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="11"/>
-      <c r="B15" s="16" t="s">
+    </row>
+    <row r="16" ht="34.799999999999997" customHeight="1">
+      <c r="A16" s="13"/>
+      <c r="B16" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="18" t="s">
+      <c r="C16" s="14" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="16" ht="34.799999999999997" customHeight="1">
-      <c r="A16" s="11"/>
-      <c r="B16" s="16" t="s">
+      <c r="D16" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="12"/>
-      <c r="D16" s="18" t="s">
+    </row>
+    <row r="17" ht="17.399999999999999" customHeight="1">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="5"/>
+    </row>
+    <row r="18" ht="46.799999999999997" customHeight="1">
+      <c r="A18" s="21" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="17" ht="14.25">
-      <c r="C17" s="1"/>
-    </row>
-    <row r="18" ht="46.799999999999997" customHeight="1">
-      <c r="A18" s="19" t="s">
+      <c r="B18" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="C18" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="D18" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="20" t="s">
+    </row>
+    <row r="19" ht="46.799999999999997" customHeight="1">
+      <c r="A19" s="21"/>
+      <c r="B19" s="15" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="19" ht="46.799999999999997" customHeight="1">
-      <c r="A19" s="19"/>
-      <c r="B19" s="22" t="s">
+      <c r="C19" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="D19" s="14"/>
+    </row>
+    <row r="20" ht="43.200000000000003" customHeight="1">
+      <c r="A20" s="21"/>
+      <c r="B20" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="D19" s="20"/>
-    </row>
-    <row r="20" ht="43.200000000000003" customHeight="1">
-      <c r="A20" s="19"/>
-      <c r="B20" s="22" t="s">
+      <c r="C20" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="D20" s="20"/>
-    </row>
-    <row r="21" ht="28.800000000000001" customHeight="1"/>
-    <row r="22" ht="27.75" customHeight="1">
-      <c r="A22" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="B22" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="C22" s="26">
-        <v>30000</v>
-      </c>
-      <c r="D22" s="27" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="23" ht="29.399999999999999" customHeight="1">
-      <c r="A23" s="24"/>
-      <c r="B23" s="25" t="s">
-        <v>38</v>
-      </c>
-      <c r="C23" s="26">
-        <v>20000</v>
-      </c>
-      <c r="D23" s="27" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="24" ht="29.399999999999999" customHeight="1">
-      <c r="A24" s="24"/>
-      <c r="B24" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="C24" s="26">
-        <v>0</v>
-      </c>
-      <c r="D24" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="25" ht="29.399999999999999" customHeight="1">
-      <c r="A25" s="24"/>
-      <c r="B25" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="C25" s="26">
-        <v>0</v>
-      </c>
-      <c r="D25" s="25" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="26" ht="29.399999999999999" customHeight="1">
-      <c r="A26" s="24"/>
-      <c r="B26" s="25"/>
-      <c r="C26" s="26"/>
-      <c r="D26" s="25"/>
-    </row>
-    <row r="27" ht="28.800000000000001" customHeight="1">
-      <c r="A27" s="24"/>
-      <c r="B27" s="25"/>
-      <c r="C27" s="26"/>
-      <c r="D27" s="25"/>
+      <c r="D20" s="14"/>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="C21" s="1"/>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="C22" s="1"/>
+    </row>
+    <row r="23" ht="14.25">
+      <c r="C23" s="1"/>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="C24" s="1"/>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="C25" s="1"/>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="C26" s="1"/>
+    </row>
+    <row r="27" ht="14.25">
+      <c r="C27" s="1"/>
+    </row>
+    <row r="28" ht="14.25">
+      <c r="C28" s="1"/>
+    </row>
+    <row r="29" ht="14.25">
+      <c r="C29" s="1"/>
+    </row>
+    <row r="34" ht="14.25">
+      <c r="C34" s="1"/>
     </row>
   </sheetData>
-  <sortState ref="B11:C23" columnSort="0">
-    <sortCondition sortBy="value" descending="0" ref="A11:A23"/>
+  <sortState ref="B11:C20" columnSort="0">
+    <sortCondition sortBy="value" descending="0" ref="A11:A20"/>
   </sortState>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A4:A7"/>
     <mergeCell ref="A9:A16"/>
     <mergeCell ref="A18:A20"/>
-    <mergeCell ref="A22:A27"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C18"/>
@@ -1449,20 +1536,20 @@
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8.00390625"/>
-    <col customWidth="1" min="2" max="2" style="28" width="52.140625"/>
-    <col bestFit="1" customWidth="1" min="3" max="3" style="29" width="63.11328125"/>
-    <col customWidth="1" min="4" max="4" style="29" width="75.42578125"/>
+    <col customWidth="1" min="2" max="2" style="24" width="52.140625"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" style="25" width="63.11328125"/>
+    <col customWidth="1" min="4" max="4" style="25" width="84.140625"/>
     <col customWidth="1" min="5" max="27" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="D1" s="27" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="2"/>
@@ -1490,340 +1577,399 @@
       <c r="AA1" s="2"/>
     </row>
     <row r="2" ht="28.5">
-      <c r="A2" s="32"/>
-      <c r="B2" s="33" t="s">
+      <c r="A2" s="28"/>
+      <c r="B2" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="30">
+        <v>1</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" ht="42.75">
+      <c r="A3" s="28"/>
+      <c r="B3" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="30">
+        <v>3</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" ht="27" customHeight="1">
+      <c r="A4" s="28"/>
+      <c r="B4" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" ht="28.5">
+      <c r="A5" s="28"/>
+      <c r="B5" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="30">
+        <v>2</v>
+      </c>
+      <c r="D5" s="30" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" ht="28.5">
+      <c r="A6" s="28"/>
+      <c r="B6" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="30">
+        <v>2</v>
+      </c>
+      <c r="D6" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="34">
-        <v>1</v>
-      </c>
-      <c r="D2" s="34" t="s">
+    </row>
+    <row r="7" s="31" customFormat="1" ht="17.399999999999999" customHeight="1">
+      <c r="A7" s="5"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+    </row>
+    <row r="8" ht="39.75" customHeight="1">
+      <c r="A8" s="34" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="3" ht="42.75">
-      <c r="A3" s="32"/>
-      <c r="B3" s="33" t="s">
+      <c r="B8" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="34">
-        <v>3</v>
-      </c>
-      <c r="D3" s="34" t="s">
+      <c r="C8" s="35">
+        <v>30000</v>
+      </c>
+      <c r="D8" s="15" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="32"/>
-      <c r="B4" s="33" t="s">
+    <row r="9" ht="39.75" customHeight="1">
+      <c r="A9" s="36"/>
+      <c r="B9" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="C9" s="35">
+        <v>20000</v>
+      </c>
+      <c r="D9" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="34" t="s">
+    </row>
+    <row r="10" ht="39.75" customHeight="1">
+      <c r="A10" s="36"/>
+      <c r="B10" s="14" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="5" ht="28.5">
-      <c r="A5" s="32"/>
-      <c r="B5" s="33" t="s">
+      <c r="C10" s="35">
+        <v>0</v>
+      </c>
+      <c r="D10" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="34">
-        <v>2</v>
-      </c>
-      <c r="D5" s="34" t="s">
+    </row>
+    <row r="11" ht="39.75" customHeight="1">
+      <c r="A11" s="36"/>
+      <c r="B11" s="14" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="6" ht="28.5">
-      <c r="A6" s="32"/>
-      <c r="B6" s="33" t="s">
+      <c r="C11" s="35">
+        <v>0</v>
+      </c>
+      <c r="D11" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="34">
-        <v>2</v>
-      </c>
-      <c r="D6" s="34" t="s">
+    </row>
+    <row r="12" ht="17.399999999999999" customHeight="1">
+      <c r="A12" s="5"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+    </row>
+    <row r="13" ht="22.800000000000001" customHeight="1">
+      <c r="A13" s="37" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="7" ht="39.75" customHeight="1">
-      <c r="B7" s="28"/>
-      <c r="C7" s="29"/>
-      <c r="D7" s="29"/>
-    </row>
-    <row r="8" ht="28.5">
-      <c r="A8" s="35" t="s">
+      <c r="B13" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="C13" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="D13" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="D8" s="34" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" ht="28.199999999999999" customHeight="1">
-      <c r="A9" s="35"/>
-      <c r="B9" s="33"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-    </row>
-    <row r="10" ht="28.199999999999999" customHeight="1">
-      <c r="A10" s="35"/>
-      <c r="B10" s="33"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-    </row>
-    <row r="11" ht="27" customHeight="1">
-      <c r="A11" s="35"/>
-      <c r="B11" s="33"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-    </row>
-    <row r="12" ht="27" customHeight="1">
-      <c r="A12" s="35"/>
-      <c r="B12" s="33"/>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-    </row>
-    <row r="13" ht="27" customHeight="1">
-      <c r="A13" s="35"/>
-      <c r="B13" s="33"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-    </row>
-    <row r="14" ht="40.5" customHeight="1">
-      <c r="A14" s="36"/>
-      <c r="B14" s="28"/>
-      <c r="C14" s="29"/>
-      <c r="D14" s="29"/>
-    </row>
-    <row r="15" ht="27" customHeight="1">
-      <c r="A15" s="37" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="33" t="s">
-        <v>60</v>
-      </c>
-      <c r="C15" s="34" t="s">
-        <v>61</v>
-      </c>
-      <c r="D15" s="34" t="s">
-        <v>62</v>
-      </c>
+    </row>
+    <row r="14" ht="28.199999999999999" customHeight="1">
+      <c r="A14" s="37"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+    </row>
+    <row r="15" ht="28.199999999999999" customHeight="1">
+      <c r="A15" s="37"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
     </row>
     <row r="16" ht="27" customHeight="1">
       <c r="A16" s="37"/>
-      <c r="B16" s="33" t="s">
-        <v>63</v>
-      </c>
-      <c r="C16" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="D16" s="34" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="17" ht="33.75" customHeight="1">
+      <c r="B16" s="29"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+    </row>
+    <row r="17" ht="27" customHeight="1">
       <c r="A17" s="37"/>
-      <c r="B17" s="34" t="s">
-        <v>66</v>
-      </c>
-      <c r="C17" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="D17" s="34"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
     </row>
     <row r="18" ht="27" customHeight="1">
       <c r="A18" s="37"/>
-      <c r="B18" s="33"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-    </row>
-    <row r="19" ht="27" customHeight="1">
-      <c r="A19" s="37"/>
-      <c r="B19" s="33"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+    </row>
+    <row r="19" ht="17.399999999999999" customHeight="1">
+      <c r="A19" s="38"/>
+      <c r="B19" s="32"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
     </row>
     <row r="20" ht="27" customHeight="1">
-      <c r="A20" s="37"/>
-      <c r="B20" s="33"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="34"/>
+      <c r="A20" s="39" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" s="29" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="D20" s="30" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="21" ht="27" customHeight="1">
-      <c r="A21" s="37"/>
-      <c r="B21" s="33"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-    </row>
-    <row r="22" ht="27" customHeight="1">
-      <c r="A22" s="37"/>
-      <c r="B22" s="33"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
+      <c r="A21" s="39"/>
+      <c r="B21" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="D21" s="30" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" ht="33.75" customHeight="1">
+      <c r="A22" s="39"/>
+      <c r="B22" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="D22" s="30"/>
     </row>
     <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="37"/>
-      <c r="B23" s="33"/>
-      <c r="C23" s="34"/>
-      <c r="D23" s="34"/>
-    </row>
-    <row r="24" ht="41.25" customHeight="1">
-      <c r="B24" s="28"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="29"/>
-    </row>
-    <row r="25" ht="27.75" customHeight="1">
-      <c r="A25" s="39" t="s">
+      <c r="A23" s="39"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+    </row>
+    <row r="24" ht="27" customHeight="1">
+      <c r="A24" s="39"/>
+      <c r="B24" s="29"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+    </row>
+    <row r="25" ht="27" customHeight="1">
+      <c r="A25" s="39"/>
+      <c r="B25" s="29"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="30"/>
+    </row>
+    <row r="26" ht="27" customHeight="1">
+      <c r="A26" s="39"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="30"/>
+      <c r="D26" s="30"/>
+    </row>
+    <row r="27" ht="27" customHeight="1">
+      <c r="A27" s="39"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="30"/>
+      <c r="D27" s="30"/>
+    </row>
+    <row r="28" ht="27" customHeight="1">
+      <c r="A28" s="39"/>
+      <c r="B28" s="29"/>
+      <c r="C28" s="30"/>
+      <c r="D28" s="30"/>
+    </row>
+    <row r="29" ht="17.399999999999999" customHeight="1">
+      <c r="A29" s="5"/>
+      <c r="B29" s="32"/>
+      <c r="C29" s="33"/>
+      <c r="D29" s="33"/>
+    </row>
+    <row r="30" ht="27.75" customHeight="1">
+      <c r="A30" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="B30" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="B25" s="33" t="s">
+      <c r="C30" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="34" t="s">
+      <c r="D30" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="D25" s="34" t="s">
+    </row>
+    <row r="31" ht="27.75" customHeight="1">
+      <c r="A31" s="40"/>
+      <c r="B31" s="29" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="26" ht="27.75" customHeight="1">
-      <c r="A26" s="39"/>
-      <c r="B26" s="33" t="s">
+      <c r="C31" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="C26" s="34" t="s">
+      <c r="D31" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="D26" s="34" t="s">
+    </row>
+    <row r="32" ht="28.5">
+      <c r="A32" s="40"/>
+      <c r="B32" s="29" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="27" ht="28.5">
-      <c r="A27" s="39"/>
-      <c r="B27" s="33" t="s">
+      <c r="C32" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="C27" s="34" t="s">
+      <c r="D32" s="30"/>
+    </row>
+    <row r="33" ht="28.5">
+      <c r="A33" s="40"/>
+      <c r="B33" s="29" t="s">
         <v>76</v>
       </c>
-      <c r="D27" s="34"/>
-    </row>
-    <row r="28" ht="28.5">
-      <c r="A28" s="39"/>
-      <c r="B28" s="33" t="s">
+      <c r="C33" s="30" t="s">
         <v>77</v>
       </c>
-      <c r="C28" s="34" t="s">
+      <c r="D33" s="30"/>
+    </row>
+    <row r="34" ht="27.75" customHeight="1">
+      <c r="A34" s="40"/>
+      <c r="B34" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="D28" s="34"/>
-    </row>
-    <row r="29" ht="27.75" customHeight="1">
-      <c r="A29" s="39"/>
-      <c r="B29" s="33" t="s">
+      <c r="C34" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="C29" s="34" t="s">
+      <c r="D34" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="D29" s="34" t="s">
+    </row>
+    <row r="35" ht="31.199999999999999" customHeight="1">
+      <c r="A35" s="40"/>
+      <c r="B35" s="29" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="30" ht="31.199999999999999" customHeight="1">
-      <c r="A30" s="39"/>
-      <c r="B30" s="33" t="s">
+      <c r="C35" s="30" t="s">
         <v>82</v>
       </c>
-      <c r="C30" s="34" t="s">
+      <c r="D35" s="30"/>
+    </row>
+    <row r="36" ht="28.800000000000001" customHeight="1">
+      <c r="A36" s="40"/>
+      <c r="B36" s="41" t="s">
         <v>83</v>
       </c>
-      <c r="D30" s="34"/>
-    </row>
-    <row r="31" ht="28.800000000000001" customHeight="1">
-      <c r="A31" s="39"/>
-      <c r="B31" s="33"/>
-      <c r="C31" s="34"/>
-      <c r="D31" s="34"/>
-    </row>
-    <row r="32" ht="29.399999999999999" customHeight="1">
-      <c r="A32" s="39"/>
-      <c r="B32" s="33"/>
-      <c r="C32" s="34"/>
-      <c r="D32" s="34"/>
-    </row>
-    <row r="33" ht="26.25" customHeight="1">
-      <c r="A33" s="39"/>
-      <c r="B33" s="33"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-    </row>
-    <row r="34" ht="28.800000000000001" customHeight="1">
-      <c r="A34" s="39"/>
-      <c r="B34" s="33"/>
-      <c r="C34" s="34"/>
-      <c r="D34" s="34"/>
-    </row>
-    <row r="35" ht="28.800000000000001" customHeight="1">
-      <c r="A35" s="39"/>
-      <c r="B35" s="33"/>
-      <c r="C35" s="34"/>
-      <c r="D35" s="34"/>
-    </row>
-    <row r="36" ht="28.5" customHeight="1">
-      <c r="A36" s="39"/>
-      <c r="B36" s="33"/>
-      <c r="C36" s="34"/>
-      <c r="D36" s="34"/>
-    </row>
-    <row r="37" ht="28.5" customHeight="1">
-      <c r="A37" s="39"/>
-      <c r="B37" s="33"/>
-      <c r="C37" s="34"/>
-      <c r="D37" s="34"/>
-    </row>
-    <row r="38" ht="28.5" customHeight="1">
-      <c r="A38" s="39"/>
-      <c r="B38" s="33"/>
-      <c r="C38" s="34"/>
-      <c r="D38" s="34"/>
-    </row>
-    <row r="39" ht="28.5" customHeight="1">
-      <c r="A39" s="39"/>
-      <c r="B39" s="33"/>
-      <c r="C39" s="34"/>
-      <c r="D39" s="34"/>
-    </row>
-    <row r="40" ht="28.5" customHeight="1">
-      <c r="A40" s="39"/>
-      <c r="B40" s="33"/>
-      <c r="C40" s="34"/>
-      <c r="D40" s="34"/>
+      <c r="C36" s="42" t="s">
+        <v>84</v>
+      </c>
+      <c r="D36" s="42" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="37" ht="29.399999999999999" customHeight="1">
+      <c r="A37" s="40"/>
+      <c r="B37" s="29"/>
+      <c r="C37" s="30"/>
+      <c r="D37" s="30"/>
+    </row>
+    <row r="38" ht="26.25" customHeight="1">
+      <c r="A38" s="40"/>
+      <c r="B38" s="29"/>
+      <c r="C38" s="30"/>
+      <c r="D38" s="30"/>
+    </row>
+    <row r="39" ht="28.800000000000001" customHeight="1">
+      <c r="A39" s="40"/>
+      <c r="B39" s="29"/>
+      <c r="C39" s="30"/>
+      <c r="D39" s="30"/>
+    </row>
+    <row r="40" ht="28.800000000000001" customHeight="1">
+      <c r="A40" s="40"/>
+      <c r="B40" s="29"/>
+      <c r="C40" s="30"/>
+      <c r="D40" s="30"/>
     </row>
     <row r="41" ht="28.5" customHeight="1">
-      <c r="B41" s="28"/>
-      <c r="C41" s="29"/>
-      <c r="D41" s="29"/>
+      <c r="A41" s="40"/>
+      <c r="B41" s="29"/>
+      <c r="C41" s="30"/>
+      <c r="D41" s="30"/>
     </row>
     <row r="42" ht="28.5" customHeight="1">
-      <c r="B42" s="28"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="29"/>
-    </row>
-    <row r="43" ht="28.5" customHeight="1"/>
-    <row r="44" ht="28.5" customHeight="1"/>
-    <row r="45" ht="28.5" customHeight="1"/>
-    <row r="46" ht="28.5" customHeight="1"/>
-    <row r="47" ht="28.5" customHeight="1"/>
+      <c r="A42" s="40"/>
+      <c r="B42" s="29"/>
+      <c r="C42" s="30"/>
+      <c r="D42" s="30"/>
+    </row>
+    <row r="43" ht="28.5" customHeight="1">
+      <c r="A43" s="40"/>
+      <c r="B43" s="29"/>
+      <c r="C43" s="30"/>
+      <c r="D43" s="30"/>
+    </row>
+    <row r="44" ht="28.5" customHeight="1">
+      <c r="A44" s="40"/>
+      <c r="B44" s="29"/>
+      <c r="C44" s="30"/>
+      <c r="D44" s="30"/>
+    </row>
+    <row r="45" ht="28.5" customHeight="1">
+      <c r="A45" s="40"/>
+      <c r="B45" s="29"/>
+      <c r="C45" s="30"/>
+      <c r="D45" s="30"/>
+    </row>
+    <row r="46" ht="28.5" customHeight="1">
+      <c r="B46" s="24"/>
+      <c r="C46" s="25"/>
+      <c r="D46" s="25"/>
+    </row>
+    <row r="47" ht="28.5" customHeight="1">
+      <c r="B47" s="24"/>
+      <c r="C47" s="25"/>
+      <c r="D47" s="25"/>
+    </row>
     <row r="48" ht="28.5" customHeight="1"/>
     <row r="49" ht="28.5" customHeight="1"/>
     <row r="50" ht="28.5" customHeight="1"/>
@@ -1832,12 +1978,18 @@
     <row r="53" ht="28.5" customHeight="1"/>
     <row r="54" ht="28.5" customHeight="1"/>
     <row r="55" ht="28.5" customHeight="1"/>
+    <row r="56" ht="28.5" customHeight="1"/>
+    <row r="57" ht="28.5" customHeight="1"/>
+    <row r="58" ht="28.5" customHeight="1"/>
+    <row r="59" ht="28.5" customHeight="1"/>
+    <row r="60" ht="28.5" customHeight="1"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A2:A6"/>
-    <mergeCell ref="A8:A13"/>
-    <mergeCell ref="A15:A23"/>
-    <mergeCell ref="A25:A40"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="A13:A18"/>
+    <mergeCell ref="A20:A28"/>
+    <mergeCell ref="A30:A45"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
@@ -1861,13 +2013,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -1894,58 +2046,58 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>94</v>
+      </c>
+      <c r="C3" t="s">
         <v>91</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C3" t="s">
-        <v>89</v>
-      </c>
       <c r="D3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C4" s="40" t="s">
-        <v>89</v>
+        <v>96</v>
+      </c>
+      <c r="C4" s="44" t="s">
+        <v>91</v>
       </c>
       <c r="D4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B5" t="s">
-        <v>97</v>
-      </c>
-      <c r="C5" s="40" t="s">
-        <v>89</v>
+        <v>99</v>
+      </c>
+      <c r="C5" s="44" t="s">
+        <v>91</v>
       </c>
       <c r="D5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1"/>
@@ -2949,4 +3101,255 @@
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="5.57421875"/>
+    <col customWidth="1" min="2" max="2" style="45" width="24.421875"/>
+    <col customWidth="1" min="3" max="3" width="55.421875"/>
+    <col customWidth="1" min="4" max="4" width="75.8515625"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18.75">
+      <c r="B1" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="27" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="27" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" ht="42.75">
+      <c r="A2" s="46"/>
+      <c r="B2" s="47" t="s">
+        <v>101</v>
+      </c>
+      <c r="C2" s="48" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" s="48" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" ht="21.600000000000001" customHeight="1">
+      <c r="A3" s="46"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+    </row>
+    <row r="4" ht="21.600000000000001" customHeight="1">
+      <c r="A4" s="46"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+    </row>
+    <row r="5" ht="21.600000000000001" customHeight="1">
+      <c r="A5" s="46"/>
+      <c r="B5" s="47"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
+    </row>
+    <row r="6" ht="21.600000000000001" customHeight="1">
+      <c r="A6" s="46"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+    </row>
+    <row r="7" ht="21.600000000000001" customHeight="1">
+      <c r="A7" s="46"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
+    </row>
+    <row r="8" ht="14.25">
+      <c r="A8" s="5"/>
+      <c r="B8" s="49"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+    </row>
+    <row r="9" ht="41.25" customHeight="1">
+      <c r="A9" s="50" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" s="51" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" ht="39.75" customHeight="1">
+      <c r="A10" s="52"/>
+      <c r="B10" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="C10" s="30">
+        <v>60000</v>
+      </c>
+      <c r="D10" s="30" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" ht="36.75" customHeight="1">
+      <c r="A11" s="52"/>
+      <c r="B11" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="C11" s="30">
+        <v>3000</v>
+      </c>
+      <c r="D11" s="30" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" ht="36.75" customHeight="1">
+      <c r="A12" s="52"/>
+      <c r="B12" s="29" t="s">
+        <v>112</v>
+      </c>
+      <c r="C12" s="30" t="s">
+        <v>113</v>
+      </c>
+      <c r="D12" s="30" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="52"/>
+      <c r="B13" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="14" ht="63.600000000000001" customHeight="1">
+      <c r="A14" s="52"/>
+      <c r="B14" s="29" t="s">
+        <v>117</v>
+      </c>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="15" ht="14.25">
+      <c r="A15" s="5"/>
+      <c r="B15" s="49"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+    </row>
+    <row r="16" ht="30.600000000000001" customHeight="1"/>
+    <row r="17" ht="28.199999999999999" customHeight="1"/>
+    <row r="18" ht="28.199999999999999" customHeight="1"/>
+    <row r="19" ht="28.199999999999999" customHeight="1"/>
+    <row r="20" ht="28.199999999999999" customHeight="1"/>
+    <row r="21" ht="28.199999999999999" customHeight="1"/>
+    <row r="22" ht="28.199999999999999" customHeight="1"/>
+    <row r="23" ht="28.199999999999999" customHeight="1"/>
+    <row r="24" ht="28.199999999999999" customHeight="1"/>
+    <row r="25" ht="28.199999999999999" customHeight="1"/>
+    <row r="26" ht="28.199999999999999" customHeight="1"/>
+    <row r="27" ht="28.199999999999999" customHeight="1"/>
+    <row r="28" ht="28.199999999999999" customHeight="1"/>
+    <row r="29" ht="28.199999999999999" customHeight="1"/>
+    <row r="30" ht="28.199999999999999" customHeight="1"/>
+    <row r="31" ht="28.199999999999999" customHeight="1"/>
+    <row r="32" ht="28.199999999999999" customHeight="1"/>
+    <row r="33" ht="28.199999999999999" customHeight="1"/>
+    <row r="34" ht="28.199999999999999" customHeight="1"/>
+    <row r="35" ht="28.199999999999999" customHeight="1"/>
+    <row r="36" ht="28.199999999999999" customHeight="1"/>
+    <row r="37" ht="28.199999999999999" customHeight="1"/>
+    <row r="38" ht="28.199999999999999" customHeight="1"/>
+    <row r="39" ht="28.199999999999999" customHeight="1"/>
+    <row r="40" ht="28.199999999999999" customHeight="1"/>
+    <row r="41" ht="28.199999999999999" customHeight="1"/>
+    <row r="42" ht="28.199999999999999" customHeight="1"/>
+    <row r="43" ht="28.199999999999999" customHeight="1"/>
+    <row r="44" ht="28.199999999999999" customHeight="1"/>
+    <row r="45" ht="28.199999999999999" customHeight="1"/>
+    <row r="46" ht="28.199999999999999" customHeight="1"/>
+    <row r="47" ht="28.199999999999999" customHeight="1"/>
+    <row r="48" ht="28.199999999999999" customHeight="1"/>
+    <row r="49" ht="28.199999999999999" customHeight="1"/>
+    <row r="50" ht="28.199999999999999" customHeight="1"/>
+    <row r="51" ht="28.199999999999999" customHeight="1"/>
+    <row r="52" ht="28.199999999999999" customHeight="1"/>
+    <row r="53" ht="28.199999999999999" customHeight="1"/>
+    <row r="54" ht="28.199999999999999" customHeight="1"/>
+    <row r="55" ht="28.199999999999999" customHeight="1"/>
+    <row r="56" ht="28.199999999999999" customHeight="1"/>
+    <row r="57" ht="28.199999999999999" customHeight="1"/>
+    <row r="58" ht="28.199999999999999" customHeight="1"/>
+    <row r="59" ht="28.199999999999999" customHeight="1"/>
+    <row r="60" ht="28.199999999999999" customHeight="1"/>
+    <row r="61" ht="28.199999999999999" customHeight="1"/>
+    <row r="62" ht="28.199999999999999" customHeight="1"/>
+    <row r="63" ht="28.199999999999999" customHeight="1"/>
+    <row r="64" ht="28.199999999999999" customHeight="1"/>
+    <row r="65" ht="28.199999999999999" customHeight="1"/>
+    <row r="66" ht="28.199999999999999" customHeight="1"/>
+    <row r="67" ht="28.199999999999999" customHeight="1"/>
+    <row r="68" ht="28.199999999999999" customHeight="1"/>
+    <row r="69" ht="28.199999999999999" customHeight="1"/>
+    <row r="70" ht="28.199999999999999" customHeight="1"/>
+    <row r="71" ht="28.199999999999999" customHeight="1"/>
+    <row r="72" ht="28.199999999999999" customHeight="1"/>
+    <row r="73" ht="28.199999999999999" customHeight="1"/>
+    <row r="74" ht="28.199999999999999" customHeight="1"/>
+    <row r="75" ht="28.199999999999999" customHeight="1"/>
+    <row r="76" ht="28.199999999999999" customHeight="1"/>
+    <row r="77" ht="28.199999999999999" customHeight="1"/>
+    <row r="78" ht="28.199999999999999" customHeight="1"/>
+    <row r="79" ht="28.199999999999999" customHeight="1"/>
+    <row r="80" ht="28.199999999999999" customHeight="1"/>
+    <row r="81" ht="28.199999999999999" customHeight="1"/>
+    <row r="82" ht="28.199999999999999" customHeight="1"/>
+    <row r="83" ht="28.199999999999999" customHeight="1"/>
+    <row r="84" ht="28.199999999999999" customHeight="1"/>
+    <row r="85" ht="28.199999999999999" customHeight="1"/>
+    <row r="86" ht="28.199999999999999" customHeight="1"/>
+    <row r="87" ht="28.199999999999999" customHeight="1"/>
+    <row r="88" ht="28.199999999999999" customHeight="1"/>
+    <row r="89" ht="28.199999999999999" customHeight="1"/>
+    <row r="90" ht="28.199999999999999" customHeight="1"/>
+    <row r="91" ht="28.199999999999999" customHeight="1"/>
+    <row r="92" ht="28.199999999999999" customHeight="1"/>
+    <row r="93" ht="28.199999999999999" customHeight="1"/>
+    <row r="94" ht="28.199999999999999" customHeight="1"/>
+    <row r="95" ht="28.199999999999999" customHeight="1"/>
+    <row r="96" ht="28.199999999999999" customHeight="1"/>
+    <row r="97" ht="28.199999999999999" customHeight="1"/>
+    <row r="98" ht="28.199999999999999" customHeight="1"/>
+    <row r="99" ht="28.199999999999999" customHeight="1"/>
+    <row r="100" ht="28.199999999999999" customHeight="1"/>
+    <row r="101" ht="28.199999999999999" customHeight="1"/>
+    <row r="102" ht="28.199999999999999" customHeight="1"/>
+    <row r="103" ht="28.199999999999999" customHeight="1"/>
+    <row r="104" ht="28.199999999999999" customHeight="1"/>
+    <row r="105" ht="28.199999999999999" customHeight="1"/>
+    <row r="106" ht="28.199999999999999" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:A7"/>
+    <mergeCell ref="A9:A14"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="C9"/>
+  </hyperlinks>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Adicionando funcionalidades para criação do documento de importação no domímio
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -471,6 +471,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <sz val="11.000000"/>
@@ -714,12 +717,6 @@
     <xf fontId="5" fillId="11" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -747,6 +744,12 @@
     </xf>
     <xf fontId="2" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1588,7 +1591,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" ht="42.75">
+    <row r="3" ht="28.5">
       <c r="A3" s="28"/>
       <c r="B3" s="29" t="s">
         <v>36</v>
@@ -1896,13 +1899,13 @@
     </row>
     <row r="36" ht="28.800000000000001" customHeight="1">
       <c r="A36" s="40"/>
-      <c r="B36" s="41" t="s">
+      <c r="B36" s="29" t="s">
         <v>83</v>
       </c>
-      <c r="C36" s="42" t="s">
+      <c r="C36" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="D36" s="42" t="s">
+      <c r="D36" s="30" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2062,7 +2065,7 @@
       <c r="A3" t="s">
         <v>93</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="41" t="s">
         <v>94</v>
       </c>
       <c r="C3" t="s">
@@ -2079,7 +2082,7 @@
       <c r="B4" t="s">
         <v>96</v>
       </c>
-      <c r="C4" s="44" t="s">
+      <c r="C4" s="42" t="s">
         <v>91</v>
       </c>
       <c r="D4" t="s">
@@ -2093,7 +2096,7 @@
       <c r="B5" t="s">
         <v>99</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="42" t="s">
         <v>91</v>
       </c>
       <c r="D5" t="s">
@@ -3108,7 +3111,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.57421875"/>
-    <col customWidth="1" min="2" max="2" style="45" width="24.421875"/>
+    <col customWidth="1" min="2" max="2" style="43" width="24.421875"/>
     <col customWidth="1" min="3" max="3" width="55.421875"/>
     <col customWidth="1" min="4" max="4" width="75.8515625"/>
   </cols>
@@ -3125,61 +3128,61 @@
       </c>
     </row>
     <row r="2" ht="42.75">
-      <c r="A2" s="46"/>
-      <c r="B2" s="47" t="s">
+      <c r="A2" s="44"/>
+      <c r="B2" s="45" t="s">
         <v>101</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="C2" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="D2" s="46" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="3" ht="21.600000000000001" customHeight="1">
-      <c r="A3" s="46"/>
-      <c r="B3" s="47"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
+      <c r="A3" s="44"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
     </row>
     <row r="4" ht="21.600000000000001" customHeight="1">
-      <c r="A4" s="46"/>
-      <c r="B4" s="47"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
+      <c r="A4" s="44"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
     </row>
     <row r="5" ht="21.600000000000001" customHeight="1">
-      <c r="A5" s="46"/>
-      <c r="B5" s="47"/>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
+      <c r="A5" s="44"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
     </row>
     <row r="6" ht="21.600000000000001" customHeight="1">
-      <c r="A6" s="46"/>
-      <c r="B6" s="47"/>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
+      <c r="A6" s="44"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
     </row>
     <row r="7" ht="21.600000000000001" customHeight="1">
-      <c r="A7" s="46"/>
-      <c r="B7" s="47"/>
-      <c r="C7" s="48"/>
-      <c r="D7" s="48"/>
+      <c r="A7" s="44"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" s="5"/>
-      <c r="B8" s="49"/>
+      <c r="B8" s="47"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
     </row>
     <row r="9" ht="41.25" customHeight="1">
-      <c r="A9" s="50" t="s">
+      <c r="A9" s="48" t="s">
         <v>104</v>
       </c>
       <c r="B9" s="29" t="s">
         <v>105</v>
       </c>
-      <c r="C9" s="51" t="s">
+      <c r="C9" s="49" t="s">
         <v>106</v>
       </c>
       <c r="D9" s="30" t="s">
@@ -3187,7 +3190,7 @@
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="52"/>
+      <c r="A10" s="50"/>
       <c r="B10" s="29" t="s">
         <v>108</v>
       </c>
@@ -3199,7 +3202,7 @@
       </c>
     </row>
     <row r="11" ht="36.75" customHeight="1">
-      <c r="A11" s="52"/>
+      <c r="A11" s="50"/>
       <c r="B11" s="29" t="s">
         <v>110</v>
       </c>
@@ -3211,7 +3214,7 @@
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="52"/>
+      <c r="A12" s="50"/>
       <c r="B12" s="29" t="s">
         <v>112</v>
       </c>
@@ -3223,28 +3226,32 @@
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="52"/>
+      <c r="A13" s="50"/>
       <c r="B13" s="29" t="s">
         <v>115</v>
       </c>
-      <c r="C13" s="30"/>
+      <c r="C13" s="51">
+        <v>45778</v>
+      </c>
       <c r="D13" s="30" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="14" ht="63.600000000000001" customHeight="1">
-      <c r="A14" s="52"/>
-      <c r="B14" s="29" t="s">
+      <c r="A14" s="50"/>
+      <c r="B14" s="52" t="s">
         <v>117</v>
       </c>
-      <c r="C14" s="30"/>
+      <c r="C14" s="51">
+        <v>46023</v>
+      </c>
       <c r="D14" s="30" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" s="5"/>
-      <c r="B15" s="49"/>
+      <c r="B15" s="47"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>

</xml_diff>

<commit_message>
Adicionando funcionalidade de criação dinâmica de arquivos de importação
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="121">
   <si>
     <t>Name</t>
   </si>
@@ -309,6 +309,12 @@
   </si>
   <si>
     <t xml:space="preserve">Opção 'enable_integration' está desabilitada, o processo não irá integrar as obrigações.</t>
+  </si>
+  <si>
+    <t>LogMessage_NoExpensesToEspecificatedDebitAccount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não existem despesas com a conta de débito especificada: </t>
   </si>
   <si>
     <t xml:space="preserve">EXCEPTION LOG MESSAGES</t>
@@ -613,7 +619,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -714,6 +720,12 @@
     <xf fontId="5" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="5" fillId="11" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
@@ -747,9 +759,6 @@
     </xf>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1789,8 +1798,12 @@
     </row>
     <row r="23" ht="27" customHeight="1">
       <c r="A23" s="39"/>
-      <c r="B23" s="29"/>
-      <c r="C23" s="30"/>
+      <c r="B23" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23" s="41" t="s">
+        <v>68</v>
+      </c>
       <c r="D23" s="30"/>
     </row>
     <row r="24" ht="27" customHeight="1">
@@ -1830,135 +1843,135 @@
       <c r="D29" s="33"/>
     </row>
     <row r="30" ht="27.75" customHeight="1">
-      <c r="A30" s="40" t="s">
-        <v>67</v>
+      <c r="A30" s="42" t="s">
+        <v>69</v>
       </c>
       <c r="B30" s="29" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C30" s="30" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D30" s="30" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31" ht="27.75" customHeight="1">
-      <c r="A31" s="40"/>
+      <c r="A31" s="42"/>
       <c r="B31" s="29" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C31" s="30" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D31" s="30" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32" ht="28.5">
-      <c r="A32" s="40"/>
+      <c r="A32" s="42"/>
       <c r="B32" s="29" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C32" s="30" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D32" s="30"/>
     </row>
     <row r="33" ht="28.5">
-      <c r="A33" s="40"/>
+      <c r="A33" s="42"/>
       <c r="B33" s="29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C33" s="30" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D33" s="30"/>
     </row>
     <row r="34" ht="27.75" customHeight="1">
-      <c r="A34" s="40"/>
+      <c r="A34" s="42"/>
       <c r="B34" s="29" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C34" s="30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D34" s="30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="35" ht="31.199999999999999" customHeight="1">
-      <c r="A35" s="40"/>
+      <c r="A35" s="42"/>
       <c r="B35" s="29" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C35" s="30" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D35" s="30"/>
     </row>
     <row r="36" ht="28.800000000000001" customHeight="1">
-      <c r="A36" s="40"/>
+      <c r="A36" s="42"/>
       <c r="B36" s="29" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C36" s="30" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D36" s="30" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="37" ht="29.399999999999999" customHeight="1">
-      <c r="A37" s="40"/>
+      <c r="A37" s="42"/>
       <c r="B37" s="29"/>
       <c r="C37" s="30"/>
       <c r="D37" s="30"/>
     </row>
     <row r="38" ht="26.25" customHeight="1">
-      <c r="A38" s="40"/>
+      <c r="A38" s="42"/>
       <c r="B38" s="29"/>
       <c r="C38" s="30"/>
       <c r="D38" s="30"/>
     </row>
     <row r="39" ht="28.800000000000001" customHeight="1">
-      <c r="A39" s="40"/>
+      <c r="A39" s="42"/>
       <c r="B39" s="29"/>
       <c r="C39" s="30"/>
       <c r="D39" s="30"/>
     </row>
     <row r="40" ht="28.800000000000001" customHeight="1">
-      <c r="A40" s="40"/>
+      <c r="A40" s="42"/>
       <c r="B40" s="29"/>
       <c r="C40" s="30"/>
       <c r="D40" s="30"/>
     </row>
     <row r="41" ht="28.5" customHeight="1">
-      <c r="A41" s="40"/>
+      <c r="A41" s="42"/>
       <c r="B41" s="29"/>
       <c r="C41" s="30"/>
       <c r="D41" s="30"/>
     </row>
     <row r="42" ht="28.5" customHeight="1">
-      <c r="A42" s="40"/>
+      <c r="A42" s="42"/>
       <c r="B42" s="29"/>
       <c r="C42" s="30"/>
       <c r="D42" s="30"/>
     </row>
     <row r="43" ht="28.5" customHeight="1">
-      <c r="A43" s="40"/>
+      <c r="A43" s="42"/>
       <c r="B43" s="29"/>
       <c r="C43" s="30"/>
       <c r="D43" s="30"/>
     </row>
     <row r="44" ht="28.5" customHeight="1">
-      <c r="A44" s="40"/>
+      <c r="A44" s="42"/>
       <c r="B44" s="29"/>
       <c r="C44" s="30"/>
       <c r="D44" s="30"/>
     </row>
     <row r="45" ht="28.5" customHeight="1">
-      <c r="A45" s="40"/>
+      <c r="A45" s="42"/>
       <c r="B45" s="29"/>
       <c r="C45" s="30"/>
       <c r="D45" s="30"/>
@@ -2016,13 +2029,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -2049,58 +2062,58 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>96</v>
+      </c>
+      <c r="C3" t="s">
         <v>93</v>
       </c>
-      <c r="B3" s="41" t="s">
-        <v>94</v>
-      </c>
-      <c r="C3" t="s">
-        <v>91</v>
-      </c>
       <c r="D3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C4" s="42" t="s">
-        <v>91</v>
+        <v>98</v>
+      </c>
+      <c r="C4" s="44" t="s">
+        <v>93</v>
       </c>
       <c r="D4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
-      </c>
-      <c r="C5" s="42" t="s">
-        <v>91</v>
+        <v>101</v>
+      </c>
+      <c r="C5" s="44" t="s">
+        <v>93</v>
       </c>
       <c r="D5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1"/>
@@ -3111,7 +3124,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.57421875"/>
-    <col customWidth="1" min="2" max="2" style="43" width="24.421875"/>
+    <col customWidth="1" min="2" max="2" style="45" width="24.421875"/>
     <col customWidth="1" min="3" max="3" width="55.421875"/>
     <col customWidth="1" min="4" max="4" width="75.8515625"/>
   </cols>
@@ -3128,130 +3141,130 @@
       </c>
     </row>
     <row r="2" ht="42.75">
-      <c r="A2" s="44"/>
-      <c r="B2" s="45" t="s">
-        <v>101</v>
-      </c>
-      <c r="C2" s="46" t="s">
-        <v>102</v>
-      </c>
-      <c r="D2" s="46" t="s">
+      <c r="A2" s="46"/>
+      <c r="B2" s="47" t="s">
         <v>103</v>
       </c>
+      <c r="C2" s="48" t="s">
+        <v>104</v>
+      </c>
+      <c r="D2" s="48" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="3" ht="21.600000000000001" customHeight="1">
-      <c r="A3" s="44"/>
-      <c r="B3" s="45"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
+      <c r="A3" s="46"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
     </row>
     <row r="4" ht="21.600000000000001" customHeight="1">
-      <c r="A4" s="44"/>
-      <c r="B4" s="45"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
+      <c r="A4" s="46"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
     </row>
     <row r="5" ht="21.600000000000001" customHeight="1">
-      <c r="A5" s="44"/>
-      <c r="B5" s="45"/>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
+      <c r="A5" s="46"/>
+      <c r="B5" s="47"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
     </row>
     <row r="6" ht="21.600000000000001" customHeight="1">
-      <c r="A6" s="44"/>
-      <c r="B6" s="45"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
+      <c r="A6" s="46"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
     </row>
     <row r="7" ht="21.600000000000001" customHeight="1">
-      <c r="A7" s="44"/>
-      <c r="B7" s="45"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
+      <c r="A7" s="46"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" s="5"/>
-      <c r="B8" s="47"/>
+      <c r="B8" s="49"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
     </row>
     <row r="9" ht="41.25" customHeight="1">
-      <c r="A9" s="48" t="s">
-        <v>104</v>
+      <c r="A9" s="50" t="s">
+        <v>106</v>
       </c>
       <c r="B9" s="29" t="s">
-        <v>105</v>
-      </c>
-      <c r="C9" s="49" t="s">
-        <v>106</v>
+        <v>107</v>
+      </c>
+      <c r="C9" s="51" t="s">
+        <v>108</v>
       </c>
       <c r="D9" s="30" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="50"/>
+      <c r="A10" s="52"/>
       <c r="B10" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C10" s="30">
         <v>60000</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11" ht="36.75" customHeight="1">
-      <c r="A11" s="50"/>
+      <c r="A11" s="52"/>
       <c r="B11" s="29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C11" s="30">
         <v>3000</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="50"/>
+      <c r="A12" s="52"/>
       <c r="B12" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D12" s="30" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="50"/>
+      <c r="A13" s="52"/>
       <c r="B13" s="29" t="s">
-        <v>115</v>
-      </c>
-      <c r="C13" s="51">
+        <v>117</v>
+      </c>
+      <c r="C13" s="53">
         <v>45778</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14" ht="63.600000000000001" customHeight="1">
-      <c r="A14" s="50"/>
-      <c r="B14" s="52" t="s">
-        <v>117</v>
-      </c>
-      <c r="C14" s="51">
+      <c r="A14" s="52"/>
+      <c r="B14" s="29" t="s">
+        <v>119</v>
+      </c>
+      <c r="C14" s="53">
         <v>46023</v>
       </c>
       <c r="D14" s="30" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" s="5"/>
-      <c r="B15" s="47"/>
+      <c r="B15" s="49"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>

</xml_diff>

<commit_message>
Commit de sexta, correção de bug de data no config.xlsx
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
   <si>
     <t>Name</t>
   </si>
@@ -426,6 +426,18 @@
   </si>
   <si>
     <t xml:space="preserve">Endereço onde serão alocados os arquivos de importação e relatórios de erros de importação do processo</t>
+  </si>
+  <si>
+    <t>allDebitAccountImportationArchiveName</t>
+  </si>
+  <si>
+    <t>ContasDeDebitoGeral</t>
+  </si>
+  <si>
+    <t>especificDebitCount</t>
+  </si>
+  <si>
+    <t>2055,1055,2074,5572</t>
   </si>
   <si>
     <t>GetExpensesSettings</t>
@@ -619,7 +631,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="52">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -719,12 +731,6 @@
     <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf fontId="5" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="5" fillId="11" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
@@ -1798,10 +1804,10 @@
     </row>
     <row r="23" ht="27" customHeight="1">
       <c r="A23" s="39"/>
-      <c r="B23" s="40" t="s">
+      <c r="B23" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="41" t="s">
+      <c r="C23" s="30" t="s">
         <v>68</v>
       </c>
       <c r="D23" s="30"/>
@@ -1843,7 +1849,7 @@
       <c r="D29" s="33"/>
     </row>
     <row r="30" ht="27.75" customHeight="1">
-      <c r="A30" s="42" t="s">
+      <c r="A30" s="40" t="s">
         <v>69</v>
       </c>
       <c r="B30" s="29" t="s">
@@ -1857,7 +1863,7 @@
       </c>
     </row>
     <row r="31" ht="27.75" customHeight="1">
-      <c r="A31" s="42"/>
+      <c r="A31" s="40"/>
       <c r="B31" s="29" t="s">
         <v>73</v>
       </c>
@@ -1869,7 +1875,7 @@
       </c>
     </row>
     <row r="32" ht="28.5">
-      <c r="A32" s="42"/>
+      <c r="A32" s="40"/>
       <c r="B32" s="29" t="s">
         <v>76</v>
       </c>
@@ -1879,7 +1885,7 @@
       <c r="D32" s="30"/>
     </row>
     <row r="33" ht="28.5">
-      <c r="A33" s="42"/>
+      <c r="A33" s="40"/>
       <c r="B33" s="29" t="s">
         <v>78</v>
       </c>
@@ -1889,7 +1895,7 @@
       <c r="D33" s="30"/>
     </row>
     <row r="34" ht="27.75" customHeight="1">
-      <c r="A34" s="42"/>
+      <c r="A34" s="40"/>
       <c r="B34" s="29" t="s">
         <v>80</v>
       </c>
@@ -1901,7 +1907,7 @@
       </c>
     </row>
     <row r="35" ht="31.199999999999999" customHeight="1">
-      <c r="A35" s="42"/>
+      <c r="A35" s="40"/>
       <c r="B35" s="29" t="s">
         <v>83</v>
       </c>
@@ -1911,7 +1917,7 @@
       <c r="D35" s="30"/>
     </row>
     <row r="36" ht="28.800000000000001" customHeight="1">
-      <c r="A36" s="42"/>
+      <c r="A36" s="40"/>
       <c r="B36" s="29" t="s">
         <v>85</v>
       </c>
@@ -1923,55 +1929,55 @@
       </c>
     </row>
     <row r="37" ht="29.399999999999999" customHeight="1">
-      <c r="A37" s="42"/>
+      <c r="A37" s="40"/>
       <c r="B37" s="29"/>
       <c r="C37" s="30"/>
       <c r="D37" s="30"/>
     </row>
     <row r="38" ht="26.25" customHeight="1">
-      <c r="A38" s="42"/>
+      <c r="A38" s="40"/>
       <c r="B38" s="29"/>
       <c r="C38" s="30"/>
       <c r="D38" s="30"/>
     </row>
     <row r="39" ht="28.800000000000001" customHeight="1">
-      <c r="A39" s="42"/>
+      <c r="A39" s="40"/>
       <c r="B39" s="29"/>
       <c r="C39" s="30"/>
       <c r="D39" s="30"/>
     </row>
     <row r="40" ht="28.800000000000001" customHeight="1">
-      <c r="A40" s="42"/>
+      <c r="A40" s="40"/>
       <c r="B40" s="29"/>
       <c r="C40" s="30"/>
       <c r="D40" s="30"/>
     </row>
     <row r="41" ht="28.5" customHeight="1">
-      <c r="A41" s="42"/>
+      <c r="A41" s="40"/>
       <c r="B41" s="29"/>
       <c r="C41" s="30"/>
       <c r="D41" s="30"/>
     </row>
     <row r="42" ht="28.5" customHeight="1">
-      <c r="A42" s="42"/>
+      <c r="A42" s="40"/>
       <c r="B42" s="29"/>
       <c r="C42" s="30"/>
       <c r="D42" s="30"/>
     </row>
     <row r="43" ht="28.5" customHeight="1">
-      <c r="A43" s="42"/>
+      <c r="A43" s="40"/>
       <c r="B43" s="29"/>
       <c r="C43" s="30"/>
       <c r="D43" s="30"/>
     </row>
     <row r="44" ht="28.5" customHeight="1">
-      <c r="A44" s="42"/>
+      <c r="A44" s="40"/>
       <c r="B44" s="29"/>
       <c r="C44" s="30"/>
       <c r="D44" s="30"/>
     </row>
     <row r="45" ht="28.5" customHeight="1">
-      <c r="A45" s="42"/>
+      <c r="A45" s="40"/>
       <c r="B45" s="29"/>
       <c r="C45" s="30"/>
       <c r="D45" s="30"/>
@@ -2078,7 +2084,7 @@
       <c r="A3" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="41" t="s">
         <v>96</v>
       </c>
       <c r="C3" t="s">
@@ -2095,7 +2101,7 @@
       <c r="B4" t="s">
         <v>98</v>
       </c>
-      <c r="C4" s="44" t="s">
+      <c r="C4" s="42" t="s">
         <v>93</v>
       </c>
       <c r="D4" t="s">
@@ -2109,7 +2115,7 @@
       <c r="B5" t="s">
         <v>101</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="42" t="s">
         <v>93</v>
       </c>
       <c r="D5" t="s">
@@ -3124,7 +3130,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.57421875"/>
-    <col customWidth="1" min="2" max="2" style="45" width="24.421875"/>
+    <col customWidth="1" min="2" max="2" style="43" width="38.421875"/>
     <col customWidth="1" min="3" max="3" width="55.421875"/>
     <col customWidth="1" min="4" max="4" width="75.8515625"/>
   </cols>
@@ -3141,130 +3147,138 @@
       </c>
     </row>
     <row r="2" ht="42.75">
-      <c r="A2" s="46"/>
-      <c r="B2" s="47" t="s">
+      <c r="A2" s="44"/>
+      <c r="B2" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="C2" s="46" t="s">
         <v>104</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="D2" s="46" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="3" ht="21.600000000000001" customHeight="1">
-      <c r="A3" s="46"/>
-      <c r="B3" s="47"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
+      <c r="A3" s="44"/>
+      <c r="B3" s="45" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="46" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="46"/>
     </row>
     <row r="4" ht="21.600000000000001" customHeight="1">
-      <c r="A4" s="46"/>
-      <c r="B4" s="47"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
+      <c r="A4" s="44"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
     </row>
     <row r="5" ht="21.600000000000001" customHeight="1">
-      <c r="A5" s="46"/>
-      <c r="B5" s="47"/>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
+      <c r="A5" s="44"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="46" t="s">
+        <v>108</v>
+      </c>
+      <c r="D5" s="46" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="6" ht="21.600000000000001" customHeight="1">
-      <c r="A6" s="46"/>
-      <c r="B6" s="47"/>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
+      <c r="A6" s="44"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
     </row>
     <row r="7" ht="21.600000000000001" customHeight="1">
-      <c r="A7" s="46"/>
-      <c r="B7" s="47"/>
-      <c r="C7" s="48"/>
-      <c r="D7" s="48"/>
+      <c r="A7" s="44"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" s="5"/>
-      <c r="B8" s="49"/>
+      <c r="B8" s="47"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
     </row>
     <row r="9" ht="41.25" customHeight="1">
-      <c r="A9" s="50" t="s">
-        <v>106</v>
+      <c r="A9" s="48" t="s">
+        <v>110</v>
       </c>
       <c r="B9" s="29" t="s">
-        <v>107</v>
-      </c>
-      <c r="C9" s="51" t="s">
-        <v>108</v>
+        <v>111</v>
+      </c>
+      <c r="C9" s="49" t="s">
+        <v>112</v>
       </c>
       <c r="D9" s="30" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="52"/>
+      <c r="A10" s="50"/>
       <c r="B10" s="29" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C10" s="30">
         <v>60000</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" ht="36.75" customHeight="1">
-      <c r="A11" s="52"/>
+      <c r="A11" s="50"/>
       <c r="B11" s="29" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C11" s="30">
         <v>3000</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="52"/>
+      <c r="A12" s="50"/>
       <c r="B12" s="29" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D12" s="30" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="52"/>
+      <c r="A13" s="50"/>
       <c r="B13" s="29" t="s">
-        <v>117</v>
-      </c>
-      <c r="C13" s="53">
+        <v>121</v>
+      </c>
+      <c r="C13" s="51">
         <v>45778</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" ht="63.600000000000001" customHeight="1">
-      <c r="A14" s="52"/>
+      <c r="A14" s="50"/>
       <c r="B14" s="29" t="s">
-        <v>119</v>
-      </c>
-      <c r="C14" s="53">
-        <v>46023</v>
+        <v>123</v>
+      </c>
+      <c r="C14" s="51">
+        <v>46022</v>
       </c>
       <c r="D14" s="30" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" s="5"/>
-      <c r="B15" s="49"/>
+      <c r="B15" s="47"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>

</xml_diff>

<commit_message>
Implementação da dinâmica de datas para os requests das despesas do backoffice.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="133">
   <si>
     <t>Name</t>
   </si>
@@ -128,6 +128,9 @@
     <t>obligationDebugCnpj</t>
   </si>
   <si>
+    <t>25385913000102</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -158,9 +161,6 @@
     <t>obligationDebugCompanyId</t>
   </si>
   <si>
-    <t>7a8d0889-71e5-4dab-9ec2-734bf7c46734</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -374,6 +374,24 @@
     <t xml:space="preserve">Caso não existam despesas na empresa em questão.</t>
   </si>
   <si>
+    <t>ExceptionMessage_ExpenseRequest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erro no processo de requisição das despesas - Get Expenses.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso haja um erro no processo de Get Expenses</t>
+  </si>
+  <si>
+    <t>ExceptionMessage_ExpenseDatesDefinition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erro ao definir as datas de inicio e final do Get Exepenses. As datas devem estar com o tipo "texto" na planilha "Config.xlsx". Verifique também se as datas estão de acordo com a realidade.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso haja um erro durante o processo de definição de datas do request das despesas. </t>
+  </si>
+  <si>
     <t>Asset</t>
   </si>
   <si>
@@ -476,10 +494,16 @@
     <t>getExpenses_dateStart</t>
   </si>
   <si>
+    <t>01/05/2025</t>
+  </si>
+  <si>
     <t xml:space="preserve">Inicio do range de datas que abrange a data de vencimento das despesas que irão ser importadas. Deve estar no formato "dd/MM/yyyy" e só deve existir caso o getExpenses_dateEnd existir também.</t>
   </si>
   <si>
     <t>getExpenses_dateEnd</t>
+  </si>
+  <si>
+    <t>31/12/2025</t>
   </si>
   <si>
     <t xml:space="preserve">Fim do range de datas que abrange a data de vencimento das despesas que irão ser importadas. Deve estar no formato "dd/MM/yyyy" e só deve existir caso o getExpenses_dateStart existir também. Deve ser posterior ao getExpenses_dateStart</t>
@@ -489,9 +513,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-  </numFmts>
   <fonts count="6">
     <font>
       <sz val="11.000000"/>
@@ -631,7 +652,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -763,7 +784,10 @@
     <xf fontId="2" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1443,19 +1467,19 @@
       <c r="B15" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="19"/>
+      <c r="C15" s="19" t="s">
+        <v>22</v>
+      </c>
       <c r="D15" s="20" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" ht="34.799999999999997" customHeight="1">
       <c r="A16" s="13"/>
       <c r="B16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="14" t="s">
         <v>24</v>
       </c>
+      <c r="C16" s="14"/>
       <c r="D16" s="20" t="s">
         <v>25</v>
       </c>
@@ -1930,15 +1954,27 @@
     </row>
     <row r="37" ht="29.399999999999999" customHeight="1">
       <c r="A37" s="40"/>
-      <c r="B37" s="29"/>
-      <c r="C37" s="30"/>
-      <c r="D37" s="30"/>
-    </row>
-    <row r="38" ht="26.25" customHeight="1">
+      <c r="B37" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="C37" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="D37" s="30" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="38" ht="42.75">
       <c r="A38" s="40"/>
-      <c r="B38" s="29"/>
-      <c r="C38" s="30"/>
-      <c r="D38" s="30"/>
+      <c r="B38" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="C38" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="D38" s="30" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="39" ht="28.800000000000001" customHeight="1">
       <c r="A39" s="40"/>
@@ -2035,13 +2071,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -2068,58 +2104,58 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B3" s="41" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="C3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D3" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C4" s="42" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D4" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D5" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1"/>
@@ -3149,22 +3185,22 @@
     <row r="2" ht="42.75">
       <c r="A2" s="44"/>
       <c r="B2" s="45" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C2" s="46" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="D2" s="46" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" ht="21.600000000000001" customHeight="1">
       <c r="A3" s="44"/>
       <c r="B3" s="45" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="C3" s="46" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="D3" s="46"/>
     </row>
@@ -3178,10 +3214,10 @@
       <c r="A5" s="44"/>
       <c r="B5" s="45"/>
       <c r="C5" s="46" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D5" s="46" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" ht="21.600000000000001" customHeight="1">
@@ -3204,76 +3240,76 @@
     </row>
     <row r="9" ht="41.25" customHeight="1">
       <c r="A9" s="48" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B9" s="29" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C9" s="49" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D9" s="30" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
       <c r="A10" s="50"/>
       <c r="B10" s="29" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="C10" s="30">
         <v>60000</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" ht="36.75" customHeight="1">
       <c r="A11" s="50"/>
       <c r="B11" s="29" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="C11" s="30">
         <v>3000</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
       <c r="A12" s="50"/>
       <c r="B12" s="29" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D12" s="30" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="50"/>
       <c r="B13" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="C13" s="51">
-        <v>45778</v>
+        <v>127</v>
+      </c>
+      <c r="C13" s="51" t="s">
+        <v>128</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14" ht="63.600000000000001" customHeight="1">
       <c r="A14" s="50"/>
       <c r="B14" s="29" t="s">
-        <v>123</v>
-      </c>
-      <c r="C14" s="51">
-        <v>46022</v>
+        <v>130</v>
+      </c>
+      <c r="C14" s="52" t="s">
+        <v>131</v>
       </c>
       <c r="D14" s="30" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="15" ht="14.25">

</xml_diff>

<commit_message>
Ajuste no gitignore e validação da lógica dinâmica dos nomes dos arquivos de importação
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="134">
   <si>
     <t>Name</t>
   </si>
@@ -452,10 +452,13 @@
     <t>ContasDeDebitoGeral</t>
   </si>
   <si>
-    <t>especificDebitCount</t>
+    <t>especificDebitAccount</t>
   </si>
   <si>
     <t>2055,1055,2074,5572</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O Domínio pode apresentar erro de acordo com a quantidade de despesas inseridas em um determinado arquivo de importação. Por isso, existem as contas de débito específicas que devem estar separadas por arquivo de importação.Deve estar no fomraco "contaDeDebito,contaDeDebito,contaDeDebito"</t>
   </si>
   <si>
     <t>GetExpensesSettings</t>
@@ -652,7 +655,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -764,13 +767,19 @@
       <alignment vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -783,9 +792,6 @@
     </xf>
     <xf fontId="2" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3182,7 +3188,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" ht="42.75">
+    <row r="2" s="43" customFormat="1" ht="42.75">
       <c r="A2" s="44"/>
       <c r="B2" s="45" t="s">
         <v>109</v>
@@ -3194,7 +3200,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="3" ht="21.600000000000001" customHeight="1">
+    <row r="3" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
       <c r="A3" s="44"/>
       <c r="B3" s="45" t="s">
         <v>112</v>
@@ -3204,29 +3210,31 @@
       </c>
       <c r="D3" s="46"/>
     </row>
-    <row r="4" ht="21.600000000000001" customHeight="1">
+    <row r="4" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
       <c r="A4" s="44"/>
       <c r="B4" s="45"/>
       <c r="C4" s="46"/>
       <c r="D4" s="46"/>
     </row>
-    <row r="5" ht="21.600000000000001" customHeight="1">
+    <row r="5" s="43" customFormat="1" ht="57">
       <c r="A5" s="44"/>
-      <c r="B5" s="45"/>
+      <c r="B5" s="47" t="s">
+        <v>114</v>
+      </c>
       <c r="C5" s="46" t="s">
-        <v>114</v>
-      </c>
-      <c r="D5" s="46" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="6" ht="21.600000000000001" customHeight="1">
+      <c r="D5" s="48" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="6" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
       <c r="A6" s="44"/>
       <c r="B6" s="45"/>
       <c r="C6" s="46"/>
       <c r="D6" s="46"/>
     </row>
-    <row r="7" ht="21.600000000000001" customHeight="1">
+    <row r="7" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
       <c r="A7" s="44"/>
       <c r="B7" s="45"/>
       <c r="C7" s="46"/>
@@ -3234,87 +3242,87 @@
     </row>
     <row r="8" ht="14.25">
       <c r="A8" s="5"/>
-      <c r="B8" s="47"/>
+      <c r="B8" s="49"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
     </row>
     <row r="9" ht="41.25" customHeight="1">
-      <c r="A9" s="48" t="s">
-        <v>116</v>
+      <c r="A9" s="50" t="s">
+        <v>117</v>
       </c>
       <c r="B9" s="29" t="s">
-        <v>117</v>
-      </c>
-      <c r="C9" s="49" t="s">
         <v>118</v>
       </c>
+      <c r="C9" s="51" t="s">
+        <v>119</v>
+      </c>
       <c r="D9" s="30" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="50"/>
+      <c r="A10" s="52"/>
       <c r="B10" s="29" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C10" s="30">
         <v>60000</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" ht="36.75" customHeight="1">
-      <c r="A11" s="50"/>
+      <c r="A11" s="52"/>
       <c r="B11" s="29" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C11" s="30">
         <v>3000</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="50"/>
+      <c r="A12" s="52"/>
       <c r="B12" s="29" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D12" s="30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="50"/>
+      <c r="A13" s="52"/>
       <c r="B13" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="C13" s="51" t="s">
         <v>128</v>
       </c>
+      <c r="C13" s="53" t="s">
+        <v>129</v>
+      </c>
       <c r="D13" s="30" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" ht="63.600000000000001" customHeight="1">
-      <c r="A14" s="50"/>
+      <c r="A14" s="52"/>
       <c r="B14" s="29" t="s">
-        <v>130</v>
-      </c>
-      <c r="C14" s="52" t="s">
         <v>131</v>
       </c>
+      <c r="C14" s="53" t="s">
+        <v>132</v>
+      </c>
       <c r="D14" s="30" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" s="5"/>
-      <c r="B15" s="47"/>
+      <c r="B15" s="49"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>

</xml_diff>

<commit_message>
Adicionando query para consultas de dadas de fechamento, inicio das atividades, inicio do periodo de trabalho e fim do mesmo
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
   <si>
     <t>Name</t>
   </si>
@@ -128,9 +128,6 @@
     <t>obligationDebugCnpj</t>
   </si>
   <si>
-    <t>25385913000102</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -161,6 +158,9 @@
     <t>obligationDebugCompanyId</t>
   </si>
   <si>
+    <t>7a8d0889-71e5-4dab-9ec2-734bf7c46734</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -435,6 +435,24 @@
   </si>
   <si>
     <t xml:space="preserve">Codigo do contador dentro do domínio</t>
+  </si>
+  <si>
+    <t>databaseConnectionString</t>
+  </si>
+  <si>
+    <t>database_connection_string</t>
+  </si>
+  <si>
+    <t xml:space="preserve">String de conexão com o banco de dados do Domínio</t>
+  </si>
+  <si>
+    <t>databaseProviderName</t>
+  </si>
+  <si>
+    <t>database_provider_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provider name para conexão no banco de dados do Domínio</t>
   </si>
   <si>
     <t>mainPath</t>
@@ -703,6 +721,7 @@
     <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="2" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
     </xf>
@@ -771,9 +790,6 @@
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1473,19 +1489,19 @@
       <c r="B15" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="19"/>
+      <c r="D15" s="20" t="s">
         <v>22</v>
-      </c>
-      <c r="D15" s="20" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="16" ht="34.799999999999997" customHeight="1">
       <c r="A16" s="13"/>
       <c r="B16" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="14"/>
       <c r="D16" s="20" t="s">
         <v>25</v>
       </c>
@@ -1497,13 +1513,13 @@
       <c r="D17" s="5"/>
     </row>
     <row r="18" ht="46.799999999999997" customHeight="1">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="22" t="s">
         <v>26</v>
       </c>
       <c r="B18" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="23" t="s">
         <v>28</v>
       </c>
       <c r="D18" s="14" t="s">
@@ -1511,21 +1527,21 @@
       </c>
     </row>
     <row r="19" ht="46.799999999999997" customHeight="1">
-      <c r="A19" s="21"/>
+      <c r="A19" s="22"/>
       <c r="B19" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="24" t="s">
         <v>31</v>
       </c>
       <c r="D19" s="14"/>
     </row>
     <row r="20" ht="43.200000000000003" customHeight="1">
-      <c r="A20" s="21"/>
+      <c r="A20" s="22"/>
       <c r="B20" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="23" t="s">
+      <c r="C20" s="24" t="s">
         <v>33</v>
       </c>
       <c r="D20" s="14"/>
@@ -1584,20 +1600,20 @@
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8.00390625"/>
-    <col customWidth="1" min="2" max="2" style="24" width="52.140625"/>
-    <col bestFit="1" customWidth="1" min="3" max="3" style="25" width="63.11328125"/>
-    <col customWidth="1" min="4" max="4" style="25" width="84.140625"/>
+    <col customWidth="1" min="2" max="2" style="25" width="52.140625"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" style="26" width="63.11328125"/>
+    <col customWidth="1" min="4" max="4" style="26" width="84.140625"/>
     <col customWidth="1" min="5" max="27" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="28" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="2"/>
@@ -1625,79 +1641,79 @@
       <c r="AA1" s="2"/>
     </row>
     <row r="2" ht="28.5">
-      <c r="A2" s="28"/>
-      <c r="B2" s="29" t="s">
+      <c r="A2" s="29"/>
+      <c r="B2" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="30">
+      <c r="C2" s="31">
         <v>1</v>
       </c>
-      <c r="D2" s="30" t="s">
+      <c r="D2" s="31" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="3" ht="28.5">
-      <c r="A3" s="28"/>
-      <c r="B3" s="29" t="s">
+      <c r="A3" s="29"/>
+      <c r="B3" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="30">
+      <c r="C3" s="31">
         <v>3</v>
       </c>
-      <c r="D3" s="30" t="s">
+      <c r="D3" s="31" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="28"/>
-      <c r="B4" s="29" t="s">
+      <c r="A4" s="29"/>
+      <c r="B4" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="D4" s="31" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="5" ht="28.5">
-      <c r="A5" s="28"/>
-      <c r="B5" s="29" t="s">
+      <c r="A5" s="29"/>
+      <c r="B5" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="31">
         <v>2</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="31" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" ht="28.5">
-      <c r="A6" s="28"/>
-      <c r="B6" s="29" t="s">
+      <c r="A6" s="29"/>
+      <c r="B6" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="30">
+      <c r="C6" s="31">
         <v>2</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="31" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" s="31" customFormat="1" ht="17.399999999999999" customHeight="1">
+    <row r="7" s="32" customFormat="1" ht="17.399999999999999" customHeight="1">
       <c r="A7" s="5"/>
-      <c r="B7" s="32"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
     </row>
     <row r="8" ht="39.75" customHeight="1">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="35" t="s">
         <v>45</v>
       </c>
       <c r="B8" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="35">
+      <c r="C8" s="36">
         <v>30000</v>
       </c>
       <c r="D8" s="15" t="s">
@@ -1705,11 +1721,11 @@
       </c>
     </row>
     <row r="9" ht="39.75" customHeight="1">
-      <c r="A9" s="36"/>
+      <c r="A9" s="37"/>
       <c r="B9" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="35">
+      <c r="C9" s="36">
         <v>20000</v>
       </c>
       <c r="D9" s="15" t="s">
@@ -1717,11 +1733,11 @@
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="36"/>
+      <c r="A10" s="37"/>
       <c r="B10" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="35">
+      <c r="C10" s="36">
         <v>0</v>
       </c>
       <c r="D10" s="15" t="s">
@@ -1729,11 +1745,11 @@
       </c>
     </row>
     <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="36"/>
+      <c r="A11" s="37"/>
       <c r="B11" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="35">
+      <c r="C11" s="36">
         <v>0</v>
       </c>
       <c r="D11" s="15" t="s">
@@ -1742,297 +1758,297 @@
     </row>
     <row r="12" ht="17.399999999999999" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="32"/>
-      <c r="C12" s="33"/>
-      <c r="D12" s="33"/>
+      <c r="B12" s="33"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
     </row>
     <row r="13" ht="22.800000000000001" customHeight="1">
-      <c r="A13" s="37" t="s">
+      <c r="A13" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="D13" s="30" t="s">
+      <c r="D13" s="31" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="14" ht="28.199999999999999" customHeight="1">
-      <c r="A14" s="37"/>
-      <c r="B14" s="29"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="30"/>
+      <c r="A14" s="38"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="31"/>
     </row>
     <row r="15" ht="28.199999999999999" customHeight="1">
-      <c r="A15" s="37"/>
-      <c r="B15" s="29"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="30"/>
+      <c r="A15" s="38"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
     </row>
     <row r="16" ht="27" customHeight="1">
-      <c r="A16" s="37"/>
-      <c r="B16" s="29"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
+      <c r="A16" s="38"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
     </row>
     <row r="17" ht="27" customHeight="1">
-      <c r="A17" s="37"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
+      <c r="A17" s="38"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="31"/>
     </row>
     <row r="18" ht="27" customHeight="1">
-      <c r="A18" s="37"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
+      <c r="A18" s="38"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
     </row>
     <row r="19" ht="17.399999999999999" customHeight="1">
-      <c r="A19" s="38"/>
-      <c r="B19" s="32"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="33"/>
+      <c r="A19" s="39"/>
+      <c r="B19" s="33"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="34"/>
     </row>
     <row r="20" ht="27" customHeight="1">
-      <c r="A20" s="39" t="s">
+      <c r="A20" s="40" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="C20" s="30" t="s">
+      <c r="C20" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="D20" s="30" t="s">
+      <c r="D20" s="31" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="21" ht="27" customHeight="1">
-      <c r="A21" s="39"/>
-      <c r="B21" s="29" t="s">
+      <c r="A21" s="40"/>
+      <c r="B21" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="30" t="s">
+      <c r="C21" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="D21" s="30" t="s">
+      <c r="D21" s="31" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="22" ht="33.75" customHeight="1">
-      <c r="A22" s="39"/>
-      <c r="B22" s="30" t="s">
+      <c r="A22" s="40"/>
+      <c r="B22" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="C22" s="30" t="s">
+      <c r="C22" s="31" t="s">
         <v>66</v>
       </c>
-      <c r="D22" s="30"/>
+      <c r="D22" s="31"/>
     </row>
     <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="39"/>
-      <c r="B23" s="29" t="s">
+      <c r="A23" s="40"/>
+      <c r="B23" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="30" t="s">
+      <c r="C23" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="D23" s="30"/>
+      <c r="D23" s="31"/>
     </row>
     <row r="24" ht="27" customHeight="1">
-      <c r="A24" s="39"/>
-      <c r="B24" s="29"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="30"/>
+      <c r="A24" s="40"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
     </row>
     <row r="25" ht="27" customHeight="1">
-      <c r="A25" s="39"/>
-      <c r="B25" s="29"/>
+      <c r="A25" s="40"/>
+      <c r="B25" s="30"/>
       <c r="C25" s="20"/>
-      <c r="D25" s="30"/>
+      <c r="D25" s="31"/>
     </row>
     <row r="26" ht="27" customHeight="1">
-      <c r="A26" s="39"/>
-      <c r="B26" s="29"/>
-      <c r="C26" s="30"/>
-      <c r="D26" s="30"/>
+      <c r="A26" s="40"/>
+      <c r="B26" s="30"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
     </row>
     <row r="27" ht="27" customHeight="1">
-      <c r="A27" s="39"/>
-      <c r="B27" s="29"/>
-      <c r="C27" s="30"/>
-      <c r="D27" s="30"/>
+      <c r="A27" s="40"/>
+      <c r="B27" s="30"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
     </row>
     <row r="28" ht="27" customHeight="1">
-      <c r="A28" s="39"/>
-      <c r="B28" s="29"/>
-      <c r="C28" s="30"/>
-      <c r="D28" s="30"/>
+      <c r="A28" s="40"/>
+      <c r="B28" s="30"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
     </row>
     <row r="29" ht="17.399999999999999" customHeight="1">
       <c r="A29" s="5"/>
-      <c r="B29" s="32"/>
-      <c r="C29" s="33"/>
-      <c r="D29" s="33"/>
+      <c r="B29" s="33"/>
+      <c r="C29" s="34"/>
+      <c r="D29" s="34"/>
     </row>
     <row r="30" ht="27.75" customHeight="1">
-      <c r="A30" s="40" t="s">
+      <c r="A30" s="41" t="s">
         <v>69</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="C30" s="30" t="s">
+      <c r="C30" s="31" t="s">
         <v>71</v>
       </c>
-      <c r="D30" s="30" t="s">
+      <c r="D30" s="31" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="31" ht="27.75" customHeight="1">
-      <c r="A31" s="40"/>
-      <c r="B31" s="29" t="s">
+      <c r="A31" s="41"/>
+      <c r="B31" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="C31" s="30" t="s">
+      <c r="C31" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="D31" s="30" t="s">
+      <c r="D31" s="31" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="32" ht="28.5">
-      <c r="A32" s="40"/>
-      <c r="B32" s="29" t="s">
+      <c r="A32" s="41"/>
+      <c r="B32" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="C32" s="30" t="s">
+      <c r="C32" s="31" t="s">
         <v>77</v>
       </c>
-      <c r="D32" s="30"/>
+      <c r="D32" s="31"/>
     </row>
     <row r="33" ht="28.5">
-      <c r="A33" s="40"/>
-      <c r="B33" s="29" t="s">
+      <c r="A33" s="41"/>
+      <c r="B33" s="30" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="30" t="s">
+      <c r="C33" s="31" t="s">
         <v>79</v>
       </c>
-      <c r="D33" s="30"/>
+      <c r="D33" s="31"/>
     </row>
     <row r="34" ht="27.75" customHeight="1">
-      <c r="A34" s="40"/>
-      <c r="B34" s="29" t="s">
+      <c r="A34" s="41"/>
+      <c r="B34" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="C34" s="30" t="s">
+      <c r="C34" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="D34" s="30" t="s">
+      <c r="D34" s="31" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="35" ht="31.199999999999999" customHeight="1">
-      <c r="A35" s="40"/>
-      <c r="B35" s="29" t="s">
+      <c r="A35" s="41"/>
+      <c r="B35" s="30" t="s">
         <v>83</v>
       </c>
-      <c r="C35" s="30" t="s">
+      <c r="C35" s="31" t="s">
         <v>84</v>
       </c>
-      <c r="D35" s="30"/>
+      <c r="D35" s="31"/>
     </row>
     <row r="36" ht="28.800000000000001" customHeight="1">
-      <c r="A36" s="40"/>
-      <c r="B36" s="29" t="s">
+      <c r="A36" s="41"/>
+      <c r="B36" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="C36" s="30" t="s">
+      <c r="C36" s="31" t="s">
         <v>86</v>
       </c>
-      <c r="D36" s="30" t="s">
+      <c r="D36" s="31" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="37" ht="29.399999999999999" customHeight="1">
-      <c r="A37" s="40"/>
-      <c r="B37" s="29" t="s">
+      <c r="A37" s="41"/>
+      <c r="B37" s="30" t="s">
         <v>88</v>
       </c>
-      <c r="C37" s="30" t="s">
+      <c r="C37" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="D37" s="30" t="s">
+      <c r="D37" s="31" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="38" ht="42.75">
-      <c r="A38" s="40"/>
-      <c r="B38" s="29" t="s">
+      <c r="A38" s="41"/>
+      <c r="B38" s="30" t="s">
         <v>91</v>
       </c>
-      <c r="C38" s="30" t="s">
+      <c r="C38" s="31" t="s">
         <v>92</v>
       </c>
-      <c r="D38" s="30" t="s">
+      <c r="D38" s="31" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="39" ht="28.800000000000001" customHeight="1">
-      <c r="A39" s="40"/>
-      <c r="B39" s="29"/>
-      <c r="C39" s="30"/>
-      <c r="D39" s="30"/>
+      <c r="A39" s="41"/>
+      <c r="B39" s="30"/>
+      <c r="C39" s="31"/>
+      <c r="D39" s="31"/>
     </row>
     <row r="40" ht="28.800000000000001" customHeight="1">
-      <c r="A40" s="40"/>
-      <c r="B40" s="29"/>
-      <c r="C40" s="30"/>
-      <c r="D40" s="30"/>
+      <c r="A40" s="41"/>
+      <c r="B40" s="30"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="31"/>
     </row>
     <row r="41" ht="28.5" customHeight="1">
-      <c r="A41" s="40"/>
-      <c r="B41" s="29"/>
-      <c r="C41" s="30"/>
-      <c r="D41" s="30"/>
+      <c r="A41" s="41"/>
+      <c r="B41" s="30"/>
+      <c r="C41" s="31"/>
+      <c r="D41" s="31"/>
     </row>
     <row r="42" ht="28.5" customHeight="1">
-      <c r="A42" s="40"/>
-      <c r="B42" s="29"/>
-      <c r="C42" s="30"/>
-      <c r="D42" s="30"/>
+      <c r="A42" s="41"/>
+      <c r="B42" s="30"/>
+      <c r="C42" s="31"/>
+      <c r="D42" s="31"/>
     </row>
     <row r="43" ht="28.5" customHeight="1">
-      <c r="A43" s="40"/>
-      <c r="B43" s="29"/>
-      <c r="C43" s="30"/>
-      <c r="D43" s="30"/>
+      <c r="A43" s="41"/>
+      <c r="B43" s="30"/>
+      <c r="C43" s="31"/>
+      <c r="D43" s="31"/>
     </row>
     <row r="44" ht="28.5" customHeight="1">
-      <c r="A44" s="40"/>
-      <c r="B44" s="29"/>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
+      <c r="A44" s="41"/>
+      <c r="B44" s="30"/>
+      <c r="C44" s="31"/>
+      <c r="D44" s="31"/>
     </row>
     <row r="45" ht="28.5" customHeight="1">
-      <c r="A45" s="40"/>
-      <c r="B45" s="29"/>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
+      <c r="A45" s="41"/>
+      <c r="B45" s="30"/>
+      <c r="C45" s="31"/>
+      <c r="D45" s="31"/>
     </row>
     <row r="46" ht="28.5" customHeight="1">
-      <c r="B46" s="24"/>
-      <c r="C46" s="25"/>
-      <c r="D46" s="25"/>
+      <c r="B46" s="25"/>
+      <c r="C46" s="26"/>
+      <c r="D46" s="26"/>
     </row>
     <row r="47" ht="28.5" customHeight="1">
-      <c r="B47" s="24"/>
-      <c r="C47" s="25"/>
-      <c r="D47" s="25"/>
+      <c r="B47" s="25"/>
+      <c r="C47" s="26"/>
+      <c r="D47" s="26"/>
     </row>
     <row r="48" ht="28.5" customHeight="1"/>
     <row r="49" ht="28.5" customHeight="1"/>
@@ -2126,7 +2142,7 @@
       <c r="A3" t="s">
         <v>101</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="42" t="s">
         <v>102</v>
       </c>
       <c r="C3" t="s">
@@ -2143,7 +2159,7 @@
       <c r="B4" t="s">
         <v>104</v>
       </c>
-      <c r="C4" s="42" t="s">
+      <c r="C4" s="43" t="s">
         <v>99</v>
       </c>
       <c r="D4" t="s">
@@ -2157,15 +2173,41 @@
       <c r="B5" t="s">
         <v>107</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="C5" s="43" t="s">
         <v>99</v>
       </c>
       <c r="D5" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="6" ht="14.25" customHeight="1"/>
-    <row r="7" ht="14.25" customHeight="1"/>
+    <row r="6" ht="14.25" customHeight="1">
+      <c r="A6" s="42" t="s">
+        <v>109</v>
+      </c>
+      <c r="B6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" s="43" t="s">
+        <v>99</v>
+      </c>
+      <c r="D6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25" customHeight="1">
+      <c r="A7" s="42" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C7" s="43" t="s">
+        <v>99</v>
+      </c>
+      <c r="D7" t="s">
+        <v>114</v>
+      </c>
+    </row>
     <row r="8" ht="14.25" customHeight="1"/>
     <row r="9" ht="14.25" customHeight="1"/>
     <row r="10" ht="14.25" customHeight="1"/>
@@ -3172,73 +3214,73 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.57421875"/>
-    <col customWidth="1" min="2" max="2" style="43" width="38.421875"/>
+    <col customWidth="1" min="2" max="2" style="44" width="38.421875"/>
     <col customWidth="1" min="3" max="3" width="55.421875"/>
     <col customWidth="1" min="4" max="4" width="75.8515625"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="28" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" s="43" customFormat="1" ht="42.75">
-      <c r="A2" s="44"/>
-      <c r="B2" s="45" t="s">
-        <v>109</v>
-      </c>
-      <c r="C2" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="D2" s="46" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="3" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A3" s="44"/>
-      <c r="B3" s="45" t="s">
-        <v>112</v>
-      </c>
-      <c r="C3" s="46" t="s">
-        <v>113</v>
-      </c>
-      <c r="D3" s="46"/>
-    </row>
-    <row r="4" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A4" s="44"/>
-      <c r="B4" s="45"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-    </row>
-    <row r="5" s="43" customFormat="1" ht="57">
-      <c r="A5" s="44"/>
+    <row r="2" s="44" customFormat="1" ht="42.75">
+      <c r="A2" s="45"/>
+      <c r="B2" s="46" t="s">
+        <v>115</v>
+      </c>
+      <c r="C2" s="47" t="s">
+        <v>116</v>
+      </c>
+      <c r="D2" s="47" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="3" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A3" s="45"/>
+      <c r="B3" s="46" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" s="47" t="s">
+        <v>119</v>
+      </c>
+      <c r="D3" s="47"/>
+    </row>
+    <row r="4" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A4" s="45"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+    </row>
+    <row r="5" s="44" customFormat="1" ht="57">
+      <c r="A5" s="45"/>
       <c r="B5" s="47" t="s">
-        <v>114</v>
-      </c>
-      <c r="C5" s="46" t="s">
-        <v>115</v>
+        <v>120</v>
+      </c>
+      <c r="C5" s="47" t="s">
+        <v>121</v>
       </c>
       <c r="D5" s="48" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="6" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A6" s="44"/>
-      <c r="B6" s="45"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-    </row>
-    <row r="7" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A7" s="44"/>
-      <c r="B7" s="45"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
+        <v>122</v>
+      </c>
+    </row>
+    <row r="6" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A6" s="45"/>
+      <c r="B6" s="46"/>
+      <c r="C6" s="47"/>
+      <c r="D6" s="47"/>
+    </row>
+    <row r="7" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A7" s="45"/>
+      <c r="B7" s="46"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" s="5"/>
@@ -3248,76 +3290,76 @@
     </row>
     <row r="9" ht="41.25" customHeight="1">
       <c r="A9" s="50" t="s">
-        <v>117</v>
-      </c>
-      <c r="B9" s="29" t="s">
-        <v>118</v>
+        <v>123</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>124</v>
       </c>
       <c r="C9" s="51" t="s">
-        <v>119</v>
-      </c>
-      <c r="D9" s="30" t="s">
-        <v>120</v>
+        <v>125</v>
+      </c>
+      <c r="D9" s="31" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
       <c r="A10" s="52"/>
-      <c r="B10" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="C10" s="30">
+      <c r="B10" s="30" t="s">
+        <v>127</v>
+      </c>
+      <c r="C10" s="31">
         <v>60000</v>
       </c>
-      <c r="D10" s="30" t="s">
-        <v>122</v>
+      <c r="D10" s="31" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="11" ht="36.75" customHeight="1">
       <c r="A11" s="52"/>
-      <c r="B11" s="29" t="s">
-        <v>123</v>
-      </c>
-      <c r="C11" s="30">
+      <c r="B11" s="30" t="s">
+        <v>129</v>
+      </c>
+      <c r="C11" s="31">
         <v>3000</v>
       </c>
-      <c r="D11" s="30" t="s">
-        <v>124</v>
+      <c r="D11" s="31" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
       <c r="A12" s="52"/>
-      <c r="B12" s="29" t="s">
-        <v>125</v>
-      </c>
-      <c r="C12" s="30" t="s">
-        <v>126</v>
-      </c>
-      <c r="D12" s="30" t="s">
-        <v>127</v>
+      <c r="B12" s="30" t="s">
+        <v>131</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>132</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="52"/>
-      <c r="B13" s="29" t="s">
-        <v>128</v>
+      <c r="B13" s="30" t="s">
+        <v>134</v>
       </c>
       <c r="C13" s="53" t="s">
-        <v>129</v>
-      </c>
-      <c r="D13" s="30" t="s">
-        <v>130</v>
+        <v>135</v>
+      </c>
+      <c r="D13" s="31" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="14" ht="63.600000000000001" customHeight="1">
       <c r="A14" s="52"/>
-      <c r="B14" s="29" t="s">
-        <v>131</v>
+      <c r="B14" s="30" t="s">
+        <v>137</v>
       </c>
       <c r="C14" s="53" t="s">
-        <v>132</v>
-      </c>
-      <c r="D14" s="30" t="s">
-        <v>133</v>
+        <v>138</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="15" ht="14.25">

</xml_diff>

<commit_message>
Estruturada lógica de alteração das datas de fechamento e de periodo de trabalho.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="149">
   <si>
     <t>Name</t>
   </si>
@@ -284,6 +284,12 @@
     <t xml:space="preserve">Mensagem de integração da obrigação no backoffice quando o processo for bem sucedido.</t>
   </si>
   <si>
+    <t>LogMessage_SuccessOpenWorkPeriod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Periodo de trabalho aberto com sucesso!</t>
+  </si>
+  <si>
     <t xml:space="preserve">INFORMATION MESSAGES</t>
   </si>
   <si>
@@ -317,6 +323,18 @@
     <t xml:space="preserve">Não existem despesas com a conta de débito especificada: </t>
   </si>
   <si>
+    <t>LogMessage_OpenWorkPeriod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abrindo periodo de trabalho...</t>
+  </si>
+  <si>
+    <t>LogMessage_OpenClosing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abrindo periodo de fechamento...</t>
+  </si>
+  <si>
     <t xml:space="preserve">EXCEPTION LOG MESSAGES</t>
   </si>
   <si>
@@ -477,6 +495,15 @@
   </si>
   <si>
     <t xml:space="preserve">O Domínio pode apresentar erro de acordo com a quantidade de despesas inseridas em um determinado arquivo de importação. Por isso, existem as contas de débito específicas que devem estar separadas por arquivo de importação.Deve estar no fomraco "contaDeDebito,contaDeDebito,contaDeDebito"</t>
+  </si>
+  <si>
+    <t>dateEndWorkPeriod</t>
+  </si>
+  <si>
+    <t>01/01/2030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data final do periodo de trabalho cadastrado no sistema Domínio.</t>
   </si>
   <si>
     <t>GetExpensesSettings</t>
@@ -673,7 +700,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -795,6 +822,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1778,8 +1808,12 @@
     </row>
     <row r="14" ht="28.199999999999999" customHeight="1">
       <c r="A14" s="38"/>
-      <c r="B14" s="30"/>
-      <c r="C14" s="31"/>
+      <c r="B14" s="30" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="31" t="s">
+        <v>59</v>
+      </c>
       <c r="D14" s="31"/>
     </row>
     <row r="15" ht="28.199999999999999" customHeight="1">
@@ -1814,60 +1848,68 @@
     </row>
     <row r="20" ht="27" customHeight="1">
       <c r="A20" s="40" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B20" s="30" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C20" s="31" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D20" s="31" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" ht="27" customHeight="1">
       <c r="A21" s="40"/>
       <c r="B21" s="30" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C21" s="31" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D21" s="31" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" ht="33.75" customHeight="1">
       <c r="A22" s="40"/>
       <c r="B22" s="31" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C22" s="31" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D22" s="31"/>
     </row>
     <row r="23" ht="27" customHeight="1">
       <c r="A23" s="40"/>
       <c r="B23" s="30" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C23" s="31" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D23" s="31"/>
     </row>
     <row r="24" ht="27" customHeight="1">
       <c r="A24" s="40"/>
-      <c r="B24" s="30"/>
-      <c r="C24" s="31"/>
+      <c r="B24" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="31" t="s">
+        <v>72</v>
+      </c>
       <c r="D24" s="31"/>
     </row>
     <row r="25" ht="27" customHeight="1">
       <c r="A25" s="40"/>
-      <c r="B25" s="30"/>
-      <c r="C25" s="20"/>
+      <c r="B25" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>74</v>
+      </c>
       <c r="D25" s="31"/>
     </row>
     <row r="26" ht="27" customHeight="1">
@@ -1896,111 +1938,111 @@
     </row>
     <row r="30" ht="27.75" customHeight="1">
       <c r="A30" s="41" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="B30" s="30" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C30" s="31" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D30" s="31" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" ht="27.75" customHeight="1">
       <c r="A31" s="41"/>
       <c r="B31" s="30" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C31" s="31" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D31" s="31" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
     </row>
     <row r="32" ht="28.5">
       <c r="A32" s="41"/>
       <c r="B32" s="30" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C32" s="31" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="D32" s="31"/>
     </row>
     <row r="33" ht="28.5">
       <c r="A33" s="41"/>
       <c r="B33" s="30" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D33" s="31"/>
     </row>
     <row r="34" ht="27.75" customHeight="1">
       <c r="A34" s="41"/>
       <c r="B34" s="30" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="D34" s="31" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="35" ht="31.199999999999999" customHeight="1">
       <c r="A35" s="41"/>
       <c r="B35" s="30" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C35" s="31" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="D35" s="31"/>
     </row>
     <row r="36" ht="28.800000000000001" customHeight="1">
       <c r="A36" s="41"/>
       <c r="B36" s="30" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="C36" s="31" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="D36" s="31" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="37" ht="29.399999999999999" customHeight="1">
       <c r="A37" s="41"/>
       <c r="B37" s="30" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C37" s="31" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="D37" s="31" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="38" ht="42.75">
       <c r="A38" s="41"/>
       <c r="B38" s="30" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C38" s="31" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D38" s="31" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
     </row>
     <row r="39" ht="28.800000000000001" customHeight="1">
       <c r="A39" s="41"/>
-      <c r="B39" s="30"/>
+      <c r="B39" s="31"/>
       <c r="C39" s="31"/>
       <c r="D39" s="31"/>
     </row>
@@ -2093,13 +2135,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -2126,86 +2168,86 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C2" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B3" s="42" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C3" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D3" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D4" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B5" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D5" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="42" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B6" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="42" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B7" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D7" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1"/>
@@ -3233,22 +3275,22 @@
     <row r="2" s="44" customFormat="1" ht="42.75">
       <c r="A2" s="45"/>
       <c r="B2" s="46" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C2" s="47" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D2" s="47" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
       <c r="A3" s="45"/>
       <c r="B3" s="46" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C3" s="47" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D3" s="47"/>
     </row>
@@ -3261,20 +3303,26 @@
     <row r="5" s="44" customFormat="1" ht="57">
       <c r="A5" s="45"/>
       <c r="B5" s="47" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C5" s="47" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="D5" s="48" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
       <c r="A6" s="45"/>
-      <c r="B6" s="46"/>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
+      <c r="B6" s="46" t="s">
+        <v>129</v>
+      </c>
+      <c r="C6" s="49" t="s">
+        <v>130</v>
+      </c>
+      <c r="D6" s="47" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="7" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
       <c r="A7" s="45"/>
@@ -3284,87 +3332,87 @@
     </row>
     <row r="8" ht="14.25">
       <c r="A8" s="5"/>
-      <c r="B8" s="49"/>
+      <c r="B8" s="50"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
     </row>
     <row r="9" ht="41.25" customHeight="1">
-      <c r="A9" s="50" t="s">
-        <v>123</v>
+      <c r="A9" s="51" t="s">
+        <v>132</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>124</v>
-      </c>
-      <c r="C9" s="51" t="s">
-        <v>125</v>
+        <v>133</v>
+      </c>
+      <c r="C9" s="52" t="s">
+        <v>134</v>
       </c>
       <c r="D9" s="31" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="52"/>
+      <c r="A10" s="53"/>
       <c r="B10" s="30" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="C10" s="31">
         <v>60000</v>
       </c>
       <c r="D10" s="31" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" ht="36.75" customHeight="1">
-      <c r="A11" s="52"/>
+      <c r="A11" s="53"/>
       <c r="B11" s="30" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="C11" s="31">
         <v>3000</v>
       </c>
       <c r="D11" s="31" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="52"/>
+      <c r="A12" s="53"/>
       <c r="B12" s="30" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="D12" s="31" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="52"/>
+      <c r="A13" s="53"/>
       <c r="B13" s="30" t="s">
-        <v>134</v>
-      </c>
-      <c r="C13" s="53" t="s">
-        <v>135</v>
+        <v>143</v>
+      </c>
+      <c r="C13" s="54" t="s">
+        <v>144</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14" ht="63.600000000000001" customHeight="1">
-      <c r="A14" s="52"/>
+      <c r="A14" s="53"/>
       <c r="B14" s="30" t="s">
-        <v>137</v>
-      </c>
-      <c r="C14" s="53" t="s">
-        <v>138</v>
+        <v>146</v>
+      </c>
+      <c r="C14" s="54" t="s">
+        <v>147</v>
       </c>
       <c r="D14" s="31" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" s="5"/>
-      <c r="B15" s="49"/>
+      <c r="B15" s="50"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>

</xml_diff>

<commit_message>
Adicionando preenchumento do formulário de importação
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="151">
   <si>
     <t>Name</t>
   </si>
@@ -110,10 +110,16 @@
     <t>obligationDateStart</t>
   </si>
   <si>
+    <t>01/03/2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">Data inicial do range de datas que deve abranger a data de vencimento da obrigação em questão, se não estiver definida nenhuma data nessa variável, o processo define o primeiro e o ultimo dia do mês como as datas de inicio e fim do range.</t>
   </si>
   <si>
     <t>obligationDateEnd</t>
+  </si>
+  <si>
+    <t>05/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Data final do range de datas que deve abranger a data de vencimento da obrigação em questão, se não estiver definida nenhuma data nessa variável, o processo define o primeiro e o ultimo dia do mês como as datas de inicio e fim do range.</t>
@@ -700,7 +706,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -742,6 +748,9 @@
     </xf>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -1479,25 +1488,29 @@
       <c r="B11" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="16"/>
+      <c r="C11" s="16" t="s">
+        <v>16</v>
+      </c>
       <c r="D11" s="15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" ht="61.200000000000003" customHeight="1">
       <c r="A12" s="13"/>
       <c r="B12" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="15" t="s">
         <v>18</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="13" ht="28.800000000000001" customHeight="1">
       <c r="A13" s="13"/>
       <c r="B13" s="14" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C13" s="14" t="b">
         <v>1</v>
@@ -1507,7 +1520,7 @@
     <row r="14" ht="28.800000000000001" customHeight="1">
       <c r="A14" s="13"/>
       <c r="B14" s="14" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C14" s="14" t="b">
         <v>0</v>
@@ -1516,24 +1529,24 @@
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="13"/>
-      <c r="B15" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="20" t="s">
-        <v>22</v>
+      <c r="B15" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="16" ht="34.799999999999997" customHeight="1">
       <c r="A16" s="13"/>
-      <c r="B16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="20" t="s">
+      <c r="B16" s="19" t="s">
         <v>25</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="21" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="17" ht="17.399999999999999" customHeight="1">
@@ -1543,36 +1556,36 @@
       <c r="D17" s="5"/>
     </row>
     <row r="18" ht="46.799999999999997" customHeight="1">
-      <c r="A18" s="22" t="s">
-        <v>26</v>
+      <c r="A18" s="23" t="s">
+        <v>28</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="23" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>30</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" ht="46.799999999999997" customHeight="1">
-      <c r="A19" s="22"/>
+      <c r="A19" s="23"/>
       <c r="B19" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C19" s="24" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>33</v>
       </c>
       <c r="D19" s="14"/>
     </row>
     <row r="20" ht="43.200000000000003" customHeight="1">
-      <c r="A20" s="22"/>
+      <c r="A20" s="23"/>
       <c r="B20" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="C20" s="24" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>35</v>
       </c>
       <c r="D20" s="14"/>
     </row>
@@ -1630,20 +1643,20 @@
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8.00390625"/>
-    <col customWidth="1" min="2" max="2" style="25" width="52.140625"/>
-    <col bestFit="1" customWidth="1" min="3" max="3" style="26" width="63.11328125"/>
-    <col customWidth="1" min="4" max="4" style="26" width="84.140625"/>
+    <col customWidth="1" min="2" max="2" style="26" width="52.140625"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" style="27" width="63.11328125"/>
+    <col customWidth="1" min="4" max="4" style="27" width="84.140625"/>
     <col customWidth="1" min="5" max="27" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="29" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="2"/>
@@ -1671,426 +1684,426 @@
       <c r="AA1" s="2"/>
     </row>
     <row r="2" ht="28.5">
-      <c r="A2" s="29"/>
-      <c r="B2" s="30" t="s">
-        <v>34</v>
-      </c>
-      <c r="C2" s="31">
+      <c r="A2" s="30"/>
+      <c r="B2" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="32">
         <v>1</v>
       </c>
-      <c r="D2" s="31" t="s">
-        <v>35</v>
+      <c r="D2" s="32" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="3" ht="28.5">
-      <c r="A3" s="29"/>
-      <c r="B3" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="C3" s="31">
+      <c r="A3" s="30"/>
+      <c r="B3" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="32">
         <v>3</v>
       </c>
-      <c r="D3" s="31" t="s">
-        <v>37</v>
+      <c r="D3" s="32" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="29"/>
-      <c r="B4" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="31" t="s">
+      <c r="A4" s="30"/>
+      <c r="B4" s="31" t="s">
         <v>40</v>
       </c>
+      <c r="C4" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" s="32" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="5" ht="28.5">
-      <c r="A5" s="29"/>
-      <c r="B5" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="31">
+      <c r="A5" s="30"/>
+      <c r="B5" s="31" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="32">
         <v>2</v>
       </c>
-      <c r="D5" s="31" t="s">
-        <v>42</v>
+      <c r="D5" s="32" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="6" ht="28.5">
-      <c r="A6" s="29"/>
-      <c r="B6" s="30" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" s="31">
+      <c r="A6" s="30"/>
+      <c r="B6" s="31" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="32">
         <v>2</v>
       </c>
-      <c r="D6" s="31" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" s="32" customFormat="1" ht="17.399999999999999" customHeight="1">
+      <c r="D6" s="32" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" s="33" customFormat="1" ht="17.399999999999999" customHeight="1">
       <c r="A7" s="5"/>
-      <c r="B7" s="33"/>
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
     </row>
     <row r="8" ht="39.75" customHeight="1">
-      <c r="A8" s="35" t="s">
-        <v>45</v>
+      <c r="A8" s="36" t="s">
+        <v>47</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C8" s="36">
+        <v>48</v>
+      </c>
+      <c r="C8" s="37">
         <v>30000</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" ht="39.75" customHeight="1">
-      <c r="A9" s="37"/>
+      <c r="A9" s="38"/>
       <c r="B9" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="36">
+        <v>50</v>
+      </c>
+      <c r="C9" s="37">
         <v>20000</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="37"/>
+      <c r="A10" s="38"/>
       <c r="B10" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="36">
+        <v>52</v>
+      </c>
+      <c r="C10" s="37">
         <v>0</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="37"/>
+      <c r="A11" s="38"/>
       <c r="B11" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="C11" s="36">
+        <v>54</v>
+      </c>
+      <c r="C11" s="37">
         <v>0</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" ht="17.399999999999999" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="33"/>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
     </row>
     <row r="13" ht="22.800000000000001" customHeight="1">
-      <c r="A13" s="38" t="s">
-        <v>54</v>
-      </c>
-      <c r="B13" s="30" t="s">
-        <v>55</v>
-      </c>
-      <c r="C13" s="31" t="s">
+      <c r="A13" s="39" t="s">
         <v>56</v>
       </c>
-      <c r="D13" s="31" t="s">
+      <c r="B13" s="31" t="s">
         <v>57</v>
       </c>
+      <c r="C13" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" s="32" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="14" ht="28.199999999999999" customHeight="1">
-      <c r="A14" s="38"/>
-      <c r="B14" s="30" t="s">
-        <v>58</v>
-      </c>
-      <c r="C14" s="31" t="s">
-        <v>59</v>
-      </c>
-      <c r="D14" s="31"/>
+      <c r="A14" s="39"/>
+      <c r="B14" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="D14" s="32"/>
     </row>
     <row r="15" ht="28.199999999999999" customHeight="1">
-      <c r="A15" s="38"/>
-      <c r="B15" s="30"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
+      <c r="A15" s="39"/>
+      <c r="B15" s="31"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
     </row>
     <row r="16" ht="27" customHeight="1">
-      <c r="A16" s="38"/>
-      <c r="B16" s="30"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="31"/>
+      <c r="A16" s="39"/>
+      <c r="B16" s="31"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
     </row>
     <row r="17" ht="27" customHeight="1">
-      <c r="A17" s="38"/>
-      <c r="B17" s="30"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="31"/>
+      <c r="A17" s="39"/>
+      <c r="B17" s="31"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="32"/>
     </row>
     <row r="18" ht="27" customHeight="1">
-      <c r="A18" s="38"/>
-      <c r="B18" s="30"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
+      <c r="A18" s="39"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
     </row>
     <row r="19" ht="17.399999999999999" customHeight="1">
-      <c r="A19" s="39"/>
-      <c r="B19" s="33"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
+      <c r="A19" s="40"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
     </row>
     <row r="20" ht="27" customHeight="1">
-      <c r="A20" s="40" t="s">
-        <v>60</v>
-      </c>
-      <c r="B20" s="30" t="s">
-        <v>61</v>
-      </c>
-      <c r="C20" s="31" t="s">
+      <c r="A20" s="41" t="s">
         <v>62</v>
       </c>
-      <c r="D20" s="31" t="s">
+      <c r="B20" s="31" t="s">
         <v>63</v>
       </c>
+      <c r="C20" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="D20" s="32" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="21" ht="27" customHeight="1">
-      <c r="A21" s="40"/>
-      <c r="B21" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="C21" s="31" t="s">
-        <v>65</v>
-      </c>
-      <c r="D21" s="31" t="s">
+      <c r="A21" s="41"/>
+      <c r="B21" s="31" t="s">
         <v>66</v>
       </c>
+      <c r="C21" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="D21" s="32" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="22" ht="33.75" customHeight="1">
-      <c r="A22" s="40"/>
-      <c r="B22" s="31" t="s">
-        <v>67</v>
-      </c>
-      <c r="C22" s="31" t="s">
-        <v>68</v>
-      </c>
-      <c r="D22" s="31"/>
+      <c r="A22" s="41"/>
+      <c r="B22" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="D22" s="32"/>
     </row>
     <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="40"/>
-      <c r="B23" s="30" t="s">
-        <v>69</v>
-      </c>
-      <c r="C23" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="D23" s="31"/>
+      <c r="A23" s="41"/>
+      <c r="B23" s="31" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="D23" s="32"/>
     </row>
     <row r="24" ht="27" customHeight="1">
-      <c r="A24" s="40"/>
-      <c r="B24" s="30" t="s">
-        <v>71</v>
-      </c>
-      <c r="C24" s="31" t="s">
-        <v>72</v>
-      </c>
-      <c r="D24" s="31"/>
+      <c r="A24" s="41"/>
+      <c r="B24" s="31" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="D24" s="32"/>
     </row>
     <row r="25" ht="27" customHeight="1">
-      <c r="A25" s="40"/>
-      <c r="B25" s="30" t="s">
-        <v>73</v>
-      </c>
-      <c r="C25" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="D25" s="31"/>
+      <c r="A25" s="41"/>
+      <c r="B25" s="31" t="s">
+        <v>75</v>
+      </c>
+      <c r="C25" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D25" s="32"/>
     </row>
     <row r="26" ht="27" customHeight="1">
-      <c r="A26" s="40"/>
-      <c r="B26" s="30"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="31"/>
+      <c r="A26" s="41"/>
+      <c r="B26" s="31"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
     </row>
     <row r="27" ht="27" customHeight="1">
-      <c r="A27" s="40"/>
-      <c r="B27" s="30"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
+      <c r="A27" s="41"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
     </row>
     <row r="28" ht="27" customHeight="1">
-      <c r="A28" s="40"/>
-      <c r="B28" s="30"/>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
+      <c r="A28" s="41"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
     </row>
     <row r="29" ht="17.399999999999999" customHeight="1">
       <c r="A29" s="5"/>
-      <c r="B29" s="33"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="34"/>
+      <c r="B29" s="34"/>
+      <c r="C29" s="35"/>
+      <c r="D29" s="35"/>
     </row>
     <row r="30" ht="27.75" customHeight="1">
-      <c r="A30" s="41" t="s">
-        <v>75</v>
-      </c>
-      <c r="B30" s="30" t="s">
-        <v>76</v>
-      </c>
-      <c r="C30" s="31" t="s">
+      <c r="A30" s="42" t="s">
         <v>77</v>
       </c>
-      <c r="D30" s="31" t="s">
+      <c r="B30" s="31" t="s">
         <v>78</v>
       </c>
+      <c r="C30" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="D30" s="32" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="31" ht="27.75" customHeight="1">
-      <c r="A31" s="41"/>
-      <c r="B31" s="30" t="s">
-        <v>79</v>
-      </c>
-      <c r="C31" s="31" t="s">
-        <v>80</v>
-      </c>
-      <c r="D31" s="31" t="s">
+      <c r="A31" s="42"/>
+      <c r="B31" s="31" t="s">
         <v>81</v>
       </c>
+      <c r="C31" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="D31" s="32" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="32" ht="28.5">
-      <c r="A32" s="41"/>
-      <c r="B32" s="30" t="s">
-        <v>82</v>
-      </c>
-      <c r="C32" s="31" t="s">
-        <v>83</v>
-      </c>
-      <c r="D32" s="31"/>
+      <c r="A32" s="42"/>
+      <c r="B32" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="C32" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="D32" s="32"/>
     </row>
     <row r="33" ht="28.5">
-      <c r="A33" s="41"/>
-      <c r="B33" s="30" t="s">
-        <v>84</v>
-      </c>
-      <c r="C33" s="31" t="s">
-        <v>85</v>
-      </c>
-      <c r="D33" s="31"/>
+      <c r="A33" s="42"/>
+      <c r="B33" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="C33" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="D33" s="32"/>
     </row>
     <row r="34" ht="27.75" customHeight="1">
-      <c r="A34" s="41"/>
-      <c r="B34" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="C34" s="31" t="s">
-        <v>87</v>
-      </c>
-      <c r="D34" s="31" t="s">
+      <c r="A34" s="42"/>
+      <c r="B34" s="31" t="s">
         <v>88</v>
       </c>
+      <c r="C34" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="D34" s="32" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="35" ht="31.199999999999999" customHeight="1">
-      <c r="A35" s="41"/>
-      <c r="B35" s="30" t="s">
-        <v>89</v>
-      </c>
-      <c r="C35" s="31" t="s">
-        <v>90</v>
-      </c>
-      <c r="D35" s="31"/>
+      <c r="A35" s="42"/>
+      <c r="B35" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="C35" s="32" t="s">
+        <v>92</v>
+      </c>
+      <c r="D35" s="32"/>
     </row>
     <row r="36" ht="28.800000000000001" customHeight="1">
-      <c r="A36" s="41"/>
-      <c r="B36" s="30" t="s">
-        <v>91</v>
-      </c>
-      <c r="C36" s="31" t="s">
-        <v>92</v>
-      </c>
-      <c r="D36" s="31" t="s">
+      <c r="A36" s="42"/>
+      <c r="B36" s="31" t="s">
         <v>93</v>
       </c>
+      <c r="C36" s="32" t="s">
+        <v>94</v>
+      </c>
+      <c r="D36" s="32" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="37" ht="29.399999999999999" customHeight="1">
-      <c r="A37" s="41"/>
-      <c r="B37" s="30" t="s">
-        <v>94</v>
-      </c>
-      <c r="C37" s="31" t="s">
-        <v>95</v>
-      </c>
-      <c r="D37" s="31" t="s">
+      <c r="A37" s="42"/>
+      <c r="B37" s="31" t="s">
         <v>96</v>
       </c>
+      <c r="C37" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="D37" s="32" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="38" ht="42.75">
-      <c r="A38" s="41"/>
-      <c r="B38" s="30" t="s">
-        <v>97</v>
-      </c>
-      <c r="C38" s="31" t="s">
-        <v>98</v>
-      </c>
-      <c r="D38" s="31" t="s">
+      <c r="A38" s="42"/>
+      <c r="B38" s="31" t="s">
         <v>99</v>
       </c>
+      <c r="C38" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="D38" s="32" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="39" ht="28.800000000000001" customHeight="1">
-      <c r="A39" s="41"/>
-      <c r="B39" s="31"/>
-      <c r="C39" s="31"/>
-      <c r="D39" s="31"/>
+      <c r="A39" s="42"/>
+      <c r="B39" s="32"/>
+      <c r="C39" s="32"/>
+      <c r="D39" s="32"/>
     </row>
     <row r="40" ht="28.800000000000001" customHeight="1">
-      <c r="A40" s="41"/>
-      <c r="B40" s="30"/>
-      <c r="C40" s="31"/>
-      <c r="D40" s="31"/>
+      <c r="A40" s="42"/>
+      <c r="B40" s="31"/>
+      <c r="C40" s="32"/>
+      <c r="D40" s="32"/>
     </row>
     <row r="41" ht="28.5" customHeight="1">
-      <c r="A41" s="41"/>
-      <c r="B41" s="30"/>
-      <c r="C41" s="31"/>
-      <c r="D41" s="31"/>
+      <c r="A41" s="42"/>
+      <c r="B41" s="31"/>
+      <c r="C41" s="32"/>
+      <c r="D41" s="32"/>
     </row>
     <row r="42" ht="28.5" customHeight="1">
-      <c r="A42" s="41"/>
-      <c r="B42" s="30"/>
-      <c r="C42" s="31"/>
-      <c r="D42" s="31"/>
+      <c r="A42" s="42"/>
+      <c r="B42" s="31"/>
+      <c r="C42" s="32"/>
+      <c r="D42" s="32"/>
     </row>
     <row r="43" ht="28.5" customHeight="1">
-      <c r="A43" s="41"/>
-      <c r="B43" s="30"/>
-      <c r="C43" s="31"/>
-      <c r="D43" s="31"/>
+      <c r="A43" s="42"/>
+      <c r="B43" s="31"/>
+      <c r="C43" s="32"/>
+      <c r="D43" s="32"/>
     </row>
     <row r="44" ht="28.5" customHeight="1">
-      <c r="A44" s="41"/>
-      <c r="B44" s="30"/>
-      <c r="C44" s="31"/>
-      <c r="D44" s="31"/>
+      <c r="A44" s="42"/>
+      <c r="B44" s="31"/>
+      <c r="C44" s="32"/>
+      <c r="D44" s="32"/>
     </row>
     <row r="45" ht="28.5" customHeight="1">
-      <c r="A45" s="41"/>
-      <c r="B45" s="30"/>
-      <c r="C45" s="31"/>
-      <c r="D45" s="31"/>
+      <c r="A45" s="42"/>
+      <c r="B45" s="31"/>
+      <c r="C45" s="32"/>
+      <c r="D45" s="32"/>
     </row>
     <row r="46" ht="28.5" customHeight="1">
-      <c r="B46" s="25"/>
-      <c r="C46" s="26"/>
-      <c r="D46" s="26"/>
+      <c r="B46" s="26"/>
+      <c r="C46" s="27"/>
+      <c r="D46" s="27"/>
     </row>
     <row r="47" ht="28.5" customHeight="1">
-      <c r="B47" s="25"/>
-      <c r="C47" s="26"/>
-      <c r="D47" s="26"/>
+      <c r="B47" s="26"/>
+      <c r="C47" s="27"/>
+      <c r="D47" s="27"/>
     </row>
     <row r="48" ht="28.5" customHeight="1"/>
     <row r="49" ht="28.5" customHeight="1"/>
@@ -2135,13 +2148,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -2168,86 +2181,86 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3" t="s">
         <v>107</v>
       </c>
-      <c r="B3" s="42" t="s">
-        <v>108</v>
-      </c>
-      <c r="C3" t="s">
-        <v>105</v>
-      </c>
       <c r="D3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B4" t="s">
-        <v>110</v>
-      </c>
-      <c r="C4" s="43" t="s">
-        <v>105</v>
+        <v>112</v>
+      </c>
+      <c r="C4" s="44" t="s">
+        <v>107</v>
       </c>
       <c r="D4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C5" s="43" t="s">
-        <v>105</v>
+        <v>115</v>
+      </c>
+      <c r="C5" s="44" t="s">
+        <v>107</v>
       </c>
       <c r="D5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="42" t="s">
-        <v>115</v>
+      <c r="A6" s="43" t="s">
+        <v>117</v>
       </c>
       <c r="B6" t="s">
-        <v>116</v>
-      </c>
-      <c r="C6" s="43" t="s">
-        <v>105</v>
+        <v>118</v>
+      </c>
+      <c r="C6" s="44" t="s">
+        <v>107</v>
       </c>
       <c r="D6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="42" t="s">
-        <v>118</v>
+      <c r="A7" s="43" t="s">
+        <v>120</v>
       </c>
       <c r="B7" t="s">
-        <v>119</v>
-      </c>
-      <c r="C7" s="43" t="s">
-        <v>105</v>
+        <v>121</v>
+      </c>
+      <c r="C7" s="44" t="s">
+        <v>107</v>
       </c>
       <c r="D7" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1"/>
@@ -3256,163 +3269,163 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.57421875"/>
-    <col customWidth="1" min="2" max="2" style="44" width="38.421875"/>
+    <col customWidth="1" min="2" max="2" style="45" width="38.421875"/>
     <col customWidth="1" min="3" max="3" width="55.421875"/>
     <col customWidth="1" min="4" max="4" width="75.8515625"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="29" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" s="44" customFormat="1" ht="42.75">
-      <c r="A2" s="45"/>
-      <c r="B2" s="46" t="s">
-        <v>121</v>
-      </c>
-      <c r="C2" s="47" t="s">
-        <v>122</v>
-      </c>
-      <c r="D2" s="47" t="s">
+    <row r="2" s="45" customFormat="1" ht="42.75">
+      <c r="A2" s="46"/>
+      <c r="B2" s="47" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="3" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A3" s="45"/>
-      <c r="B3" s="46" t="s">
+      <c r="C2" s="48" t="s">
         <v>124</v>
       </c>
-      <c r="C3" s="47" t="s">
+      <c r="D2" s="48" t="s">
         <v>125</v>
       </c>
-      <c r="D3" s="47"/>
-    </row>
-    <row r="4" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A4" s="45"/>
-      <c r="B4" s="46"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
-    </row>
-    <row r="5" s="44" customFormat="1" ht="57">
-      <c r="A5" s="45"/>
-      <c r="B5" s="47" t="s">
+    </row>
+    <row r="3" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A3" s="46"/>
+      <c r="B3" s="47" t="s">
         <v>126</v>
       </c>
-      <c r="C5" s="47" t="s">
+      <c r="C3" s="48" t="s">
         <v>127</v>
       </c>
-      <c r="D5" s="48" t="s">
+      <c r="D3" s="48"/>
+    </row>
+    <row r="4" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A4" s="46"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+    </row>
+    <row r="5" s="45" customFormat="1" ht="57">
+      <c r="A5" s="46"/>
+      <c r="B5" s="48" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="6" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A6" s="45"/>
-      <c r="B6" s="46" t="s">
+      <c r="C5" s="48" t="s">
         <v>129</v>
       </c>
-      <c r="C6" s="49" t="s">
+      <c r="D5" s="49" t="s">
         <v>130</v>
       </c>
-      <c r="D6" s="47" t="s">
+    </row>
+    <row r="6" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A6" s="46"/>
+      <c r="B6" s="47" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="7" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A7" s="45"/>
-      <c r="B7" s="46"/>
-      <c r="C7" s="47"/>
-      <c r="D7" s="47"/>
+      <c r="C6" s="50" t="s">
+        <v>132</v>
+      </c>
+      <c r="D6" s="48" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A7" s="46"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" s="5"/>
-      <c r="B8" s="50"/>
+      <c r="B8" s="51"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
     </row>
     <row r="9" ht="41.25" customHeight="1">
-      <c r="A9" s="51" t="s">
-        <v>132</v>
-      </c>
-      <c r="B9" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="C9" s="52" t="s">
+      <c r="A9" s="52" t="s">
         <v>134</v>
       </c>
-      <c r="D9" s="31" t="s">
+      <c r="B9" s="31" t="s">
         <v>135</v>
       </c>
+      <c r="C9" s="53" t="s">
+        <v>136</v>
+      </c>
+      <c r="D9" s="32" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="53"/>
-      <c r="B10" s="30" t="s">
-        <v>136</v>
-      </c>
-      <c r="C10" s="31">
+      <c r="A10" s="54"/>
+      <c r="B10" s="31" t="s">
+        <v>138</v>
+      </c>
+      <c r="C10" s="32">
         <v>60000</v>
       </c>
-      <c r="D10" s="31" t="s">
-        <v>137</v>
+      <c r="D10" s="32" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="11" ht="36.75" customHeight="1">
-      <c r="A11" s="53"/>
-      <c r="B11" s="30" t="s">
-        <v>138</v>
-      </c>
-      <c r="C11" s="31">
+      <c r="A11" s="54"/>
+      <c r="B11" s="31" t="s">
+        <v>140</v>
+      </c>
+      <c r="C11" s="32">
         <v>3000</v>
       </c>
-      <c r="D11" s="31" t="s">
-        <v>139</v>
+      <c r="D11" s="32" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="53"/>
-      <c r="B12" s="30" t="s">
-        <v>140</v>
-      </c>
-      <c r="C12" s="31" t="s">
-        <v>141</v>
-      </c>
-      <c r="D12" s="31" t="s">
+      <c r="A12" s="54"/>
+      <c r="B12" s="31" t="s">
         <v>142</v>
       </c>
+      <c r="C12" s="32" t="s">
+        <v>143</v>
+      </c>
+      <c r="D12" s="32" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="53"/>
-      <c r="B13" s="30" t="s">
-        <v>143</v>
-      </c>
-      <c r="C13" s="54" t="s">
-        <v>144</v>
-      </c>
-      <c r="D13" s="31" t="s">
+      <c r="A13" s="54"/>
+      <c r="B13" s="31" t="s">
         <v>145</v>
       </c>
+      <c r="C13" s="55" t="s">
+        <v>146</v>
+      </c>
+      <c r="D13" s="32" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="14" ht="63.600000000000001" customHeight="1">
-      <c r="A14" s="53"/>
-      <c r="B14" s="30" t="s">
-        <v>146</v>
-      </c>
-      <c r="C14" s="54" t="s">
-        <v>147</v>
-      </c>
-      <c r="D14" s="31" t="s">
+      <c r="A14" s="54"/>
+      <c r="B14" s="31" t="s">
         <v>148</v>
+      </c>
+      <c r="C14" s="55" t="s">
+        <v>149</v>
+      </c>
+      <c r="D14" s="32" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" s="5"/>
-      <c r="B15" s="50"/>
+      <c r="B15" s="51"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>

</xml_diff>

<commit_message>
Correção de bug na criação dos arquivos de importação e alteração do endereço de escrita dos mesmos.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -482,7 +482,7 @@
     <t>mainPath</t>
   </si>
   <si>
-    <t xml:space="preserve">\\192.168.8.8\Razonet\18- OPERAÇÃO RAZONET\01- ROTINAS AUTOMATICAS\04- LANÇAMENTOS CONTÁBEIS\AUTOMACAO\LANÇAMENTOS DESPESAS</t>
+    <t xml:space="preserve">\\192.168.8.8\Razonet\18- OPERAÇÃO RAZONET\Robo de despesas</t>
   </si>
   <si>
     <t xml:space="preserve">Endereço onde serão alocados os arquivos de importação e relatórios de erros de importação do processo</t>
@@ -706,7 +706,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="55">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -748,16 +748,12 @@
     </xf>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="2" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
     </xf>
@@ -826,6 +822,9 @@
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1503,7 +1502,7 @@
       <c r="C12" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="15" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1529,23 +1528,23 @@
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="13"/>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="21" t="s">
+      <c r="C15" s="19"/>
+      <c r="D15" s="20" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="16" ht="34.799999999999997" customHeight="1">
       <c r="A16" s="13"/>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="D16" s="20" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1556,13 +1555,13 @@
       <c r="D17" s="5"/>
     </row>
     <row r="18" ht="46.799999999999997" customHeight="1">
-      <c r="A18" s="23" t="s">
+      <c r="A18" s="21" t="s">
         <v>28</v>
       </c>
       <c r="B18" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="C18" s="22" t="s">
         <v>30</v>
       </c>
       <c r="D18" s="14" t="s">
@@ -1570,21 +1569,21 @@
       </c>
     </row>
     <row r="19" ht="46.799999999999997" customHeight="1">
-      <c r="A19" s="23"/>
+      <c r="A19" s="21"/>
       <c r="B19" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="25" t="s">
+      <c r="C19" s="23" t="s">
         <v>33</v>
       </c>
       <c r="D19" s="14"/>
     </row>
     <row r="20" ht="43.200000000000003" customHeight="1">
-      <c r="A20" s="23"/>
+      <c r="A20" s="21"/>
       <c r="B20" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="25" t="s">
+      <c r="C20" s="23" t="s">
         <v>35</v>
       </c>
       <c r="D20" s="14"/>
@@ -1643,20 +1642,20 @@
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8.00390625"/>
-    <col customWidth="1" min="2" max="2" style="26" width="52.140625"/>
-    <col bestFit="1" customWidth="1" min="3" max="3" style="27" width="63.11328125"/>
-    <col customWidth="1" min="4" max="4" style="27" width="84.140625"/>
+    <col customWidth="1" min="2" max="2" style="24" width="52.140625"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" style="25" width="63.11328125"/>
+    <col customWidth="1" min="4" max="4" style="25" width="84.140625"/>
     <col customWidth="1" min="5" max="27" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="C1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="D1" s="27" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="2"/>
@@ -1684,79 +1683,79 @@
       <c r="AA1" s="2"/>
     </row>
     <row r="2" ht="28.5">
-      <c r="A2" s="30"/>
-      <c r="B2" s="31" t="s">
+      <c r="A2" s="28"/>
+      <c r="B2" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="32">
+      <c r="C2" s="30">
         <v>1</v>
       </c>
-      <c r="D2" s="32" t="s">
+      <c r="D2" s="30" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="3" ht="28.5">
-      <c r="A3" s="30"/>
-      <c r="B3" s="31" t="s">
+      <c r="A3" s="28"/>
+      <c r="B3" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="32">
+      <c r="C3" s="30">
         <v>3</v>
       </c>
-      <c r="D3" s="32" t="s">
+      <c r="D3" s="30" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="30"/>
-      <c r="B4" s="31" t="s">
+      <c r="A4" s="28"/>
+      <c r="B4" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="32" t="s">
+      <c r="C4" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="30" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="5" ht="28.5">
-      <c r="A5" s="30"/>
-      <c r="B5" s="31" t="s">
+      <c r="A5" s="28"/>
+      <c r="B5" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="32">
+      <c r="C5" s="30">
         <v>2</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="D5" s="30" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" ht="28.5">
-      <c r="A6" s="30"/>
-      <c r="B6" s="31" t="s">
+      <c r="A6" s="28"/>
+      <c r="B6" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="32">
+      <c r="C6" s="30">
         <v>2</v>
       </c>
-      <c r="D6" s="32" t="s">
+      <c r="D6" s="30" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="7" s="33" customFormat="1" ht="17.399999999999999" customHeight="1">
+    <row r="7" s="31" customFormat="1" ht="17.399999999999999" customHeight="1">
       <c r="A7" s="5"/>
-      <c r="B7" s="34"/>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
     </row>
     <row r="8" ht="39.75" customHeight="1">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="34" t="s">
         <v>47</v>
       </c>
       <c r="B8" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="37">
+      <c r="C8" s="35">
         <v>30000</v>
       </c>
       <c r="D8" s="15" t="s">
@@ -1764,11 +1763,11 @@
       </c>
     </row>
     <row r="9" ht="39.75" customHeight="1">
-      <c r="A9" s="38"/>
+      <c r="A9" s="36"/>
       <c r="B9" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="37">
+      <c r="C9" s="35">
         <v>20000</v>
       </c>
       <c r="D9" s="15" t="s">
@@ -1776,11 +1775,11 @@
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="38"/>
+      <c r="A10" s="36"/>
       <c r="B10" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="37">
+      <c r="C10" s="35">
         <v>0</v>
       </c>
       <c r="D10" s="15" t="s">
@@ -1788,11 +1787,11 @@
       </c>
     </row>
     <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="38"/>
+      <c r="A11" s="36"/>
       <c r="B11" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="37">
+      <c r="C11" s="35">
         <v>0</v>
       </c>
       <c r="D11" s="15" t="s">
@@ -1801,309 +1800,309 @@
     </row>
     <row r="12" ht="17.399999999999999" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="34"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
     </row>
     <row r="13" ht="22.800000000000001" customHeight="1">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="37" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="32" t="s">
+      <c r="C13" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="32" t="s">
+      <c r="D13" s="30" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="14" ht="28.199999999999999" customHeight="1">
-      <c r="A14" s="39"/>
-      <c r="B14" s="31" t="s">
+      <c r="A14" s="37"/>
+      <c r="B14" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="C14" s="32" t="s">
+      <c r="C14" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="32"/>
+      <c r="D14" s="30"/>
     </row>
     <row r="15" ht="28.199999999999999" customHeight="1">
-      <c r="A15" s="39"/>
-      <c r="B15" s="31"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="32"/>
+      <c r="A15" s="37"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
     </row>
     <row r="16" ht="27" customHeight="1">
-      <c r="A16" s="39"/>
-      <c r="B16" s="31"/>
-      <c r="C16" s="32"/>
-      <c r="D16" s="32"/>
+      <c r="A16" s="37"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
     </row>
     <row r="17" ht="27" customHeight="1">
-      <c r="A17" s="39"/>
-      <c r="B17" s="31"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="32"/>
+      <c r="A17" s="37"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
     </row>
     <row r="18" ht="27" customHeight="1">
-      <c r="A18" s="39"/>
-      <c r="B18" s="31"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
     </row>
     <row r="19" ht="17.399999999999999" customHeight="1">
-      <c r="A19" s="40"/>
-      <c r="B19" s="34"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
+      <c r="A19" s="38"/>
+      <c r="B19" s="32"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
     </row>
     <row r="20" ht="27" customHeight="1">
-      <c r="A20" s="41" t="s">
+      <c r="A20" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="31" t="s">
+      <c r="B20" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="C20" s="32" t="s">
+      <c r="C20" s="30" t="s">
         <v>64</v>
       </c>
-      <c r="D20" s="32" t="s">
+      <c r="D20" s="30" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="21" ht="27" customHeight="1">
-      <c r="A21" s="41"/>
-      <c r="B21" s="31" t="s">
+      <c r="A21" s="39"/>
+      <c r="B21" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="C21" s="32" t="s">
+      <c r="C21" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="30" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="22" ht="33.75" customHeight="1">
-      <c r="A22" s="41"/>
-      <c r="B22" s="32" t="s">
+      <c r="A22" s="39"/>
+      <c r="B22" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="C22" s="32" t="s">
+      <c r="C22" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="D22" s="32"/>
+      <c r="D22" s="30"/>
     </row>
     <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="41"/>
-      <c r="B23" s="31" t="s">
+      <c r="A23" s="39"/>
+      <c r="B23" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="C23" s="32" t="s">
+      <c r="C23" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="D23" s="32"/>
+      <c r="D23" s="30"/>
     </row>
     <row r="24" ht="27" customHeight="1">
-      <c r="A24" s="41"/>
-      <c r="B24" s="31" t="s">
+      <c r="A24" s="39"/>
+      <c r="B24" s="29" t="s">
         <v>73</v>
       </c>
-      <c r="C24" s="32" t="s">
+      <c r="C24" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="D24" s="32"/>
+      <c r="D24" s="30"/>
     </row>
     <row r="25" ht="27" customHeight="1">
-      <c r="A25" s="41"/>
-      <c r="B25" s="31" t="s">
+      <c r="A25" s="39"/>
+      <c r="B25" s="29" t="s">
         <v>75</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="C25" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="D25" s="32"/>
+      <c r="D25" s="30"/>
     </row>
     <row r="26" ht="27" customHeight="1">
-      <c r="A26" s="41"/>
-      <c r="B26" s="31"/>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
+      <c r="A26" s="39"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="30"/>
+      <c r="D26" s="30"/>
     </row>
     <row r="27" ht="27" customHeight="1">
-      <c r="A27" s="41"/>
-      <c r="B27" s="31"/>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
+      <c r="A27" s="39"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="30"/>
+      <c r="D27" s="30"/>
     </row>
     <row r="28" ht="27" customHeight="1">
-      <c r="A28" s="41"/>
-      <c r="B28" s="31"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
+      <c r="A28" s="39"/>
+      <c r="B28" s="29"/>
+      <c r="C28" s="30"/>
+      <c r="D28" s="30"/>
     </row>
     <row r="29" ht="17.399999999999999" customHeight="1">
       <c r="A29" s="5"/>
-      <c r="B29" s="34"/>
-      <c r="C29" s="35"/>
-      <c r="D29" s="35"/>
+      <c r="B29" s="32"/>
+      <c r="C29" s="33"/>
+      <c r="D29" s="33"/>
     </row>
     <row r="30" ht="27.75" customHeight="1">
-      <c r="A30" s="42" t="s">
+      <c r="A30" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="B30" s="31" t="s">
+      <c r="B30" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="C30" s="32" t="s">
+      <c r="C30" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="D30" s="32" t="s">
+      <c r="D30" s="30" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="31" ht="27.75" customHeight="1">
-      <c r="A31" s="42"/>
-      <c r="B31" s="31" t="s">
+      <c r="A31" s="40"/>
+      <c r="B31" s="29" t="s">
         <v>81</v>
       </c>
-      <c r="C31" s="32" t="s">
+      <c r="C31" s="30" t="s">
         <v>82</v>
       </c>
-      <c r="D31" s="32" t="s">
+      <c r="D31" s="30" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="32" ht="28.5">
-      <c r="A32" s="42"/>
-      <c r="B32" s="31" t="s">
+      <c r="A32" s="40"/>
+      <c r="B32" s="29" t="s">
         <v>84</v>
       </c>
-      <c r="C32" s="32" t="s">
+      <c r="C32" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="D32" s="32"/>
+      <c r="D32" s="30"/>
     </row>
     <row r="33" ht="28.5">
-      <c r="A33" s="42"/>
-      <c r="B33" s="31" t="s">
+      <c r="A33" s="40"/>
+      <c r="B33" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="C33" s="32" t="s">
+      <c r="C33" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="D33" s="32"/>
+      <c r="D33" s="30"/>
     </row>
     <row r="34" ht="27.75" customHeight="1">
-      <c r="A34" s="42"/>
-      <c r="B34" s="31" t="s">
+      <c r="A34" s="40"/>
+      <c r="B34" s="29" t="s">
         <v>88</v>
       </c>
-      <c r="C34" s="32" t="s">
+      <c r="C34" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="D34" s="32" t="s">
+      <c r="D34" s="30" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="35" ht="31.199999999999999" customHeight="1">
-      <c r="A35" s="42"/>
-      <c r="B35" s="31" t="s">
+      <c r="A35" s="40"/>
+      <c r="B35" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="C35" s="32" t="s">
+      <c r="C35" s="30" t="s">
         <v>92</v>
       </c>
-      <c r="D35" s="32"/>
+      <c r="D35" s="30"/>
     </row>
     <row r="36" ht="28.800000000000001" customHeight="1">
-      <c r="A36" s="42"/>
-      <c r="B36" s="31" t="s">
+      <c r="A36" s="40"/>
+      <c r="B36" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="C36" s="32" t="s">
+      <c r="C36" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="D36" s="32" t="s">
+      <c r="D36" s="30" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="37" ht="29.399999999999999" customHeight="1">
-      <c r="A37" s="42"/>
-      <c r="B37" s="31" t="s">
+      <c r="A37" s="40"/>
+      <c r="B37" s="29" t="s">
         <v>96</v>
       </c>
-      <c r="C37" s="32" t="s">
+      <c r="C37" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="D37" s="32" t="s">
+      <c r="D37" s="30" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="38" ht="42.75">
-      <c r="A38" s="42"/>
-      <c r="B38" s="31" t="s">
+      <c r="A38" s="40"/>
+      <c r="B38" s="29" t="s">
         <v>99</v>
       </c>
-      <c r="C38" s="32" t="s">
+      <c r="C38" s="30" t="s">
         <v>100</v>
       </c>
-      <c r="D38" s="32" t="s">
+      <c r="D38" s="30" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="39" ht="28.800000000000001" customHeight="1">
-      <c r="A39" s="42"/>
-      <c r="B39" s="32"/>
-      <c r="C39" s="32"/>
-      <c r="D39" s="32"/>
+      <c r="A39" s="40"/>
+      <c r="B39" s="30"/>
+      <c r="C39" s="30"/>
+      <c r="D39" s="30"/>
     </row>
     <row r="40" ht="28.800000000000001" customHeight="1">
-      <c r="A40" s="42"/>
-      <c r="B40" s="31"/>
-      <c r="C40" s="32"/>
-      <c r="D40" s="32"/>
+      <c r="A40" s="40"/>
+      <c r="B40" s="29"/>
+      <c r="C40" s="30"/>
+      <c r="D40" s="30"/>
     </row>
     <row r="41" ht="28.5" customHeight="1">
-      <c r="A41" s="42"/>
-      <c r="B41" s="31"/>
-      <c r="C41" s="32"/>
-      <c r="D41" s="32"/>
+      <c r="A41" s="40"/>
+      <c r="B41" s="29"/>
+      <c r="C41" s="30"/>
+      <c r="D41" s="30"/>
     </row>
     <row r="42" ht="28.5" customHeight="1">
-      <c r="A42" s="42"/>
-      <c r="B42" s="31"/>
-      <c r="C42" s="32"/>
-      <c r="D42" s="32"/>
+      <c r="A42" s="40"/>
+      <c r="B42" s="29"/>
+      <c r="C42" s="30"/>
+      <c r="D42" s="30"/>
     </row>
     <row r="43" ht="28.5" customHeight="1">
-      <c r="A43" s="42"/>
-      <c r="B43" s="31"/>
-      <c r="C43" s="32"/>
-      <c r="D43" s="32"/>
+      <c r="A43" s="40"/>
+      <c r="B43" s="29"/>
+      <c r="C43" s="30"/>
+      <c r="D43" s="30"/>
     </row>
     <row r="44" ht="28.5" customHeight="1">
-      <c r="A44" s="42"/>
-      <c r="B44" s="31"/>
-      <c r="C44" s="32"/>
-      <c r="D44" s="32"/>
+      <c r="A44" s="40"/>
+      <c r="B44" s="29"/>
+      <c r="C44" s="30"/>
+      <c r="D44" s="30"/>
     </row>
     <row r="45" ht="28.5" customHeight="1">
-      <c r="A45" s="42"/>
-      <c r="B45" s="31"/>
-      <c r="C45" s="32"/>
-      <c r="D45" s="32"/>
+      <c r="A45" s="40"/>
+      <c r="B45" s="29"/>
+      <c r="C45" s="30"/>
+      <c r="D45" s="30"/>
     </row>
     <row r="46" ht="28.5" customHeight="1">
-      <c r="B46" s="26"/>
-      <c r="C46" s="27"/>
-      <c r="D46" s="27"/>
+      <c r="B46" s="24"/>
+      <c r="C46" s="25"/>
+      <c r="D46" s="25"/>
     </row>
     <row r="47" ht="28.5" customHeight="1">
-      <c r="B47" s="26"/>
-      <c r="C47" s="27"/>
-      <c r="D47" s="27"/>
+      <c r="B47" s="24"/>
+      <c r="C47" s="25"/>
+      <c r="D47" s="25"/>
     </row>
     <row r="48" ht="28.5" customHeight="1"/>
     <row r="49" ht="28.5" customHeight="1"/>
@@ -2197,7 +2196,7 @@
       <c r="A3" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="41" t="s">
         <v>110</v>
       </c>
       <c r="C3" t="s">
@@ -2214,7 +2213,7 @@
       <c r="B4" t="s">
         <v>112</v>
       </c>
-      <c r="C4" s="44" t="s">
+      <c r="C4" s="42" t="s">
         <v>107</v>
       </c>
       <c r="D4" t="s">
@@ -2228,7 +2227,7 @@
       <c r="B5" t="s">
         <v>115</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="42" t="s">
         <v>107</v>
       </c>
       <c r="D5" t="s">
@@ -2236,13 +2235,13 @@
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="41" t="s">
         <v>117</v>
       </c>
       <c r="B6" t="s">
         <v>118</v>
       </c>
-      <c r="C6" s="44" t="s">
+      <c r="C6" s="42" t="s">
         <v>107</v>
       </c>
       <c r="D6" t="s">
@@ -2250,13 +2249,13 @@
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="41" t="s">
         <v>120</v>
       </c>
       <c r="B7" t="s">
         <v>121</v>
       </c>
-      <c r="C7" s="44" t="s">
+      <c r="C7" s="42" t="s">
         <v>107</v>
       </c>
       <c r="D7" t="s">
@@ -3269,163 +3268,163 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.57421875"/>
-    <col customWidth="1" min="2" max="2" style="45" width="38.421875"/>
+    <col customWidth="1" min="2" max="2" style="43" width="38.421875"/>
     <col customWidth="1" min="3" max="3" width="55.421875"/>
     <col customWidth="1" min="4" max="4" width="75.8515625"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="C1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="D1" s="27" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" s="45" customFormat="1" ht="42.75">
-      <c r="A2" s="46"/>
-      <c r="B2" s="47" t="s">
+    <row r="2" s="43" customFormat="1" ht="42.75">
+      <c r="A2" s="44"/>
+      <c r="B2" s="45" t="s">
         <v>123</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="C2" s="46" t="s">
         <v>124</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="D2" s="47" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="3" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A3" s="46"/>
-      <c r="B3" s="47" t="s">
+    <row r="3" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A3" s="44"/>
+      <c r="B3" s="45" t="s">
         <v>126</v>
       </c>
-      <c r="C3" s="48" t="s">
+      <c r="C3" s="47" t="s">
         <v>127</v>
       </c>
-      <c r="D3" s="48"/>
-    </row>
-    <row r="4" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A4" s="46"/>
-      <c r="B4" s="47"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-    </row>
-    <row r="5" s="45" customFormat="1" ht="57">
-      <c r="A5" s="46"/>
-      <c r="B5" s="48" t="s">
+      <c r="D3" s="47"/>
+    </row>
+    <row r="4" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A4" s="44"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+    </row>
+    <row r="5" s="43" customFormat="1" ht="57">
+      <c r="A5" s="44"/>
+      <c r="B5" s="47" t="s">
         <v>128</v>
       </c>
-      <c r="C5" s="48" t="s">
+      <c r="C5" s="47" t="s">
         <v>129</v>
       </c>
-      <c r="D5" s="49" t="s">
+      <c r="D5" s="48" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="6" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A6" s="46"/>
-      <c r="B6" s="47" t="s">
+    <row r="6" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A6" s="44"/>
+      <c r="B6" s="45" t="s">
         <v>131</v>
       </c>
-      <c r="C6" s="50" t="s">
+      <c r="C6" s="49" t="s">
         <v>132</v>
       </c>
-      <c r="D6" s="48" t="s">
+      <c r="D6" s="47" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="7" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A7" s="46"/>
-      <c r="B7" s="47"/>
-      <c r="C7" s="48"/>
-      <c r="D7" s="48"/>
+    <row r="7" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A7" s="44"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" s="5"/>
-      <c r="B8" s="51"/>
+      <c r="B8" s="50"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
     </row>
     <row r="9" ht="41.25" customHeight="1">
-      <c r="A9" s="52" t="s">
+      <c r="A9" s="51" t="s">
         <v>134</v>
       </c>
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="29" t="s">
         <v>135</v>
       </c>
-      <c r="C9" s="53" t="s">
+      <c r="C9" s="52" t="s">
         <v>136</v>
       </c>
-      <c r="D9" s="32" t="s">
+      <c r="D9" s="30" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="54"/>
-      <c r="B10" s="31" t="s">
+      <c r="A10" s="53"/>
+      <c r="B10" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="C10" s="32">
+      <c r="C10" s="30">
         <v>60000</v>
       </c>
-      <c r="D10" s="32" t="s">
+      <c r="D10" s="30" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="11" ht="36.75" customHeight="1">
-      <c r="A11" s="54"/>
-      <c r="B11" s="31" t="s">
+      <c r="A11" s="53"/>
+      <c r="B11" s="29" t="s">
         <v>140</v>
       </c>
-      <c r="C11" s="32">
+      <c r="C11" s="30">
         <v>3000</v>
       </c>
-      <c r="D11" s="32" t="s">
+      <c r="D11" s="30" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="54"/>
-      <c r="B12" s="31" t="s">
+      <c r="A12" s="53"/>
+      <c r="B12" s="29" t="s">
         <v>142</v>
       </c>
-      <c r="C12" s="32" t="s">
+      <c r="C12" s="30" t="s">
         <v>143</v>
       </c>
-      <c r="D12" s="32" t="s">
+      <c r="D12" s="30" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="54"/>
-      <c r="B13" s="31" t="s">
+      <c r="A13" s="53"/>
+      <c r="B13" s="29" t="s">
         <v>145</v>
       </c>
-      <c r="C13" s="55" t="s">
+      <c r="C13" s="54" t="s">
         <v>146</v>
       </c>
-      <c r="D13" s="32" t="s">
+      <c r="D13" s="30" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="14" ht="63.600000000000001" customHeight="1">
-      <c r="A14" s="54"/>
-      <c r="B14" s="31" t="s">
+      <c r="A14" s="53"/>
+      <c r="B14" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="C14" s="55" t="s">
+      <c r="C14" s="54" t="s">
         <v>149</v>
       </c>
-      <c r="D14" s="32" t="s">
+      <c r="D14" s="30" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" s="5"/>
-      <c r="B15" s="51"/>
+      <c r="B15" s="50"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>

</xml_diff>

<commit_message>
Adicionando tratamento das criticas de estruturação dos arquivos de importação do UIPath
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="153">
   <si>
     <t>Name</t>
   </si>
@@ -414,6 +414,12 @@
   </si>
   <si>
     <t xml:space="preserve">Caso haja um erro durante o processo de definição de datas do request das despesas. </t>
+  </si>
+  <si>
+    <t>ExceptionMessage_CriticasDeEstruturasAosTxtsDeImportacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foram exibidas criticas de estruturas aos txts de importação no processo de importação. Favor verificar</t>
   </si>
   <si>
     <t>Asset</t>
@@ -706,7 +712,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -810,6 +816,12 @@
     <xf fontId="5" fillId="11" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -822,9 +834,6 @@
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2042,7 +2051,7 @@
     </row>
     <row r="38" ht="42.75">
       <c r="A38" s="40"/>
-      <c r="B38" s="29" t="s">
+      <c r="B38" s="41" t="s">
         <v>99</v>
       </c>
       <c r="C38" s="30" t="s">
@@ -2054,8 +2063,12 @@
     </row>
     <row r="39" ht="28.800000000000001" customHeight="1">
       <c r="A39" s="40"/>
-      <c r="B39" s="30"/>
-      <c r="C39" s="30"/>
+      <c r="B39" s="42" t="s">
+        <v>102</v>
+      </c>
+      <c r="C39" s="42" t="s">
+        <v>103</v>
+      </c>
       <c r="D39" s="30"/>
     </row>
     <row r="40" ht="28.800000000000001" customHeight="1">
@@ -2147,13 +2160,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -2180,86 +2193,86 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>112</v>
+      </c>
+      <c r="C3" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="41" t="s">
-        <v>110</v>
-      </c>
-      <c r="C3" t="s">
-        <v>107</v>
-      </c>
       <c r="D3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B4" t="s">
-        <v>112</v>
-      </c>
-      <c r="C4" s="42" t="s">
-        <v>107</v>
+        <v>114</v>
+      </c>
+      <c r="C4" s="44" t="s">
+        <v>109</v>
       </c>
       <c r="D4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B5" t="s">
-        <v>115</v>
-      </c>
-      <c r="C5" s="42" t="s">
-        <v>107</v>
+        <v>117</v>
+      </c>
+      <c r="C5" s="44" t="s">
+        <v>109</v>
       </c>
       <c r="D5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="41" t="s">
-        <v>117</v>
+      <c r="A6" s="43" t="s">
+        <v>119</v>
       </c>
       <c r="B6" t="s">
-        <v>118</v>
-      </c>
-      <c r="C6" s="42" t="s">
-        <v>107</v>
+        <v>120</v>
+      </c>
+      <c r="C6" s="44" t="s">
+        <v>109</v>
       </c>
       <c r="D6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="41" t="s">
-        <v>120</v>
+      <c r="A7" s="43" t="s">
+        <v>122</v>
       </c>
       <c r="B7" t="s">
-        <v>121</v>
-      </c>
-      <c r="C7" s="42" t="s">
-        <v>107</v>
+        <v>123</v>
+      </c>
+      <c r="C7" s="44" t="s">
+        <v>109</v>
       </c>
       <c r="D7" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1"/>
@@ -3268,7 +3281,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.57421875"/>
-    <col customWidth="1" min="2" max="2" style="43" width="38.421875"/>
+    <col customWidth="1" min="2" max="2" style="45" width="38.421875"/>
     <col customWidth="1" min="3" max="3" width="55.421875"/>
     <col customWidth="1" min="4" max="4" width="75.8515625"/>
   </cols>
@@ -3284,147 +3297,147 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" s="43" customFormat="1" ht="42.75">
-      <c r="A2" s="44"/>
-      <c r="B2" s="45" t="s">
-        <v>123</v>
-      </c>
-      <c r="C2" s="46" t="s">
-        <v>124</v>
-      </c>
-      <c r="D2" s="47" t="s">
+    <row r="2" s="45" customFormat="1" ht="28.5">
+      <c r="A2" s="46"/>
+      <c r="B2" s="47" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="3" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A3" s="44"/>
-      <c r="B3" s="45" t="s">
+      <c r="C2" s="48" t="s">
         <v>126</v>
       </c>
-      <c r="C3" s="47" t="s">
+      <c r="D2" s="48" t="s">
         <v>127</v>
       </c>
-      <c r="D3" s="47"/>
-    </row>
-    <row r="4" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A4" s="44"/>
-      <c r="B4" s="45"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
-    </row>
-    <row r="5" s="43" customFormat="1" ht="57">
-      <c r="A5" s="44"/>
-      <c r="B5" s="47" t="s">
+    </row>
+    <row r="3" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A3" s="46"/>
+      <c r="B3" s="47" t="s">
         <v>128</v>
       </c>
-      <c r="C5" s="47" t="s">
+      <c r="C3" s="48" t="s">
         <v>129</v>
       </c>
-      <c r="D5" s="48" t="s">
+      <c r="D3" s="48"/>
+    </row>
+    <row r="4" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A4" s="46"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+    </row>
+    <row r="5" s="45" customFormat="1" ht="57">
+      <c r="A5" s="46"/>
+      <c r="B5" s="48" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="6" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A6" s="44"/>
-      <c r="B6" s="45" t="s">
+      <c r="C5" s="48" t="s">
         <v>131</v>
       </c>
-      <c r="C6" s="49" t="s">
+      <c r="D5" s="49" t="s">
         <v>132</v>
       </c>
-      <c r="D6" s="47" t="s">
+    </row>
+    <row r="6" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A6" s="46"/>
+      <c r="B6" s="47" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="7" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A7" s="44"/>
-      <c r="B7" s="45"/>
-      <c r="C7" s="47"/>
-      <c r="D7" s="47"/>
+      <c r="C6" s="50" t="s">
+        <v>134</v>
+      </c>
+      <c r="D6" s="48" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="7" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A7" s="46"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" s="5"/>
-      <c r="B8" s="50"/>
+      <c r="B8" s="51"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
     </row>
     <row r="9" ht="41.25" customHeight="1">
-      <c r="A9" s="51" t="s">
-        <v>134</v>
+      <c r="A9" s="52" t="s">
+        <v>136</v>
       </c>
       <c r="B9" s="29" t="s">
-        <v>135</v>
-      </c>
-      <c r="C9" s="52" t="s">
-        <v>136</v>
+        <v>137</v>
+      </c>
+      <c r="C9" s="53" t="s">
+        <v>138</v>
       </c>
       <c r="D9" s="30" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="53"/>
+      <c r="A10" s="54"/>
       <c r="B10" s="29" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C10" s="30">
         <v>60000</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" ht="36.75" customHeight="1">
-      <c r="A11" s="53"/>
+      <c r="A11" s="54"/>
       <c r="B11" s="29" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C11" s="30">
         <v>3000</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="53"/>
+      <c r="A12" s="54"/>
       <c r="B12" s="29" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D12" s="30" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="53"/>
+      <c r="A13" s="54"/>
       <c r="B13" s="29" t="s">
-        <v>145</v>
-      </c>
-      <c r="C13" s="54" t="s">
-        <v>146</v>
+        <v>147</v>
+      </c>
+      <c r="C13" s="55" t="s">
+        <v>148</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14" ht="63.600000000000001" customHeight="1">
-      <c r="A14" s="53"/>
+      <c r="A14" s="54"/>
       <c r="B14" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="C14" s="54" t="s">
-        <v>149</v>
+        <v>150</v>
+      </c>
+      <c r="C14" s="55" t="s">
+        <v>151</v>
       </c>
       <c r="D14" s="30" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" s="5"/>
-      <c r="B15" s="50"/>
+      <c r="B15" s="51"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>

</xml_diff>

<commit_message>
Teste de tratamento das criticas de construção ao documento de importação
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="154">
   <si>
     <t>Name</t>
   </si>
@@ -110,7 +110,7 @@
     <t>obligationDateStart</t>
   </si>
   <si>
-    <t>01/03/2026</t>
+    <t>20/01/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Data inicial do range de datas que deve abranger a data de vencimento da obrigação em questão, se não estiver definida nenhuma data nessa variável, o processo define o primeiro e o ultimo dia do mês como as datas de inicio e fim do range.</t>
@@ -119,7 +119,7 @@
     <t>obligationDateEnd</t>
   </si>
   <si>
-    <t>05/03/2026</t>
+    <t>05/02/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Data final do range de datas que deve abranger a data de vencimento da obrigação em questão, se não estiver definida nenhuma data nessa variável, o processo define o primeiro e o ultimo dia do mês como as datas de inicio e fim do range.</t>
@@ -485,6 +485,9 @@
     <t xml:space="preserve">Provider name para conexão no banco de dados do Domínio</t>
   </si>
   <si>
+    <t>s</t>
+  </si>
+  <si>
     <t>mainPath</t>
   </si>
   <si>
@@ -554,7 +557,7 @@
     <t>getExpenses_dateStart</t>
   </si>
   <si>
-    <t>01/05/2025</t>
+    <t>01/01/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Inicio do range de datas que abrange a data de vencimento das despesas que irão ser importadas. Deve estar no formato "dd/MM/yyyy" e só deve existir caso o getExpenses_dateEnd existir também.</t>
@@ -563,7 +566,7 @@
     <t>getExpenses_dateEnd</t>
   </si>
   <si>
-    <t>31/12/2025</t>
+    <t>01/02/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Fim do range de datas que abrange a data de vencimento das despesas que irão ser importadas. Deve estar no formato "dd/MM/yyyy" e só deve existir caso o getExpenses_dateStart existir também. Deve ser posterior ao getExpenses_dateStart</t>
@@ -712,7 +715,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="54">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -815,12 +818,6 @@
     </xf>
     <xf fontId="5" fillId="11" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
@@ -2051,7 +2048,7 @@
     </row>
     <row r="38" ht="42.75">
       <c r="A38" s="40"/>
-      <c r="B38" s="41" t="s">
+      <c r="B38" s="29" t="s">
         <v>99</v>
       </c>
       <c r="C38" s="30" t="s">
@@ -2063,10 +2060,10 @@
     </row>
     <row r="39" ht="28.800000000000001" customHeight="1">
       <c r="A39" s="40"/>
-      <c r="B39" s="42" t="s">
+      <c r="B39" s="30" t="s">
         <v>102</v>
       </c>
-      <c r="C39" s="42" t="s">
+      <c r="C39" s="30" t="s">
         <v>103</v>
       </c>
       <c r="D39" s="30"/>
@@ -2209,7 +2206,7 @@
       <c r="A3" t="s">
         <v>111</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="41" t="s">
         <v>112</v>
       </c>
       <c r="C3" t="s">
@@ -2226,7 +2223,7 @@
       <c r="B4" t="s">
         <v>114</v>
       </c>
-      <c r="C4" s="44" t="s">
+      <c r="C4" s="42" t="s">
         <v>109</v>
       </c>
       <c r="D4" t="s">
@@ -2240,7 +2237,7 @@
       <c r="B5" t="s">
         <v>117</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="42" t="s">
         <v>109</v>
       </c>
       <c r="D5" t="s">
@@ -2248,13 +2245,13 @@
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="41" t="s">
         <v>119</v>
       </c>
       <c r="B6" t="s">
         <v>120</v>
       </c>
-      <c r="C6" s="44" t="s">
+      <c r="C6" s="42" t="s">
         <v>109</v>
       </c>
       <c r="D6" t="s">
@@ -2262,13 +2259,13 @@
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="41" t="s">
         <v>122</v>
       </c>
       <c r="B7" t="s">
         <v>123</v>
       </c>
-      <c r="C7" s="44" t="s">
+      <c r="C7" s="42" t="s">
         <v>109</v>
       </c>
       <c r="D7" t="s">
@@ -3281,12 +3278,15 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.57421875"/>
-    <col customWidth="1" min="2" max="2" style="45" width="38.421875"/>
+    <col customWidth="1" min="2" max="2" style="43" width="38.421875"/>
     <col customWidth="1" min="3" max="3" width="55.421875"/>
     <col customWidth="1" min="4" max="4" width="75.8515625"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
+      <c r="A1" t="s">
+        <v>125</v>
+      </c>
       <c r="B1" s="26" t="s">
         <v>0</v>
       </c>
@@ -3297,147 +3297,147 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" s="45" customFormat="1" ht="28.5">
-      <c r="A2" s="46"/>
-      <c r="B2" s="47" t="s">
-        <v>125</v>
-      </c>
-      <c r="C2" s="48" t="s">
+    <row r="2" s="43" customFormat="1" ht="28.5">
+      <c r="A2" s="44"/>
+      <c r="B2" s="45" t="s">
         <v>126</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="C2" s="46" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="3" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A3" s="46"/>
-      <c r="B3" s="47" t="s">
+      <c r="D2" s="46" t="s">
         <v>128</v>
       </c>
-      <c r="C3" s="48" t="s">
+    </row>
+    <row r="3" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A3" s="44"/>
+      <c r="B3" s="45" t="s">
         <v>129</v>
       </c>
-      <c r="D3" s="48"/>
-    </row>
-    <row r="4" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A4" s="46"/>
-      <c r="B4" s="47"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-    </row>
-    <row r="5" s="45" customFormat="1" ht="57">
-      <c r="A5" s="46"/>
-      <c r="B5" s="48" t="s">
+      <c r="C3" s="46" t="s">
         <v>130</v>
       </c>
-      <c r="C5" s="48" t="s">
+      <c r="D3" s="46"/>
+    </row>
+    <row r="4" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A4" s="44"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+    </row>
+    <row r="5" s="43" customFormat="1" ht="57">
+      <c r="A5" s="44"/>
+      <c r="B5" s="46" t="s">
         <v>131</v>
       </c>
-      <c r="D5" s="49" t="s">
+      <c r="C5" s="46" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="6" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A6" s="46"/>
-      <c r="B6" s="47" t="s">
+      <c r="D5" s="47" t="s">
         <v>133</v>
       </c>
-      <c r="C6" s="50" t="s">
+    </row>
+    <row r="6" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A6" s="44"/>
+      <c r="B6" s="45" t="s">
         <v>134</v>
       </c>
-      <c r="D6" s="48" t="s">
+      <c r="C6" s="48" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="7" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A7" s="46"/>
-      <c r="B7" s="47"/>
-      <c r="C7" s="48"/>
-      <c r="D7" s="48"/>
+      <c r="D6" s="46" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="7" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A7" s="44"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="46"/>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" s="5"/>
-      <c r="B8" s="51"/>
+      <c r="B8" s="49"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
     </row>
     <row r="9" ht="41.25" customHeight="1">
-      <c r="A9" s="52" t="s">
-        <v>136</v>
+      <c r="A9" s="50" t="s">
+        <v>137</v>
       </c>
       <c r="B9" s="29" t="s">
-        <v>137</v>
-      </c>
-      <c r="C9" s="53" t="s">
         <v>138</v>
       </c>
+      <c r="C9" s="51" t="s">
+        <v>139</v>
+      </c>
       <c r="D9" s="30" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="54"/>
+      <c r="A10" s="52"/>
       <c r="B10" s="29" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C10" s="30">
         <v>60000</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11" ht="36.75" customHeight="1">
-      <c r="A11" s="54"/>
+      <c r="A11" s="52"/>
       <c r="B11" s="29" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C11" s="30">
         <v>3000</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="54"/>
+      <c r="A12" s="52"/>
       <c r="B12" s="29" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D12" s="30" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="54"/>
+      <c r="A13" s="52"/>
       <c r="B13" s="29" t="s">
-        <v>147</v>
-      </c>
-      <c r="C13" s="55" t="s">
         <v>148</v>
       </c>
+      <c r="C13" s="53" t="s">
+        <v>149</v>
+      </c>
       <c r="D13" s="30" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14" ht="63.600000000000001" customHeight="1">
-      <c r="A14" s="54"/>
+      <c r="A14" s="52"/>
       <c r="B14" s="29" t="s">
-        <v>150</v>
-      </c>
-      <c r="C14" s="55" t="s">
         <v>151</v>
       </c>
+      <c r="C14" s="53" t="s">
+        <v>152</v>
+      </c>
       <c r="D14" s="30" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" s="5"/>
-      <c r="B15" s="51"/>
+      <c r="B15" s="49"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>

</xml_diff>

<commit_message>
Inicio da implementação da integração da integração das despesas importadas.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -715,7 +715,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -846,6 +846,9 @@
     </xf>
     <xf fontId="2" fillId="7" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf fontId="4" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3365,10 +3368,10 @@
       <c r="A9" s="50" t="s">
         <v>137</v>
       </c>
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="51" t="s">
         <v>138</v>
       </c>
-      <c r="C9" s="51" t="s">
+      <c r="C9" s="52" t="s">
         <v>139</v>
       </c>
       <c r="D9" s="30" t="s">
@@ -3376,7 +3379,7 @@
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="52"/>
+      <c r="A10" s="53"/>
       <c r="B10" s="29" t="s">
         <v>141</v>
       </c>
@@ -3388,7 +3391,7 @@
       </c>
     </row>
     <row r="11" ht="36.75" customHeight="1">
-      <c r="A11" s="52"/>
+      <c r="A11" s="53"/>
       <c r="B11" s="29" t="s">
         <v>143</v>
       </c>
@@ -3400,7 +3403,7 @@
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="52"/>
+      <c r="A12" s="53"/>
       <c r="B12" s="29" t="s">
         <v>145</v>
       </c>
@@ -3412,11 +3415,11 @@
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="52"/>
+      <c r="A13" s="53"/>
       <c r="B13" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="C13" s="53" t="s">
+      <c r="C13" s="54" t="s">
         <v>149</v>
       </c>
       <c r="D13" s="30" t="s">
@@ -3424,11 +3427,11 @@
       </c>
     </row>
     <row r="14" ht="63.600000000000001" customHeight="1">
-      <c r="A14" s="52"/>
+      <c r="A14" s="53"/>
       <c r="B14" s="29" t="s">
         <v>151</v>
       </c>
-      <c r="C14" s="53" t="s">
+      <c r="C14" s="54" t="s">
         <v>152</v>
       </c>
       <c r="D14" s="30" t="s">

</xml_diff>

<commit_message>
Alteração da pasta do VerificacaoDaImportacao e desenvolvimento da funcionalidade de integração das despesas
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="162">
   <si>
     <t>Name</t>
   </si>
@@ -566,10 +566,34 @@
     <t>getExpenses_dateEnd</t>
   </si>
   <si>
-    <t>01/02/2026</t>
+    <t>01/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Fim do range de datas que abrange a data de vencimento das despesas que irão ser importadas. Deve estar no formato "dd/MM/yyyy" e só deve existir caso o getExpenses_dateStart existir também. Deve ser posterior ao getExpenses_dateStart</t>
+  </si>
+  <si>
+    <t>PostExpensesSettings</t>
+  </si>
+  <si>
+    <t>postExpenses_endPoint</t>
+  </si>
+  <si>
+    <t>set_as_integrated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">endpoint para request post para integrar as obrigações, o formato final do endpoint fica "expensesUrl + /:id/set_as_integrated</t>
+  </si>
+  <si>
+    <t>postExpenses_timeout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Timeout do request</t>
+  </si>
+  <si>
+    <t>postExpenses_contentType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Content-type do post expenses</t>
   </si>
 </sst>
 </file>
@@ -611,7 +635,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -678,6 +702,12 @@
         <bgColor indexed="2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor theme="0" tint="-0.14999847407452621"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -715,7 +745,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="58">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -847,9 +877,6 @@
     <xf fontId="2" fillId="7" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf fontId="4" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -858,6 +885,18 @@
     </xf>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="12" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="12" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="12" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3368,10 +3407,10 @@
       <c r="A9" s="50" t="s">
         <v>137</v>
       </c>
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="C9" s="52" t="s">
+      <c r="C9" s="51" t="s">
         <v>139</v>
       </c>
       <c r="D9" s="30" t="s">
@@ -3379,7 +3418,7 @@
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="53"/>
+      <c r="A10" s="52"/>
       <c r="B10" s="29" t="s">
         <v>141</v>
       </c>
@@ -3391,7 +3430,7 @@
       </c>
     </row>
     <row r="11" ht="36.75" customHeight="1">
-      <c r="A11" s="53"/>
+      <c r="A11" s="52"/>
       <c r="B11" s="29" t="s">
         <v>143</v>
       </c>
@@ -3403,7 +3442,7 @@
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="53"/>
+      <c r="A12" s="52"/>
       <c r="B12" s="29" t="s">
         <v>145</v>
       </c>
@@ -3415,11 +3454,11 @@
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="53"/>
+      <c r="A13" s="52"/>
       <c r="B13" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="C13" s="54" t="s">
+      <c r="C13" s="53" t="s">
         <v>149</v>
       </c>
       <c r="D13" s="30" t="s">
@@ -3427,11 +3466,11 @@
       </c>
     </row>
     <row r="14" ht="63.600000000000001" customHeight="1">
-      <c r="A14" s="53"/>
+      <c r="A14" s="52"/>
       <c r="B14" s="29" t="s">
         <v>151</v>
       </c>
-      <c r="C14" s="54" t="s">
+      <c r="C14" s="53" t="s">
         <v>152</v>
       </c>
       <c r="D14" s="30" t="s">
@@ -3444,9 +3483,44 @@
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>
-    <row r="16" ht="30.600000000000001" customHeight="1"/>
-    <row r="17" ht="28.199999999999999" customHeight="1"/>
-    <row r="18" ht="28.199999999999999" customHeight="1"/>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="54" t="s">
+        <v>154</v>
+      </c>
+      <c r="B16" s="55" t="s">
+        <v>155</v>
+      </c>
+      <c r="C16" s="56" t="s">
+        <v>156</v>
+      </c>
+      <c r="D16" s="57" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="54"/>
+      <c r="B17" s="55" t="s">
+        <v>158</v>
+      </c>
+      <c r="C17" s="56">
+        <v>5000</v>
+      </c>
+      <c r="D17" s="56" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="54"/>
+      <c r="B18" s="55" t="s">
+        <v>160</v>
+      </c>
+      <c r="C18" s="56" t="s">
+        <v>146</v>
+      </c>
+      <c r="D18" s="56" t="s">
+        <v>161</v>
+      </c>
+    </row>
     <row r="19" ht="28.199999999999999" customHeight="1"/>
     <row r="20" ht="28.199999999999999" customHeight="1"/>
     <row r="21" ht="28.199999999999999" customHeight="1"/>
@@ -3536,9 +3610,10 @@
     <row r="105" ht="28.199999999999999" customHeight="1"/>
     <row r="106" ht="28.199999999999999" customHeight="1"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:A7"/>
     <mergeCell ref="A9:A14"/>
+    <mergeCell ref="A16:A18"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C9"/>

</xml_diff>

<commit_message>
Adicionando funcionalidade de não importação das despesas especificadas no config.xlsx
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
   <si>
     <t>Name</t>
   </si>
@@ -512,6 +512,15 @@
     <t xml:space="preserve">O Domínio pode apresentar erro de acordo com a quantidade de despesas inseridas em um determinado arquivo de importação. Por isso, existem as contas de débito específicas que devem estar separadas por arquivo de importação.Deve estar no fomraco "contaDeDebito,contaDeDebito,contaDeDebito"</t>
   </si>
   <si>
+    <t>especificExceptDebitAccounts</t>
+  </si>
+  <si>
+    <t>2110,2074,1204,2103,2112,2055</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contas de débito que não devem ser importadas para o Domínio.</t>
+  </si>
+  <si>
     <t>dateEndWorkPeriod</t>
   </si>
   <si>
@@ -557,7 +566,7 @@
     <t>getExpenses_dateStart</t>
   </si>
   <si>
-    <t>01/01/2026</t>
+    <t>01/01/2025</t>
   </si>
   <si>
     <t xml:space="preserve">Inicio do range de datas que abrange a data de vencimento das despesas que irão ser importadas. Deve estar no formato "dd/MM/yyyy" e só deve existir caso o getExpenses_dateEnd existir também.</t>
@@ -865,7 +874,7 @@
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -3375,16 +3384,16 @@
       <c r="C5" s="46" t="s">
         <v>132</v>
       </c>
-      <c r="D5" s="47" t="s">
+      <c r="D5" s="46" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="6" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
+    <row r="6" s="43" customFormat="1" ht="36" customHeight="1">
       <c r="A6" s="44"/>
-      <c r="B6" s="45" t="s">
+      <c r="B6" s="47" t="s">
         <v>134</v>
       </c>
-      <c r="C6" s="48" t="s">
+      <c r="C6" s="46" t="s">
         <v>135</v>
       </c>
       <c r="D6" s="46" t="s">
@@ -3393,79 +3402,79 @@
     </row>
     <row r="7" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
       <c r="A7" s="44"/>
-      <c r="B7" s="45"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-    </row>
-    <row r="8" ht="14.25">
-      <c r="A8" s="5"/>
-      <c r="B8" s="49"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-    </row>
-    <row r="9" ht="41.25" customHeight="1">
-      <c r="A9" s="50" t="s">
+      <c r="B7" s="45" t="s">
         <v>137</v>
       </c>
-      <c r="B9" s="29" t="s">
+      <c r="C7" s="48" t="s">
         <v>138</v>
       </c>
-      <c r="C9" s="51" t="s">
+      <c r="D7" s="46" t="s">
         <v>139</v>
       </c>
-      <c r="D9" s="30" t="s">
+    </row>
+    <row r="8" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A8" s="44"/>
+      <c r="B8" s="45"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="46"/>
+    </row>
+    <row r="9" ht="14.25">
+      <c r="A9" s="5"/>
+      <c r="B9" s="49"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+    </row>
+    <row r="10" ht="41.25" customHeight="1">
+      <c r="A10" s="50" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="52"/>
       <c r="B10" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="C10" s="30">
-        <v>60000</v>
+      <c r="C10" s="51" t="s">
+        <v>142</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="11" ht="36.75" customHeight="1">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="11" ht="39.75" customHeight="1">
       <c r="A11" s="52"/>
       <c r="B11" s="29" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C11" s="30">
-        <v>3000</v>
+        <v>60000</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
       <c r="A12" s="52"/>
       <c r="B12" s="29" t="s">
-        <v>145</v>
-      </c>
-      <c r="C12" s="30" t="s">
         <v>146</v>
+      </c>
+      <c r="C12" s="30">
+        <v>3000</v>
       </c>
       <c r="D12" s="30" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1">
+    <row r="13" ht="36.75" customHeight="1">
       <c r="A13" s="52"/>
       <c r="B13" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="C13" s="53" t="s">
+      <c r="C13" s="30" t="s">
         <v>149</v>
       </c>
       <c r="D13" s="30" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="14" ht="63.600000000000001" customHeight="1">
+    <row r="14" ht="48" customHeight="1">
       <c r="A14" s="52"/>
       <c r="B14" s="29" t="s">
         <v>151</v>
@@ -3477,51 +3486,62 @@
         <v>153</v>
       </c>
     </row>
-    <row r="15" ht="14.25">
-      <c r="A15" s="5"/>
-      <c r="B15" s="49"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-    </row>
-    <row r="16" ht="42" customHeight="1">
-      <c r="A16" s="54" t="s">
+    <row r="15" ht="63.600000000000001" customHeight="1">
+      <c r="A15" s="52"/>
+      <c r="B15" s="29" t="s">
         <v>154</v>
       </c>
-      <c r="B16" s="55" t="s">
+      <c r="C15" s="53" t="s">
         <v>155</v>
       </c>
-      <c r="C16" s="56" t="s">
+      <c r="D15" s="30" t="s">
         <v>156</v>
       </c>
-      <c r="D16" s="57" t="s">
+    </row>
+    <row r="16" ht="14.25">
+      <c r="A16" s="5"/>
+      <c r="B16" s="49"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="54" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="54"/>
       <c r="B17" s="55" t="s">
         <v>158</v>
       </c>
-      <c r="C17" s="56">
-        <v>5000</v>
-      </c>
-      <c r="D17" s="56" t="s">
+      <c r="C17" s="56" t="s">
         <v>159</v>
+      </c>
+      <c r="D17" s="57" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="54"/>
       <c r="B18" s="55" t="s">
-        <v>160</v>
-      </c>
-      <c r="C18" s="56" t="s">
-        <v>146</v>
+        <v>161</v>
+      </c>
+      <c r="C18" s="56">
+        <v>5000</v>
       </c>
       <c r="D18" s="56" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="19" ht="28.199999999999999" customHeight="1"/>
+        <v>162</v>
+      </c>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="54"/>
+      <c r="B19" s="55" t="s">
+        <v>163</v>
+      </c>
+      <c r="C19" s="56" t="s">
+        <v>149</v>
+      </c>
+      <c r="D19" s="56" t="s">
+        <v>164</v>
+      </c>
+    </row>
     <row r="20" ht="28.199999999999999" customHeight="1"/>
     <row r="21" ht="28.199999999999999" customHeight="1"/>
     <row r="22" ht="28.199999999999999" customHeight="1"/>
@@ -3609,14 +3629,15 @@
     <row r="104" ht="28.199999999999999" customHeight="1"/>
     <row r="105" ht="28.199999999999999" customHeight="1"/>
     <row r="106" ht="28.199999999999999" customHeight="1"/>
+    <row r="107" ht="28.199999999999999" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:A7"/>
-    <mergeCell ref="A9:A14"/>
-    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="A2:A8"/>
+    <mergeCell ref="A10:A15"/>
+    <mergeCell ref="A17:A19"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="C9"/>
+    <hyperlink r:id="rId1" ref="C10"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Bug fix da criação dos arquivos de importação, para despesas com quebra de linha na nota. Edição do SetObligationStatus para integrar as obrigações devidas, e dinâmica do get transaction data para erro no request get companies alterado
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -89,6 +89,9 @@
     </r>
   </si>
   <si>
+    <t>enableExpensesIntegration</t>
+  </si>
+  <si>
     <t xml:space="preserve">OBLIGATION SETTINGS</t>
   </si>
   <si>
@@ -110,7 +113,7 @@
     <t>obligationDateStart</t>
   </si>
   <si>
-    <t>20/01/2026</t>
+    <t>20/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Data inicial do range de datas que deve abranger a data de vencimento da obrigação em questão, se não estiver definida nenhuma data nessa variável, o processo define o primeiro e o ultimo dia do mês como as datas de inicio e fim do range.</t>
@@ -119,7 +122,7 @@
     <t>obligationDateEnd</t>
   </si>
   <si>
-    <t>05/02/2026</t>
+    <t>05/04/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Data final do range de datas que deve abranger a data de vencimento da obrigação em questão, se não estiver definida nenhuma data nessa variável, o processo define o primeiro e o ultimo dia do mês como as datas de inicio e fim do range.</t>
@@ -164,9 +167,6 @@
     <t>obligationDebugCompanyId</t>
   </si>
   <si>
-    <t>7a8d0889-71e5-4dab-9ec2-734bf7c46734</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -566,7 +566,7 @@
     <t>getExpenses_dateStart</t>
   </si>
   <si>
-    <t>01/01/2025</t>
+    <t>01/01/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Inicio do range de datas que abrange a data de vencimento das despesas que irão ser importadas. Deve estar no formato "dd/MM/yyyy" e só deve existir caso o getExpenses_dateEnd existir também.</t>
@@ -575,7 +575,7 @@
     <t>getExpenses_dateEnd</t>
   </si>
   <si>
-    <t>01/03/2026</t>
+    <t>01/02/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Fim do range de datas que abrange a data de vencimento das despesas que irão ser importadas. Deve estar no formato "dd/MM/yyyy" e só deve existir caso o getExpenses_dateStart existir também. Deve ser posterior ao getExpenses_dateStart</t>
@@ -632,15 +632,15 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <b/>
+      <sz val="14.000000"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <u/>
       <sz val="11.000000"/>
       <color theme="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14.000000"/>
-      <color theme="1"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -754,7 +754,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="56">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -776,14 +776,17 @@
     <xf fontId="2" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
+    <xf fontId="3" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="3" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="2" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
@@ -805,12 +808,6 @@
     <xf fontId="2" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="4" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -839,7 +836,7 @@
     <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="5" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="4" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -848,14 +845,14 @@
     <xf fontId="2" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
-    <xf fontId="5" fillId="9" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="4" fillId="9" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
     <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf fontId="5" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="4" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="5" fillId="11" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="4" fillId="11" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
@@ -874,9 +871,6 @@
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -886,7 +880,7 @@
     <xf fontId="2" fillId="7" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="4" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1481,33 +1475,37 @@
       <c r="A4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="11"/>
+      <c r="B4" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="5" ht="27" customHeight="1">
       <c r="A5" s="8"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="10"/>
+      <c r="B5" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="D5" s="11"/>
     </row>
     <row r="6" ht="27" customHeight="1">
       <c r="A6" s="8"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="10"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="13"/>
       <c r="D6" s="11"/>
     </row>
     <row r="7" ht="27" customHeight="1">
       <c r="A7" s="8"/>
-      <c r="B7" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="10" t="b">
-        <v>0</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>8</v>
-      </c>
+      <c r="B7" s="12"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="11"/>
     </row>
     <row r="8" ht="17.399999999999999" customHeight="1">
       <c r="A8" s="5"/>
@@ -1516,92 +1514,90 @@
       <c r="D8" s="7"/>
     </row>
     <row r="9" ht="31.199999999999999" customHeight="1">
-      <c r="A9" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="14" t="s">
+      <c r="A9" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="15" t="s">
+      <c r="B9" s="12" t="s">
         <v>11</v>
       </c>
+      <c r="C9" s="15"/>
+      <c r="D9" s="16" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="10" ht="33.600000000000001" customHeight="1">
-      <c r="A10" s="13"/>
-      <c r="B10" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="14" t="s">
+      <c r="A10" s="14"/>
+      <c r="B10" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="C10" s="15" t="s">
         <v>14</v>
       </c>
+      <c r="D10" s="15" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="11" ht="43.200000000000003" customHeight="1">
-      <c r="A11" s="13"/>
-      <c r="B11" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="16" t="s">
+      <c r="A11" s="14"/>
+      <c r="B11" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="C11" s="17" t="s">
         <v>17</v>
       </c>
+      <c r="D11" s="16" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="12" ht="61.200000000000003" customHeight="1">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="17" t="s">
+      <c r="A12" s="14"/>
+      <c r="B12" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="C12" s="18" t="s">
         <v>20</v>
       </c>
+      <c r="D12" s="16" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="13" ht="28.800000000000001" customHeight="1">
-      <c r="A13" s="13"/>
-      <c r="B13" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="C13" s="14" t="b">
+      <c r="A13" s="14"/>
+      <c r="B13" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="15" t="b">
         <v>1</v>
       </c>
-      <c r="D13" s="14"/>
+      <c r="D13" s="15"/>
     </row>
     <row r="14" ht="28.800000000000001" customHeight="1">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="14" t="b">
+      <c r="A14" s="14"/>
+      <c r="B14" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="D14" s="14"/>
+      <c r="D14" s="15"/>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="13"/>
-      <c r="B15" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="20" t="s">
+      <c r="A15" s="14"/>
+      <c r="B15" s="19" t="s">
         <v>24</v>
       </c>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="16" ht="34.799999999999997" customHeight="1">
-      <c r="A16" s="13"/>
-      <c r="B16" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="14" t="s">
+      <c r="A16" s="14"/>
+      <c r="B16" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="20" t="s">
+      <c r="C16" s="15"/>
+      <c r="D16" s="21" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1612,38 +1608,38 @@
       <c r="D17" s="5"/>
     </row>
     <row r="18" ht="46.799999999999997" customHeight="1">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="D18" s="16" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="19" ht="46.799999999999997" customHeight="1">
-      <c r="A19" s="21"/>
+      <c r="A19" s="22"/>
       <c r="B19" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="14"/>
+      <c r="D19" s="15"/>
     </row>
     <row r="20" ht="43.200000000000003" customHeight="1">
-      <c r="A20" s="21"/>
+      <c r="A20" s="22"/>
       <c r="B20" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="23" t="s">
+      <c r="C20" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="14"/>
+      <c r="D20" s="16"/>
     </row>
     <row r="21" ht="14.25">
       <c r="C21" s="1"/>
@@ -1699,20 +1695,20 @@
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8.00390625"/>
-    <col customWidth="1" min="2" max="2" style="24" width="52.140625"/>
-    <col bestFit="1" customWidth="1" min="3" max="3" style="25" width="63.11328125"/>
-    <col customWidth="1" min="4" max="4" style="25" width="84.140625"/>
+    <col customWidth="1" min="2" max="2" style="23" width="52.140625"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" style="24" width="63.11328125"/>
+    <col customWidth="1" min="4" max="4" style="24" width="84.140625"/>
     <col customWidth="1" min="5" max="27" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="26" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="2"/>
@@ -1740,430 +1736,430 @@
       <c r="AA1" s="2"/>
     </row>
     <row r="2" ht="28.5">
-      <c r="A2" s="28"/>
-      <c r="B2" s="29" t="s">
+      <c r="A2" s="27"/>
+      <c r="B2" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="30">
+      <c r="C2" s="29">
         <v>1</v>
       </c>
-      <c r="D2" s="30" t="s">
+      <c r="D2" s="29" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="3" ht="28.5">
-      <c r="A3" s="28"/>
-      <c r="B3" s="29" t="s">
+      <c r="A3" s="27"/>
+      <c r="B3" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="30">
+      <c r="C3" s="29">
         <v>3</v>
       </c>
-      <c r="D3" s="30" t="s">
+      <c r="D3" s="29" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="28"/>
-      <c r="B4" s="29" t="s">
+      <c r="A4" s="27"/>
+      <c r="B4" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="D4" s="29" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="5" ht="28.5">
-      <c r="A5" s="28"/>
-      <c r="B5" s="29" t="s">
+      <c r="A5" s="27"/>
+      <c r="B5" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="29">
+        <v>15</v>
+      </c>
+      <c r="D5" s="29" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" ht="28.5">
+      <c r="A6" s="27"/>
+      <c r="B6" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="29">
         <v>2</v>
       </c>
-      <c r="D5" s="30" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" ht="28.5">
-      <c r="A6" s="28"/>
-      <c r="B6" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="C6" s="30">
-        <v>2</v>
-      </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="29" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="7" s="31" customFormat="1" ht="17.399999999999999" customHeight="1">
+    <row r="7" s="30" customFormat="1" ht="17.399999999999999" customHeight="1">
       <c r="A7" s="5"/>
-      <c r="B7" s="32"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
+      <c r="B7" s="31"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
     </row>
     <row r="8" ht="39.75" customHeight="1">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="33" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="35">
+      <c r="C8" s="34">
         <v>30000</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="16" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="9" ht="39.75" customHeight="1">
-      <c r="A9" s="36"/>
-      <c r="B9" s="14" t="s">
+      <c r="A9" s="35"/>
+      <c r="B9" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="35">
+      <c r="C9" s="34">
         <v>20000</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="16" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="36"/>
-      <c r="B10" s="14" t="s">
+      <c r="A10" s="35"/>
+      <c r="B10" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="35">
+      <c r="C10" s="34">
         <v>0</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="16" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="36"/>
-      <c r="B11" s="14" t="s">
+      <c r="A11" s="35"/>
+      <c r="B11" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="35">
+      <c r="C11" s="34">
         <v>0</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="16" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="12" ht="17.399999999999999" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="32"/>
-      <c r="C12" s="33"/>
-      <c r="D12" s="33"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
     </row>
     <row r="13" ht="22.800000000000001" customHeight="1">
-      <c r="A13" s="37" t="s">
+      <c r="A13" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="29" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="30" t="s">
+      <c r="D13" s="29" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="14" ht="28.199999999999999" customHeight="1">
-      <c r="A14" s="37"/>
-      <c r="B14" s="29" t="s">
+      <c r="A14" s="36"/>
+      <c r="B14" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="C14" s="30" t="s">
+      <c r="C14" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="30"/>
+      <c r="D14" s="29"/>
     </row>
     <row r="15" ht="28.199999999999999" customHeight="1">
-      <c r="A15" s="37"/>
-      <c r="B15" s="29"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="30"/>
+      <c r="A15" s="36"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
     </row>
     <row r="16" ht="27" customHeight="1">
-      <c r="A16" s="37"/>
-      <c r="B16" s="29"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
+      <c r="A16" s="36"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
     </row>
     <row r="17" ht="27" customHeight="1">
-      <c r="A17" s="37"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
+      <c r="A17" s="36"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
     </row>
     <row r="18" ht="27" customHeight="1">
-      <c r="A18" s="37"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
+      <c r="A18" s="36"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
     </row>
     <row r="19" ht="17.399999999999999" customHeight="1">
-      <c r="A19" s="38"/>
-      <c r="B19" s="32"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="33"/>
+      <c r="A19" s="37"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
     </row>
     <row r="20" ht="27" customHeight="1">
-      <c r="A20" s="39" t="s">
+      <c r="A20" s="38" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="C20" s="30" t="s">
+      <c r="C20" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="D20" s="30" t="s">
+      <c r="D20" s="29" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="21" ht="27" customHeight="1">
-      <c r="A21" s="39"/>
-      <c r="B21" s="29" t="s">
+      <c r="A21" s="38"/>
+      <c r="B21" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="C21" s="30" t="s">
+      <c r="C21" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="D21" s="30" t="s">
+      <c r="D21" s="29" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="22" ht="33.75" customHeight="1">
-      <c r="A22" s="39"/>
-      <c r="B22" s="30" t="s">
+      <c r="A22" s="38"/>
+      <c r="B22" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="C22" s="30" t="s">
+      <c r="C22" s="29" t="s">
         <v>70</v>
       </c>
-      <c r="D22" s="30"/>
+      <c r="D22" s="29"/>
     </row>
     <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="39"/>
-      <c r="B23" s="29" t="s">
+      <c r="A23" s="38"/>
+      <c r="B23" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="C23" s="30" t="s">
+      <c r="C23" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="D23" s="30"/>
+      <c r="D23" s="29"/>
     </row>
     <row r="24" ht="27" customHeight="1">
-      <c r="A24" s="39"/>
-      <c r="B24" s="29" t="s">
+      <c r="A24" s="38"/>
+      <c r="B24" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="C24" s="30" t="s">
+      <c r="C24" s="29" t="s">
         <v>74</v>
       </c>
-      <c r="D24" s="30"/>
+      <c r="D24" s="29"/>
     </row>
     <row r="25" ht="27" customHeight="1">
-      <c r="A25" s="39"/>
-      <c r="B25" s="29" t="s">
+      <c r="A25" s="38"/>
+      <c r="B25" s="28" t="s">
         <v>75</v>
       </c>
-      <c r="C25" s="20" t="s">
+      <c r="C25" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="D25" s="30"/>
+      <c r="D25" s="29"/>
     </row>
     <row r="26" ht="27" customHeight="1">
-      <c r="A26" s="39"/>
-      <c r="B26" s="29"/>
-      <c r="C26" s="30"/>
-      <c r="D26" s="30"/>
+      <c r="A26" s="38"/>
+      <c r="B26" s="28"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
     </row>
     <row r="27" ht="27" customHeight="1">
-      <c r="A27" s="39"/>
-      <c r="B27" s="29"/>
-      <c r="C27" s="30"/>
-      <c r="D27" s="30"/>
+      <c r="A27" s="38"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
     </row>
     <row r="28" ht="27" customHeight="1">
-      <c r="A28" s="39"/>
-      <c r="B28" s="29"/>
-      <c r="C28" s="30"/>
-      <c r="D28" s="30"/>
+      <c r="A28" s="38"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
     </row>
     <row r="29" ht="17.399999999999999" customHeight="1">
       <c r="A29" s="5"/>
-      <c r="B29" s="32"/>
-      <c r="C29" s="33"/>
-      <c r="D29" s="33"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="32"/>
+      <c r="D29" s="32"/>
     </row>
     <row r="30" ht="27.75" customHeight="1">
-      <c r="A30" s="40" t="s">
+      <c r="A30" s="39" t="s">
         <v>77</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="C30" s="30" t="s">
+      <c r="C30" s="29" t="s">
         <v>79</v>
       </c>
-      <c r="D30" s="30" t="s">
+      <c r="D30" s="29" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="31" ht="27.75" customHeight="1">
-      <c r="A31" s="40"/>
-      <c r="B31" s="29" t="s">
+      <c r="A31" s="39"/>
+      <c r="B31" s="28" t="s">
         <v>81</v>
       </c>
-      <c r="C31" s="30" t="s">
+      <c r="C31" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="D31" s="30" t="s">
+      <c r="D31" s="29" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="32" ht="28.5">
-      <c r="A32" s="40"/>
-      <c r="B32" s="29" t="s">
+      <c r="A32" s="39"/>
+      <c r="B32" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="C32" s="30" t="s">
+      <c r="C32" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="D32" s="30"/>
+      <c r="D32" s="29"/>
     </row>
     <row r="33" ht="28.5">
-      <c r="A33" s="40"/>
-      <c r="B33" s="29" t="s">
+      <c r="A33" s="39"/>
+      <c r="B33" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="C33" s="30" t="s">
+      <c r="C33" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="D33" s="30"/>
+      <c r="D33" s="29"/>
     </row>
     <row r="34" ht="27.75" customHeight="1">
-      <c r="A34" s="40"/>
-      <c r="B34" s="29" t="s">
+      <c r="A34" s="39"/>
+      <c r="B34" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="C34" s="30" t="s">
+      <c r="C34" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="D34" s="30" t="s">
+      <c r="D34" s="29" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="35" ht="31.199999999999999" customHeight="1">
-      <c r="A35" s="40"/>
-      <c r="B35" s="29" t="s">
+      <c r="A35" s="39"/>
+      <c r="B35" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="C35" s="30" t="s">
+      <c r="C35" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="D35" s="30"/>
+      <c r="D35" s="29"/>
     </row>
     <row r="36" ht="28.800000000000001" customHeight="1">
-      <c r="A36" s="40"/>
-      <c r="B36" s="29" t="s">
+      <c r="A36" s="39"/>
+      <c r="B36" s="28" t="s">
         <v>93</v>
       </c>
-      <c r="C36" s="30" t="s">
+      <c r="C36" s="29" t="s">
         <v>94</v>
       </c>
-      <c r="D36" s="30" t="s">
+      <c r="D36" s="29" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="37" ht="29.399999999999999" customHeight="1">
-      <c r="A37" s="40"/>
-      <c r="B37" s="29" t="s">
+      <c r="A37" s="39"/>
+      <c r="B37" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="C37" s="30" t="s">
+      <c r="C37" s="29" t="s">
         <v>97</v>
       </c>
-      <c r="D37" s="30" t="s">
+      <c r="D37" s="29" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="38" ht="42.75">
-      <c r="A38" s="40"/>
-      <c r="B38" s="29" t="s">
+      <c r="A38" s="39"/>
+      <c r="B38" s="28" t="s">
         <v>99</v>
       </c>
-      <c r="C38" s="30" t="s">
+      <c r="C38" s="29" t="s">
         <v>100</v>
       </c>
-      <c r="D38" s="30" t="s">
+      <c r="D38" s="29" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="39" ht="28.800000000000001" customHeight="1">
-      <c r="A39" s="40"/>
-      <c r="B39" s="30" t="s">
+      <c r="A39" s="39"/>
+      <c r="B39" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="C39" s="30" t="s">
+      <c r="C39" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="D39" s="30"/>
+      <c r="D39" s="29"/>
     </row>
     <row r="40" ht="28.800000000000001" customHeight="1">
-      <c r="A40" s="40"/>
-      <c r="B40" s="29"/>
-      <c r="C40" s="30"/>
-      <c r="D40" s="30"/>
+      <c r="A40" s="39"/>
+      <c r="B40" s="28"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="29"/>
     </row>
     <row r="41" ht="28.5" customHeight="1">
-      <c r="A41" s="40"/>
-      <c r="B41" s="29"/>
-      <c r="C41" s="30"/>
-      <c r="D41" s="30"/>
+      <c r="A41" s="39"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="29"/>
+      <c r="D41" s="29"/>
     </row>
     <row r="42" ht="28.5" customHeight="1">
-      <c r="A42" s="40"/>
-      <c r="B42" s="29"/>
-      <c r="C42" s="30"/>
-      <c r="D42" s="30"/>
+      <c r="A42" s="39"/>
+      <c r="B42" s="28"/>
+      <c r="C42" s="29"/>
+      <c r="D42" s="29"/>
     </row>
     <row r="43" ht="28.5" customHeight="1">
-      <c r="A43" s="40"/>
-      <c r="B43" s="29"/>
-      <c r="C43" s="30"/>
-      <c r="D43" s="30"/>
+      <c r="A43" s="39"/>
+      <c r="B43" s="28"/>
+      <c r="C43" s="29"/>
+      <c r="D43" s="29"/>
     </row>
     <row r="44" ht="28.5" customHeight="1">
-      <c r="A44" s="40"/>
-      <c r="B44" s="29"/>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
+      <c r="A44" s="39"/>
+      <c r="B44" s="28"/>
+      <c r="C44" s="29"/>
+      <c r="D44" s="29"/>
     </row>
     <row r="45" ht="28.5" customHeight="1">
-      <c r="A45" s="40"/>
-      <c r="B45" s="29"/>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
+      <c r="A45" s="39"/>
+      <c r="B45" s="28"/>
+      <c r="C45" s="29"/>
+      <c r="D45" s="29"/>
     </row>
     <row r="46" ht="28.5" customHeight="1">
-      <c r="B46" s="24"/>
-      <c r="C46" s="25"/>
-      <c r="D46" s="25"/>
+      <c r="B46" s="23"/>
+      <c r="C46" s="24"/>
+      <c r="D46" s="24"/>
     </row>
     <row r="47" ht="28.5" customHeight="1">
-      <c r="B47" s="24"/>
-      <c r="C47" s="25"/>
-      <c r="D47" s="25"/>
+      <c r="B47" s="23"/>
+      <c r="C47" s="24"/>
+      <c r="D47" s="24"/>
     </row>
     <row r="48" ht="28.5" customHeight="1"/>
     <row r="49" ht="28.5" customHeight="1"/>
@@ -2257,7 +2253,7 @@
       <c r="A3" t="s">
         <v>111</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="40" t="s">
         <v>112</v>
       </c>
       <c r="C3" t="s">
@@ -2274,7 +2270,7 @@
       <c r="B4" t="s">
         <v>114</v>
       </c>
-      <c r="C4" s="42" t="s">
+      <c r="C4" s="41" t="s">
         <v>109</v>
       </c>
       <c r="D4" t="s">
@@ -2288,7 +2284,7 @@
       <c r="B5" t="s">
         <v>117</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="C5" s="41" t="s">
         <v>109</v>
       </c>
       <c r="D5" t="s">
@@ -2296,13 +2292,13 @@
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="40" t="s">
         <v>119</v>
       </c>
       <c r="B6" t="s">
         <v>120</v>
       </c>
-      <c r="C6" s="42" t="s">
+      <c r="C6" s="41" t="s">
         <v>109</v>
       </c>
       <c r="D6" t="s">
@@ -2310,13 +2306,13 @@
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="41" t="s">
+      <c r="A7" s="40" t="s">
         <v>122</v>
       </c>
       <c r="B7" t="s">
         <v>123</v>
       </c>
-      <c r="C7" s="42" t="s">
+      <c r="C7" s="41" t="s">
         <v>109</v>
       </c>
       <c r="D7" t="s">
@@ -3329,7 +3325,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.57421875"/>
-    <col customWidth="1" min="2" max="2" style="43" width="38.421875"/>
+    <col customWidth="1" min="2" max="2" style="42" width="38.421875"/>
     <col customWidth="1" min="3" max="3" width="55.421875"/>
     <col customWidth="1" min="4" max="4" width="75.8515625"/>
   </cols>
@@ -3338,207 +3334,208 @@
       <c r="A1" t="s">
         <v>125</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" s="43" customFormat="1" ht="28.5">
-      <c r="A2" s="44"/>
-      <c r="B2" s="45" t="s">
+    <row r="2" s="42" customFormat="1" ht="28.5">
+      <c r="A2" s="43"/>
+      <c r="B2" s="44" t="s">
         <v>126</v>
       </c>
-      <c r="C2" s="46" t="s">
+      <c r="C2" s="45" t="s">
         <v>127</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="D2" s="45" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="3" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A3" s="44"/>
-      <c r="B3" s="45" t="s">
+    <row r="3" s="42" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A3" s="43"/>
+      <c r="B3" s="44" t="s">
         <v>129</v>
       </c>
-      <c r="C3" s="46" t="s">
+      <c r="C3" s="45" t="s">
         <v>130</v>
       </c>
-      <c r="D3" s="46"/>
-    </row>
-    <row r="4" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A4" s="44"/>
-      <c r="B4" s="45"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-    </row>
-    <row r="5" s="43" customFormat="1" ht="57">
-      <c r="A5" s="44"/>
-      <c r="B5" s="46" t="s">
+      <c r="D3" s="45"/>
+    </row>
+    <row r="4" s="42" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A4" s="43"/>
+      <c r="B4" s="44"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+    </row>
+    <row r="5" s="42" customFormat="1" ht="57">
+      <c r="A5" s="43"/>
+      <c r="B5" s="45" t="s">
         <v>131</v>
       </c>
-      <c r="C5" s="46" t="s">
+      <c r="C5" s="45" t="s">
         <v>132</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="45" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="6" s="43" customFormat="1" ht="36" customHeight="1">
-      <c r="A6" s="44"/>
-      <c r="B6" s="47" t="s">
+    <row r="6" s="42" customFormat="1" ht="36" customHeight="1">
+      <c r="A6" s="43"/>
+      <c r="B6" s="45" t="s">
         <v>134</v>
       </c>
-      <c r="C6" s="46" t="s">
+      <c r="C6" s="45" t="s">
         <v>135</v>
       </c>
-      <c r="D6" s="46" t="s">
+      <c r="D6" s="45" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="7" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A7" s="44"/>
-      <c r="B7" s="45" t="s">
+      <c r="G6" s="42"/>
+    </row>
+    <row r="7" s="42" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A7" s="43"/>
+      <c r="B7" s="44" t="s">
         <v>137</v>
       </c>
-      <c r="C7" s="48" t="s">
+      <c r="C7" s="46" t="s">
         <v>138</v>
       </c>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="45" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="8" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A8" s="44"/>
-      <c r="B8" s="45"/>
-      <c r="C8" s="46"/>
-      <c r="D8" s="46"/>
+    <row r="8" s="42" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A8" s="43"/>
+      <c r="B8" s="44"/>
+      <c r="C8" s="45"/>
+      <c r="D8" s="45"/>
     </row>
     <row r="9" ht="14.25">
       <c r="A9" s="5"/>
-      <c r="B9" s="49"/>
+      <c r="B9" s="47"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
     </row>
     <row r="10" ht="41.25" customHeight="1">
-      <c r="A10" s="50" t="s">
+      <c r="A10" s="48" t="s">
         <v>140</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="C10" s="51" t="s">
+      <c r="C10" s="49" t="s">
         <v>142</v>
       </c>
-      <c r="D10" s="30" t="s">
+      <c r="D10" s="29" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="52"/>
-      <c r="B11" s="29" t="s">
+      <c r="A11" s="50"/>
+      <c r="B11" s="28" t="s">
         <v>144</v>
       </c>
-      <c r="C11" s="30">
+      <c r="C11" s="29">
         <v>60000</v>
       </c>
-      <c r="D11" s="30" t="s">
+      <c r="D11" s="29" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="52"/>
-      <c r="B12" s="29" t="s">
+      <c r="A12" s="50"/>
+      <c r="B12" s="28" t="s">
         <v>146</v>
       </c>
-      <c r="C12" s="30">
+      <c r="C12" s="29">
         <v>3000</v>
       </c>
-      <c r="D12" s="30" t="s">
+      <c r="D12" s="29" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="13" ht="36.75" customHeight="1">
-      <c r="A13" s="52"/>
-      <c r="B13" s="29" t="s">
+      <c r="A13" s="50"/>
+      <c r="B13" s="28" t="s">
         <v>148</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="29" t="s">
         <v>149</v>
       </c>
-      <c r="D13" s="30" t="s">
+      <c r="D13" s="29" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="52"/>
-      <c r="B14" s="29" t="s">
+      <c r="A14" s="50"/>
+      <c r="B14" s="28" t="s">
         <v>151</v>
       </c>
-      <c r="C14" s="53" t="s">
+      <c r="C14" s="51" t="s">
         <v>152</v>
       </c>
-      <c r="D14" s="30" t="s">
+      <c r="D14" s="29" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="15" ht="63.600000000000001" customHeight="1">
-      <c r="A15" s="52"/>
-      <c r="B15" s="29" t="s">
+      <c r="A15" s="50"/>
+      <c r="B15" s="28" t="s">
         <v>154</v>
       </c>
-      <c r="C15" s="53" t="s">
+      <c r="C15" s="51" t="s">
         <v>155</v>
       </c>
-      <c r="D15" s="30" t="s">
+      <c r="D15" s="29" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="16" ht="14.25">
       <c r="A16" s="5"/>
-      <c r="B16" s="49"/>
+      <c r="B16" s="47"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
     </row>
     <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="54" t="s">
+      <c r="A17" s="52" t="s">
         <v>157</v>
       </c>
-      <c r="B17" s="55" t="s">
+      <c r="B17" s="53" t="s">
         <v>158</v>
       </c>
-      <c r="C17" s="56" t="s">
+      <c r="C17" s="54" t="s">
         <v>159</v>
       </c>
-      <c r="D17" s="57" t="s">
+      <c r="D17" s="55" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="54"/>
-      <c r="B18" s="55" t="s">
+      <c r="A18" s="52"/>
+      <c r="B18" s="53" t="s">
         <v>161</v>
       </c>
-      <c r="C18" s="56">
+      <c r="C18" s="54">
         <v>5000</v>
       </c>
-      <c r="D18" s="56" t="s">
+      <c r="D18" s="54" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="54"/>
-      <c r="B19" s="55" t="s">
+      <c r="A19" s="52"/>
+      <c r="B19" s="53" t="s">
         <v>163</v>
       </c>
-      <c r="C19" s="56" t="s">
+      <c r="C19" s="54" t="s">
         <v>149</v>
       </c>
-      <c r="D19" s="56" t="s">
+      <c r="D19" s="54" t="s">
         <v>164</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adição de tratamento de erros na integração das despesas
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="182">
   <si>
     <t>Name</t>
   </si>
@@ -296,6 +296,12 @@
     <t xml:space="preserve">Periodo de trabalho aberto com sucesso!</t>
   </si>
   <si>
+    <t>LogMessage_SuccessArcriveRead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arquivo de importação lido com sucesso!</t>
+  </si>
+  <si>
     <t xml:space="preserve">INFORMATION MESSAGES</t>
   </si>
   <si>
@@ -341,6 +347,36 @@
     <t xml:space="preserve">Abrindo periodo de fechamento...</t>
   </si>
   <si>
+    <t>LogMessage_ImportationError</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Houve um erro no momento da importação!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quando, no momento de apresentação dos relatórios, após ler os arquivos de importação, é apresentado um erro.</t>
+  </si>
+  <si>
+    <t>LogMessage_ImportationStructuralCritiques</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foram apresentadas criticas às estruturas dos arquivos txt de importação.</t>
+  </si>
+  <si>
+    <t>LogMessage_ImportationAdvertencies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Existem advertências relativas aos arquivos de importação.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quando, no momento de apresentação dos relatórios, após ler os arquivos de importação, é apresentada a tela de advertências. É necessário selecionar todos os registros à serem importados.</t>
+  </si>
+  <si>
+    <t>LogMessage_EnableExpensesIntegration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opção 'enableExpensesIntegration' está desabilitada, o processo não irá integrar as obrigações.</t>
+  </si>
+  <si>
     <t xml:space="preserve">EXCEPTION LOG MESSAGES</t>
   </si>
   <si>
@@ -416,12 +452,18 @@
     <t xml:space="preserve">Caso haja um erro durante o processo de definição de datas do request das despesas. </t>
   </si>
   <si>
-    <t>ExceptionMessage_CriticasDeEstruturasAosTxtsDeImportacao</t>
+    <t>ExceptionMessage_StructuralCritiquesToImportationArchives</t>
   </si>
   <si>
     <t xml:space="preserve">Foram exibidas criticas de estruturas aos txts de importação no processo de importação. Favor verificar</t>
   </si>
   <si>
+    <t>ExceptionMessage_ImportationReportDoNotExist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O relatorio de importações do Domínio não foi apresentado.</t>
+  </si>
+  <si>
     <t>Asset</t>
   </si>
   <si>
@@ -528,6 +570,15 @@
   </si>
   <si>
     <t xml:space="preserve">Data final do periodo de trabalho cadastrado no sistema Domínio.</t>
+  </si>
+  <si>
+    <t>attribute_invisibleElement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">não disponível</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atributo que é apresentado quando um determinado elemento é apresentado na tela, mas não está disponivel para iteração. </t>
   </si>
   <si>
     <t>GetExpensesSettings</t>
@@ -754,7 +805,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="63">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -787,6 +838,7 @@
     <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="2" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
@@ -848,6 +900,12 @@
     <xf fontId="4" fillId="9" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf fontId="4" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
@@ -874,6 +932,12 @@
     <xf fontId="0" fillId="0" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -900,6 +964,12 @@
     </xf>
     <xf fontId="0" fillId="12" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="12" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="12" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1497,13 +1567,13 @@
     </row>
     <row r="6" ht="27" customHeight="1">
       <c r="A6" s="8"/>
-      <c r="B6" s="12"/>
+      <c r="B6" s="14"/>
       <c r="C6" s="13"/>
       <c r="D6" s="11"/>
     </row>
     <row r="7" ht="27" customHeight="1">
       <c r="A7" s="8"/>
-      <c r="B7" s="12"/>
+      <c r="B7" s="14"/>
       <c r="C7" s="13"/>
       <c r="D7" s="11"/>
     </row>
@@ -1514,90 +1584,90 @@
       <c r="D8" s="7"/>
     </row>
     <row r="9" ht="31.199999999999999" customHeight="1">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="16" t="s">
+      <c r="C9" s="16"/>
+      <c r="D9" s="17" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" ht="33.600000000000001" customHeight="1">
-      <c r="A10" s="14"/>
-      <c r="B10" s="15" t="s">
+      <c r="A10" s="15"/>
+      <c r="B10" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="16" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" ht="43.200000000000003" customHeight="1">
-      <c r="A11" s="14"/>
-      <c r="B11" s="15" t="s">
+      <c r="A11" s="15"/>
+      <c r="B11" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="17" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="12" ht="61.200000000000003" customHeight="1">
-      <c r="A12" s="14"/>
-      <c r="B12" s="15" t="s">
+      <c r="A12" s="15"/>
+      <c r="B12" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="16" t="s">
+      <c r="D12" s="17" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="13" ht="28.800000000000001" customHeight="1">
-      <c r="A13" s="14"/>
-      <c r="B13" s="15" t="s">
+      <c r="A13" s="15"/>
+      <c r="B13" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="15" t="b">
+      <c r="C13" s="16" t="b">
         <v>1</v>
       </c>
-      <c r="D13" s="15"/>
+      <c r="D13" s="16"/>
     </row>
     <row r="14" ht="28.800000000000001" customHeight="1">
-      <c r="A14" s="14"/>
-      <c r="B14" s="15" t="s">
+      <c r="A14" s="15"/>
+      <c r="B14" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="15" t="b">
+      <c r="C14" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="D14" s="15"/>
+      <c r="D14" s="16"/>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="14"/>
-      <c r="B15" s="19" t="s">
+      <c r="A15" s="15"/>
+      <c r="B15" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="21" t="s">
+      <c r="C15" s="21"/>
+      <c r="D15" s="22" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="16" ht="34.799999999999997" customHeight="1">
-      <c r="A16" s="14"/>
-      <c r="B16" s="19" t="s">
+      <c r="A16" s="15"/>
+      <c r="B16" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="21" t="s">
+      <c r="C16" s="16"/>
+      <c r="D16" s="22" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1608,38 +1678,38 @@
       <c r="D17" s="5"/>
     </row>
     <row r="18" ht="46.799999999999997" customHeight="1">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="16" t="s">
+      <c r="D18" s="17" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="19" ht="46.799999999999997" customHeight="1">
-      <c r="A19" s="22"/>
-      <c r="B19" s="15" t="s">
+      <c r="A19" s="23"/>
+      <c r="B19" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="15"/>
+      <c r="D19" s="16"/>
     </row>
     <row r="20" ht="43.200000000000003" customHeight="1">
-      <c r="A20" s="22"/>
-      <c r="B20" s="15" t="s">
+      <c r="A20" s="23"/>
+      <c r="B20" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="16"/>
+      <c r="D20" s="17"/>
     </row>
     <row r="21" ht="14.25">
       <c r="C21" s="1"/>
@@ -1695,20 +1765,20 @@
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8.00390625"/>
-    <col customWidth="1" min="2" max="2" style="23" width="52.140625"/>
-    <col bestFit="1" customWidth="1" min="3" max="3" style="24" width="63.11328125"/>
-    <col customWidth="1" min="4" max="4" style="24" width="84.140625"/>
+    <col customWidth="1" min="2" max="2" style="24" width="53.8515625"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" style="25" width="63.11328125"/>
+    <col customWidth="1" min="4" max="4" style="25" width="84.140625"/>
     <col customWidth="1" min="5" max="27" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="27" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="2"/>
@@ -1736,435 +1806,485 @@
       <c r="AA1" s="2"/>
     </row>
     <row r="2" ht="28.5">
-      <c r="A2" s="27"/>
-      <c r="B2" s="28" t="s">
+      <c r="A2" s="28"/>
+      <c r="B2" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="29">
+      <c r="C2" s="30">
         <v>1</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="30" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="3" ht="28.5">
-      <c r="A3" s="27"/>
-      <c r="B3" s="28" t="s">
+      <c r="A3" s="28"/>
+      <c r="B3" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="29">
+      <c r="C3" s="30">
         <v>3</v>
       </c>
-      <c r="D3" s="29" t="s">
+      <c r="D3" s="30" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="27"/>
-      <c r="B4" s="28" t="s">
+      <c r="A4" s="28"/>
+      <c r="B4" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="30" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="5" ht="28.5">
-      <c r="A5" s="27"/>
-      <c r="B5" s="28" t="s">
+      <c r="A5" s="28"/>
+      <c r="B5" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="29">
+      <c r="C5" s="30">
         <v>15</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="30" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" ht="28.5">
-      <c r="A6" s="27"/>
-      <c r="B6" s="28" t="s">
+      <c r="A6" s="28"/>
+      <c r="B6" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="29">
+      <c r="C6" s="30">
         <v>2</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="30" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="7" s="30" customFormat="1" ht="17.399999999999999" customHeight="1">
+    <row r="7" s="31" customFormat="1" ht="17.399999999999999" customHeight="1">
       <c r="A7" s="5"/>
-      <c r="B7" s="31"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
     </row>
     <row r="8" ht="39.75" customHeight="1">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="34">
+      <c r="C8" s="35">
         <v>30000</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="17" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="9" ht="39.75" customHeight="1">
-      <c r="A9" s="35"/>
-      <c r="B9" s="15" t="s">
+      <c r="A9" s="36"/>
+      <c r="B9" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="34">
+      <c r="C9" s="35">
         <v>20000</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="17" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="35"/>
-      <c r="B10" s="15" t="s">
+      <c r="A10" s="36"/>
+      <c r="B10" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="34">
+      <c r="C10" s="35">
         <v>0</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="17" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="35"/>
-      <c r="B11" s="15" t="s">
+      <c r="A11" s="36"/>
+      <c r="B11" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="34">
+      <c r="C11" s="35">
         <v>0</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="17" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="12" ht="17.399999999999999" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="31"/>
-      <c r="C12" s="32"/>
-      <c r="D12" s="32"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
     </row>
     <row r="13" ht="22.800000000000001" customHeight="1">
-      <c r="A13" s="36" t="s">
+      <c r="A13" s="37" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="28" t="s">
+      <c r="B13" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C13" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="29" t="s">
+      <c r="D13" s="30" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="14" ht="28.199999999999999" customHeight="1">
-      <c r="A14" s="36"/>
-      <c r="B14" s="28" t="s">
+      <c r="A14" s="37"/>
+      <c r="B14" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C14" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="29"/>
+      <c r="D14" s="30"/>
     </row>
     <row r="15" ht="28.199999999999999" customHeight="1">
-      <c r="A15" s="36"/>
-      <c r="B15" s="28"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
+      <c r="A15" s="37"/>
+      <c r="B15" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="D15" s="30"/>
     </row>
     <row r="16" ht="27" customHeight="1">
-      <c r="A16" s="36"/>
-      <c r="B16" s="28"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
+      <c r="A16" s="37"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
     </row>
     <row r="17" ht="27" customHeight="1">
-      <c r="A17" s="36"/>
-      <c r="B17" s="28"/>
-      <c r="C17" s="29"/>
-      <c r="D17" s="29"/>
+      <c r="A17" s="37"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
     </row>
     <row r="18" ht="27" customHeight="1">
-      <c r="A18" s="36"/>
-      <c r="B18" s="28"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
     </row>
     <row r="19" ht="17.399999999999999" customHeight="1">
-      <c r="A19" s="37"/>
-      <c r="B19" s="31"/>
-      <c r="C19" s="32"/>
-      <c r="D19" s="32"/>
+      <c r="A19" s="40"/>
+      <c r="B19" s="32"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
     </row>
     <row r="20" ht="27" customHeight="1">
-      <c r="A20" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="B20" s="28" t="s">
-        <v>63</v>
-      </c>
-      <c r="C20" s="29" t="s">
+      <c r="A20" s="41" t="s">
         <v>64</v>
       </c>
-      <c r="D20" s="29" t="s">
+      <c r="B20" s="29" t="s">
         <v>65</v>
       </c>
+      <c r="C20" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="D20" s="30" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="21" ht="27" customHeight="1">
-      <c r="A21" s="38"/>
-      <c r="B21" s="28" t="s">
-        <v>66</v>
-      </c>
-      <c r="C21" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="D21" s="29" t="s">
+      <c r="A21" s="41"/>
+      <c r="B21" s="29" t="s">
         <v>68</v>
       </c>
+      <c r="C21" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="D21" s="30" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="22" ht="33.75" customHeight="1">
-      <c r="A22" s="38"/>
-      <c r="B22" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="C22" s="29" t="s">
-        <v>70</v>
-      </c>
-      <c r="D22" s="29"/>
+      <c r="A22" s="41"/>
+      <c r="B22" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="C22" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="D22" s="30"/>
     </row>
     <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="38"/>
-      <c r="B23" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="C23" s="29" t="s">
-        <v>72</v>
-      </c>
-      <c r="D23" s="29"/>
+      <c r="A23" s="41"/>
+      <c r="B23" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="C23" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="D23" s="30"/>
     </row>
     <row r="24" ht="27" customHeight="1">
-      <c r="A24" s="38"/>
-      <c r="B24" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="C24" s="29" t="s">
-        <v>74</v>
-      </c>
-      <c r="D24" s="29"/>
+      <c r="A24" s="41"/>
+      <c r="B24" s="29" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="D24" s="30"/>
     </row>
     <row r="25" ht="27" customHeight="1">
-      <c r="A25" s="38"/>
-      <c r="B25" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="C25" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="D25" s="29"/>
-    </row>
-    <row r="26" ht="27" customHeight="1">
-      <c r="A26" s="38"/>
-      <c r="B26" s="28"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-    </row>
-    <row r="27" ht="27" customHeight="1">
-      <c r="A27" s="38"/>
-      <c r="B27" s="28"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-    </row>
-    <row r="28" ht="27" customHeight="1">
-      <c r="A28" s="38"/>
-      <c r="B28" s="28"/>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
-    </row>
-    <row r="29" ht="17.399999999999999" customHeight="1">
-      <c r="A29" s="5"/>
-      <c r="B29" s="31"/>
-      <c r="C29" s="32"/>
-      <c r="D29" s="32"/>
-    </row>
-    <row r="30" ht="27.75" customHeight="1">
-      <c r="A30" s="39" t="s">
+      <c r="A25" s="41"/>
+      <c r="B25" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="B30" s="28" t="s">
+      <c r="C25" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="C30" s="29" t="s">
+      <c r="D25" s="30"/>
+    </row>
+    <row r="26" ht="28.5">
+      <c r="A26" s="41"/>
+      <c r="B26" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="D30" s="29" t="s">
+      <c r="C26" s="39" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="31" ht="27.75" customHeight="1">
-      <c r="A31" s="39"/>
-      <c r="B31" s="28" t="s">
+      <c r="D26" s="39" t="s">
         <v>81</v>
       </c>
-      <c r="C31" s="29" t="s">
+    </row>
+    <row r="27" ht="28.5">
+      <c r="A27" s="41"/>
+      <c r="B27" s="38" t="s">
         <v>82</v>
       </c>
-      <c r="D31" s="29" t="s">
+      <c r="C27" s="39" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="32" ht="28.5">
-      <c r="A32" s="39"/>
-      <c r="B32" s="28" t="s">
+      <c r="D27" s="39" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" ht="42.75">
+      <c r="A28" s="41"/>
+      <c r="B28" s="38" t="s">
         <v>84</v>
       </c>
-      <c r="C32" s="29" t="s">
+      <c r="C28" s="39" t="s">
         <v>85</v>
       </c>
-      <c r="D32" s="29"/>
-    </row>
-    <row r="33" ht="28.5">
-      <c r="A33" s="39"/>
-      <c r="B33" s="28" t="s">
+      <c r="D28" s="39" t="s">
         <v>86</v>
       </c>
-      <c r="C33" s="29" t="s">
+    </row>
+    <row r="29" ht="28.800000000000001" customHeight="1">
+      <c r="A29" s="41"/>
+      <c r="B29" s="38" t="s">
         <v>87</v>
       </c>
-      <c r="D33" s="29"/>
+      <c r="C29" s="39" t="s">
+        <v>88</v>
+      </c>
+      <c r="D29" s="39"/>
+    </row>
+    <row r="30" ht="27.600000000000001" customHeight="1">
+      <c r="A30" s="41"/>
+      <c r="B30" s="38"/>
+      <c r="C30" s="39"/>
+      <c r="D30" s="39"/>
+    </row>
+    <row r="31" ht="26.399999999999999" customHeight="1">
+      <c r="A31" s="41"/>
+      <c r="B31" s="38"/>
+      <c r="C31" s="39"/>
+      <c r="D31" s="39"/>
+    </row>
+    <row r="32" ht="27" customHeight="1">
+      <c r="A32" s="41"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="30"/>
+      <c r="D32" s="30"/>
+    </row>
+    <row r="33" ht="17.399999999999999" customHeight="1">
+      <c r="A33" s="5"/>
+      <c r="B33" s="32"/>
+      <c r="C33" s="33"/>
+      <c r="D33" s="33"/>
     </row>
     <row r="34" ht="27.75" customHeight="1">
-      <c r="A34" s="39"/>
-      <c r="B34" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="C34" s="29" t="s">
+      <c r="A34" s="42" t="s">
         <v>89</v>
       </c>
-      <c r="D34" s="29" t="s">
+      <c r="B34" s="29" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="35" ht="31.199999999999999" customHeight="1">
-      <c r="A35" s="39"/>
-      <c r="B35" s="28" t="s">
+      <c r="C34" s="30" t="s">
         <v>91</v>
       </c>
-      <c r="C35" s="29" t="s">
+      <c r="D34" s="30" t="s">
         <v>92</v>
       </c>
-      <c r="D35" s="29"/>
-    </row>
-    <row r="36" ht="28.800000000000001" customHeight="1">
-      <c r="A36" s="39"/>
-      <c r="B36" s="28" t="s">
+    </row>
+    <row r="35" ht="27.75" customHeight="1">
+      <c r="A35" s="42"/>
+      <c r="B35" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="C36" s="29" t="s">
+      <c r="C35" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="D36" s="29" t="s">
+      <c r="D35" s="30" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="37" ht="29.399999999999999" customHeight="1">
-      <c r="A37" s="39"/>
-      <c r="B37" s="28" t="s">
+    <row r="36" ht="28.5">
+      <c r="A36" s="42"/>
+      <c r="B36" s="29" t="s">
         <v>96</v>
       </c>
-      <c r="C37" s="29" t="s">
+      <c r="C36" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="D37" s="29" t="s">
+      <c r="D36" s="30"/>
+    </row>
+    <row r="37" ht="28.5">
+      <c r="A37" s="42"/>
+      <c r="B37" s="29" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="38" ht="42.75">
-      <c r="A38" s="39"/>
-      <c r="B38" s="28" t="s">
+      <c r="C37" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="C38" s="29" t="s">
+      <c r="D37" s="30"/>
+    </row>
+    <row r="38" ht="27.75" customHeight="1">
+      <c r="A38" s="42"/>
+      <c r="B38" s="29" t="s">
         <v>100</v>
       </c>
-      <c r="D38" s="29" t="s">
+      <c r="C38" s="30" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="39" ht="28.800000000000001" customHeight="1">
-      <c r="A39" s="39"/>
+      <c r="D38" s="30" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="39" ht="31.199999999999999" customHeight="1">
+      <c r="A39" s="42"/>
       <c r="B39" s="29" t="s">
-        <v>102</v>
-      </c>
-      <c r="C39" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="D39" s="29"/>
+      <c r="C39" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="D39" s="30"/>
     </row>
     <row r="40" ht="28.800000000000001" customHeight="1">
-      <c r="A40" s="39"/>
-      <c r="B40" s="28"/>
-      <c r="C40" s="29"/>
-      <c r="D40" s="29"/>
-    </row>
-    <row r="41" ht="28.5" customHeight="1">
-      <c r="A41" s="39"/>
-      <c r="B41" s="28"/>
-      <c r="C41" s="29"/>
-      <c r="D41" s="29"/>
-    </row>
-    <row r="42" ht="28.5" customHeight="1">
-      <c r="A42" s="39"/>
-      <c r="B42" s="28"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="29"/>
-    </row>
-    <row r="43" ht="28.5" customHeight="1">
-      <c r="A43" s="39"/>
-      <c r="B43" s="28"/>
-      <c r="C43" s="29"/>
-      <c r="D43" s="29"/>
-    </row>
-    <row r="44" ht="28.5" customHeight="1">
-      <c r="A44" s="39"/>
-      <c r="B44" s="28"/>
-      <c r="C44" s="29"/>
-      <c r="D44" s="29"/>
+      <c r="A40" s="42"/>
+      <c r="B40" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="D40" s="30" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="41" ht="29.399999999999999" customHeight="1">
+      <c r="A41" s="42"/>
+      <c r="B41" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="C41" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="D41" s="30" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="42" ht="42.75">
+      <c r="A42" s="42"/>
+      <c r="B42" s="29" t="s">
+        <v>111</v>
+      </c>
+      <c r="C42" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="D42" s="30" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="43" ht="28.800000000000001" customHeight="1">
+      <c r="A43" s="42"/>
+      <c r="B43" s="39" t="s">
+        <v>114</v>
+      </c>
+      <c r="C43" s="30" t="s">
+        <v>115</v>
+      </c>
+      <c r="D43" s="30"/>
+    </row>
+    <row r="44" ht="28.800000000000001" customHeight="1">
+      <c r="A44" s="42"/>
+      <c r="B44" s="38" t="s">
+        <v>116</v>
+      </c>
+      <c r="C44" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="D44" s="30"/>
     </row>
     <row r="45" ht="28.5" customHeight="1">
-      <c r="A45" s="39"/>
-      <c r="B45" s="28"/>
-      <c r="C45" s="29"/>
-      <c r="D45" s="29"/>
+      <c r="A45" s="42"/>
+      <c r="B45" s="29"/>
+      <c r="C45" s="30"/>
+      <c r="D45" s="30"/>
     </row>
     <row r="46" ht="28.5" customHeight="1">
-      <c r="B46" s="23"/>
-      <c r="C46" s="24"/>
-      <c r="D46" s="24"/>
+      <c r="A46" s="42"/>
+      <c r="B46" s="29"/>
+      <c r="C46" s="30"/>
+      <c r="D46" s="30"/>
     </row>
     <row r="47" ht="28.5" customHeight="1">
-      <c r="B47" s="23"/>
-      <c r="C47" s="24"/>
-      <c r="D47" s="24"/>
-    </row>
-    <row r="48" ht="28.5" customHeight="1"/>
-    <row r="49" ht="28.5" customHeight="1"/>
-    <row r="50" ht="28.5" customHeight="1"/>
-    <row r="51" ht="28.5" customHeight="1"/>
+      <c r="A47" s="42"/>
+      <c r="B47" s="29"/>
+      <c r="C47" s="30"/>
+      <c r="D47" s="30"/>
+    </row>
+    <row r="48" ht="28.5" customHeight="1">
+      <c r="A48" s="42"/>
+      <c r="B48" s="29"/>
+      <c r="C48" s="30"/>
+      <c r="D48" s="30"/>
+    </row>
+    <row r="49" ht="28.5" customHeight="1">
+      <c r="A49" s="42"/>
+      <c r="B49" s="29"/>
+      <c r="C49" s="30"/>
+      <c r="D49" s="30"/>
+    </row>
+    <row r="50" ht="28.5" customHeight="1">
+      <c r="B50" s="24"/>
+      <c r="C50" s="25"/>
+      <c r="D50" s="25"/>
+    </row>
+    <row r="51" ht="28.5" customHeight="1">
+      <c r="B51" s="24"/>
+      <c r="C51" s="25"/>
+      <c r="D51" s="25"/>
+    </row>
     <row r="52" ht="28.5" customHeight="1"/>
     <row r="53" ht="28.5" customHeight="1"/>
     <row r="54" ht="28.5" customHeight="1"/>
@@ -2174,13 +2294,17 @@
     <row r="58" ht="28.5" customHeight="1"/>
     <row r="59" ht="28.5" customHeight="1"/>
     <row r="60" ht="28.5" customHeight="1"/>
+    <row r="61" ht="28.5" customHeight="1"/>
+    <row r="62" ht="28.5" customHeight="1"/>
+    <row r="63" ht="28.5" customHeight="1"/>
+    <row r="64" ht="28.5" customHeight="1"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:A6"/>
     <mergeCell ref="A8:A11"/>
     <mergeCell ref="A13:A18"/>
-    <mergeCell ref="A20:A28"/>
-    <mergeCell ref="A30:A45"/>
+    <mergeCell ref="A20:A32"/>
+    <mergeCell ref="A34:A49"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
@@ -2204,13 +2328,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -2237,86 +2361,86 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="B2" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="C2" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="D2" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>111</v>
-      </c>
-      <c r="B3" s="40" t="s">
-        <v>112</v>
+        <v>125</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>126</v>
       </c>
       <c r="C3" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="D3" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="B4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C4" s="41" t="s">
-        <v>109</v>
+        <v>128</v>
+      </c>
+      <c r="C4" s="44" t="s">
+        <v>123</v>
       </c>
       <c r="D4" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="B5" t="s">
-        <v>117</v>
-      </c>
-      <c r="C5" s="41" t="s">
-        <v>109</v>
+        <v>131</v>
+      </c>
+      <c r="C5" s="44" t="s">
+        <v>123</v>
       </c>
       <c r="D5" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="40" t="s">
-        <v>119</v>
+      <c r="A6" s="43" t="s">
+        <v>133</v>
       </c>
       <c r="B6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C6" s="41" t="s">
-        <v>109</v>
+        <v>134</v>
+      </c>
+      <c r="C6" s="44" t="s">
+        <v>123</v>
       </c>
       <c r="D6" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="40" t="s">
-        <v>122</v>
+      <c r="A7" s="43" t="s">
+        <v>136</v>
       </c>
       <c r="B7" t="s">
+        <v>137</v>
+      </c>
+      <c r="C7" s="44" t="s">
         <v>123</v>
       </c>
-      <c r="C7" s="41" t="s">
-        <v>109</v>
-      </c>
       <c r="D7" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1"/>
@@ -3325,221 +3449,229 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.57421875"/>
-    <col customWidth="1" min="2" max="2" style="42" width="38.421875"/>
+    <col customWidth="1" min="2" max="2" style="45" width="38.421875"/>
     <col customWidth="1" min="3" max="3" width="55.421875"/>
     <col customWidth="1" min="4" max="4" width="75.8515625"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
       <c r="A1" t="s">
-        <v>125</v>
-      </c>
-      <c r="B1" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="B1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="27" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" s="42" customFormat="1" ht="28.5">
-      <c r="A2" s="43"/>
-      <c r="B2" s="44" t="s">
-        <v>126</v>
-      </c>
-      <c r="C2" s="45" t="s">
-        <v>127</v>
-      </c>
-      <c r="D2" s="45" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="3" s="42" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A3" s="43"/>
-      <c r="B3" s="44" t="s">
-        <v>129</v>
-      </c>
-      <c r="C3" s="45" t="s">
-        <v>130</v>
-      </c>
-      <c r="D3" s="45"/>
-    </row>
-    <row r="4" s="42" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A4" s="43"/>
-      <c r="B4" s="44"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-    </row>
-    <row r="5" s="42" customFormat="1" ht="57">
-      <c r="A5" s="43"/>
-      <c r="B5" s="45" t="s">
-        <v>131</v>
-      </c>
-      <c r="C5" s="45" t="s">
-        <v>132</v>
-      </c>
-      <c r="D5" s="45" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="6" s="42" customFormat="1" ht="36" customHeight="1">
-      <c r="A6" s="43"/>
-      <c r="B6" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="C6" s="45" t="s">
-        <v>135</v>
-      </c>
-      <c r="D6" s="45" t="s">
-        <v>136</v>
-      </c>
-      <c r="G6" s="42"/>
-    </row>
-    <row r="7" s="42" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A7" s="43"/>
-      <c r="B7" s="44" t="s">
-        <v>137</v>
-      </c>
-      <c r="C7" s="46" t="s">
-        <v>138</v>
-      </c>
-      <c r="D7" s="45" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="8" s="42" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A8" s="43"/>
-      <c r="B8" s="44"/>
-      <c r="C8" s="45"/>
-      <c r="D8" s="45"/>
+    <row r="2" s="45" customFormat="1" ht="28.5">
+      <c r="A2" s="46"/>
+      <c r="B2" s="47" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" s="48" t="s">
+        <v>141</v>
+      </c>
+      <c r="D2" s="48" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A3" s="46"/>
+      <c r="B3" s="47" t="s">
+        <v>143</v>
+      </c>
+      <c r="C3" s="48" t="s">
+        <v>144</v>
+      </c>
+      <c r="D3" s="48"/>
+    </row>
+    <row r="4" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A4" s="46"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+    </row>
+    <row r="5" s="45" customFormat="1" ht="57">
+      <c r="A5" s="46"/>
+      <c r="B5" s="48" t="s">
+        <v>145</v>
+      </c>
+      <c r="C5" s="48" t="s">
+        <v>146</v>
+      </c>
+      <c r="D5" s="48" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="6" s="45" customFormat="1" ht="36" customHeight="1">
+      <c r="A6" s="46"/>
+      <c r="B6" s="48" t="s">
+        <v>148</v>
+      </c>
+      <c r="C6" s="48" t="s">
+        <v>149</v>
+      </c>
+      <c r="D6" s="48" t="s">
+        <v>150</v>
+      </c>
+      <c r="G6" s="45"/>
+    </row>
+    <row r="7" s="45" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A7" s="46"/>
+      <c r="B7" s="47" t="s">
+        <v>151</v>
+      </c>
+      <c r="C7" s="49" t="s">
+        <v>152</v>
+      </c>
+      <c r="D7" s="48" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="8" s="45" customFormat="1" ht="28.5">
+      <c r="A8" s="46"/>
+      <c r="B8" s="50" t="s">
+        <v>154</v>
+      </c>
+      <c r="C8" s="48" t="s">
+        <v>155</v>
+      </c>
+      <c r="D8" s="51" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="9" ht="14.25">
       <c r="A9" s="5"/>
-      <c r="B9" s="47"/>
+      <c r="B9" s="52"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
     </row>
     <row r="10" ht="41.25" customHeight="1">
-      <c r="A10" s="48" t="s">
-        <v>140</v>
-      </c>
-      <c r="B10" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="C10" s="49" t="s">
-        <v>142</v>
-      </c>
-      <c r="D10" s="29" t="s">
-        <v>143</v>
+      <c r="A10" s="53" t="s">
+        <v>157</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="C10" s="54" t="s">
+        <v>159</v>
+      </c>
+      <c r="D10" s="30" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="50"/>
-      <c r="B11" s="28" t="s">
-        <v>144</v>
-      </c>
-      <c r="C11" s="29">
+      <c r="A11" s="55"/>
+      <c r="B11" s="29" t="s">
+        <v>161</v>
+      </c>
+      <c r="C11" s="30">
         <v>60000</v>
       </c>
-      <c r="D11" s="29" t="s">
-        <v>145</v>
+      <c r="D11" s="30" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="50"/>
-      <c r="B12" s="28" t="s">
-        <v>146</v>
-      </c>
-      <c r="C12" s="29">
+      <c r="A12" s="55"/>
+      <c r="B12" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="C12" s="30">
         <v>3000</v>
       </c>
-      <c r="D12" s="29" t="s">
-        <v>147</v>
+      <c r="D12" s="30" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="13" ht="36.75" customHeight="1">
-      <c r="A13" s="50"/>
-      <c r="B13" s="28" t="s">
-        <v>148</v>
-      </c>
-      <c r="C13" s="29" t="s">
-        <v>149</v>
-      </c>
-      <c r="D13" s="29" t="s">
-        <v>150</v>
+      <c r="A13" s="55"/>
+      <c r="B13" s="29" t="s">
+        <v>165</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="D13" s="30" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="50"/>
-      <c r="B14" s="28" t="s">
-        <v>151</v>
-      </c>
-      <c r="C14" s="51" t="s">
-        <v>152</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>153</v>
+      <c r="A14" s="55"/>
+      <c r="B14" s="29" t="s">
+        <v>168</v>
+      </c>
+      <c r="C14" s="56" t="s">
+        <v>169</v>
+      </c>
+      <c r="D14" s="30" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="15" ht="63.600000000000001" customHeight="1">
-      <c r="A15" s="50"/>
-      <c r="B15" s="28" t="s">
-        <v>154</v>
-      </c>
-      <c r="C15" s="51" t="s">
-        <v>155</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>156</v>
+      <c r="A15" s="55"/>
+      <c r="B15" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="C15" s="56" t="s">
+        <v>172</v>
+      </c>
+      <c r="D15" s="30" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="16" ht="14.25">
       <c r="A16" s="5"/>
-      <c r="B16" s="47"/>
+      <c r="B16" s="52"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
     </row>
     <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="52" t="s">
-        <v>157</v>
-      </c>
-      <c r="B17" s="53" t="s">
-        <v>158</v>
-      </c>
-      <c r="C17" s="54" t="s">
-        <v>159</v>
-      </c>
-      <c r="D17" s="55" t="s">
-        <v>160</v>
+      <c r="A17" s="57" t="s">
+        <v>174</v>
+      </c>
+      <c r="B17" s="58" t="s">
+        <v>175</v>
+      </c>
+      <c r="C17" s="59" t="s">
+        <v>176</v>
+      </c>
+      <c r="D17" s="60" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="52"/>
-      <c r="B18" s="53" t="s">
-        <v>161</v>
-      </c>
-      <c r="C18" s="54">
+      <c r="A18" s="57"/>
+      <c r="B18" s="61" t="s">
+        <v>178</v>
+      </c>
+      <c r="C18" s="62">
         <v>5000</v>
       </c>
-      <c r="D18" s="54" t="s">
-        <v>162</v>
+      <c r="D18" s="62" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="52"/>
-      <c r="B19" s="53" t="s">
-        <v>163</v>
-      </c>
-      <c r="C19" s="54" t="s">
-        <v>149</v>
-      </c>
-      <c r="D19" s="54" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="20" ht="28.199999999999999" customHeight="1"/>
+      <c r="A19" s="57"/>
+      <c r="B19" s="58" t="s">
+        <v>180</v>
+      </c>
+      <c r="C19" s="62" t="s">
+        <v>166</v>
+      </c>
+      <c r="D19" s="62" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="20" ht="28.199999999999999" customHeight="1">
+      <c r="B20" s="45"/>
+    </row>
     <row r="21" ht="28.199999999999999" customHeight="1"/>
     <row r="22" ht="28.199999999999999" customHeight="1"/>
     <row r="23" ht="28.199999999999999" customHeight="1"/>

</xml_diff>

<commit_message>
Correção de pequenos bugs e inicio da implementação da lógica das datas e da estruturação das datas do get expenses
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="181">
   <si>
     <t>Name</t>
   </si>
@@ -548,16 +548,13 @@
     <t>especificDebitAccount</t>
   </si>
   <si>
-    <t>2055,1055,2074,5572</t>
-  </si>
-  <si>
     <t xml:space="preserve">O Domínio pode apresentar erro de acordo com a quantidade de despesas inseridas em um determinado arquivo de importação. Por isso, existem as contas de débito específicas que devem estar separadas por arquivo de importação.Deve estar no fomraco "contaDeDebito,contaDeDebito,contaDeDebito"</t>
   </si>
   <si>
     <t>especificExceptDebitAccounts</t>
   </si>
   <si>
-    <t>2110,2074,1204,2103,2112,2055</t>
+    <t>2110,2074,1204,2103,2112,6</t>
   </si>
   <si>
     <t xml:space="preserve">Contas de débito que não devem ser importadas para o Domínio.</t>
@@ -805,7 +802,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="61">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -845,6 +842,7 @@
     <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="5" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -906,12 +904,6 @@
     <xf fontId="4" fillId="11" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -928,12 +920,21 @@
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="2" fillId="7" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
     </xf>
@@ -942,6 +943,9 @@
     </xf>
     <xf fontId="2" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1587,7 +1591,7 @@
       <c r="B10" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="17" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="15" t="s">
@@ -1599,7 +1603,7 @@
       <c r="B11" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="18" t="s">
         <v>17</v>
       </c>
       <c r="D11" s="16" t="s">
@@ -1611,7 +1615,7 @@
       <c r="B12" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="19" t="s">
         <v>20</v>
       </c>
       <c r="D12" s="16" t="s">
@@ -1640,21 +1644,21 @@
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="14"/>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="21" t="s">
+      <c r="C15" s="21"/>
+      <c r="D15" s="22" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="16" ht="34.799999999999997" customHeight="1">
       <c r="A16" s="14"/>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="20" t="s">
         <v>26</v>
       </c>
       <c r="C16" s="15"/>
-      <c r="D16" s="21" t="s">
+      <c r="D16" s="22" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1665,7 +1669,7 @@
       <c r="D17" s="5"/>
     </row>
     <row r="18" ht="46.799999999999997" customHeight="1">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="23" t="s">
         <v>28</v>
       </c>
       <c r="B18" s="12" t="s">
@@ -1679,7 +1683,7 @@
       </c>
     </row>
     <row r="19" ht="46.799999999999997" customHeight="1">
-      <c r="A19" s="22"/>
+      <c r="A19" s="23"/>
       <c r="B19" s="15" t="s">
         <v>32</v>
       </c>
@@ -1689,11 +1693,11 @@
       <c r="D19" s="15"/>
     </row>
     <row r="20" ht="43.200000000000003" customHeight="1">
-      <c r="A20" s="22"/>
+      <c r="A20" s="23"/>
       <c r="B20" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="18" t="s">
         <v>35</v>
       </c>
       <c r="D20" s="16"/>
@@ -1752,20 +1756,20 @@
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8.00390625"/>
-    <col customWidth="1" min="2" max="2" style="23" width="53.8515625"/>
-    <col bestFit="1" customWidth="1" min="3" max="3" style="24" width="63.11328125"/>
-    <col customWidth="1" min="4" max="4" style="24" width="84.140625"/>
+    <col customWidth="1" min="2" max="2" style="24" width="53.8515625"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" style="25" width="63.11328125"/>
+    <col customWidth="1" min="4" max="4" style="25" width="84.140625"/>
     <col customWidth="1" min="5" max="27" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="27" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="2"/>
@@ -1793,79 +1797,79 @@
       <c r="AA1" s="2"/>
     </row>
     <row r="2" ht="28.5">
-      <c r="A2" s="27"/>
-      <c r="B2" s="28" t="s">
+      <c r="A2" s="28"/>
+      <c r="B2" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="29">
+      <c r="C2" s="30">
         <v>1</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="30" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="3" ht="28.5">
-      <c r="A3" s="27"/>
-      <c r="B3" s="28" t="s">
+      <c r="A3" s="28"/>
+      <c r="B3" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="29">
+      <c r="C3" s="30">
         <v>3</v>
       </c>
-      <c r="D3" s="29" t="s">
+      <c r="D3" s="30" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="27"/>
-      <c r="B4" s="28" t="s">
+      <c r="A4" s="28"/>
+      <c r="B4" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="30" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="5" ht="28.5">
-      <c r="A5" s="27"/>
-      <c r="B5" s="28" t="s">
+      <c r="A5" s="28"/>
+      <c r="B5" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="29">
+      <c r="C5" s="30">
         <v>15</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="30" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" ht="28.5">
-      <c r="A6" s="27"/>
-      <c r="B6" s="28" t="s">
+      <c r="A6" s="28"/>
+      <c r="B6" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="29">
+      <c r="C6" s="30">
         <v>2</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="30" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="7" s="30" customFormat="1" ht="17.399999999999999" customHeight="1">
+    <row r="7" s="31" customFormat="1" ht="17.399999999999999" customHeight="1">
       <c r="A7" s="5"/>
-      <c r="B7" s="31"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
     </row>
     <row r="8" ht="39.75" customHeight="1">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="34" t="s">
         <v>47</v>
       </c>
       <c r="B8" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="34">
+      <c r="C8" s="35">
         <v>30000</v>
       </c>
       <c r="D8" s="16" t="s">
@@ -1873,11 +1877,11 @@
       </c>
     </row>
     <row r="9" ht="39.75" customHeight="1">
-      <c r="A9" s="35"/>
+      <c r="A9" s="36"/>
       <c r="B9" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="34">
+      <c r="C9" s="35">
         <v>20000</v>
       </c>
       <c r="D9" s="16" t="s">
@@ -1885,11 +1889,11 @@
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="35"/>
+      <c r="A10" s="36"/>
       <c r="B10" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="34">
+      <c r="C10" s="35">
         <v>0</v>
       </c>
       <c r="D10" s="16" t="s">
@@ -1897,11 +1901,11 @@
       </c>
     </row>
     <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="35"/>
+      <c r="A11" s="36"/>
       <c r="B11" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="34">
+      <c r="C11" s="35">
         <v>0</v>
       </c>
       <c r="D11" s="16" t="s">
@@ -1910,367 +1914,367 @@
     </row>
     <row r="12" ht="17.399999999999999" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="31"/>
-      <c r="C12" s="32"/>
-      <c r="D12" s="32"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
     </row>
     <row r="13" ht="22.800000000000001" customHeight="1">
-      <c r="A13" s="36" t="s">
+      <c r="A13" s="37" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="28" t="s">
+      <c r="B13" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C13" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="29" t="s">
+      <c r="D13" s="30" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="14" ht="28.199999999999999" customHeight="1">
-      <c r="A14" s="36"/>
-      <c r="B14" s="28" t="s">
+      <c r="A14" s="37"/>
+      <c r="B14" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C14" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="29"/>
+      <c r="D14" s="30"/>
     </row>
     <row r="15" ht="28.199999999999999" customHeight="1">
-      <c r="A15" s="36"/>
-      <c r="B15" s="28" t="s">
+      <c r="A15" s="37"/>
+      <c r="B15" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="C15" s="29" t="s">
+      <c r="C15" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="D15" s="29"/>
+      <c r="D15" s="30"/>
     </row>
     <row r="16" ht="27" customHeight="1">
-      <c r="A16" s="36"/>
-      <c r="B16" s="28"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
+      <c r="A16" s="37"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
     </row>
     <row r="17" ht="27" customHeight="1">
-      <c r="A17" s="36"/>
-      <c r="B17" s="28"/>
-      <c r="C17" s="29"/>
-      <c r="D17" s="29"/>
+      <c r="A17" s="37"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
     </row>
     <row r="18" ht="27" customHeight="1">
-      <c r="A18" s="36"/>
-      <c r="B18" s="28"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
     </row>
     <row r="19" ht="17.399999999999999" customHeight="1">
-      <c r="A19" s="37"/>
-      <c r="B19" s="31"/>
-      <c r="C19" s="32"/>
-      <c r="D19" s="32"/>
+      <c r="A19" s="38"/>
+      <c r="B19" s="32"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
     </row>
     <row r="20" ht="27" customHeight="1">
-      <c r="A20" s="38" t="s">
+      <c r="A20" s="39" t="s">
         <v>64</v>
       </c>
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="C20" s="29" t="s">
+      <c r="C20" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="D20" s="29" t="s">
+      <c r="D20" s="30" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="21" ht="27" customHeight="1">
-      <c r="A21" s="38"/>
-      <c r="B21" s="28" t="s">
+      <c r="A21" s="39"/>
+      <c r="B21" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="C21" s="29" t="s">
+      <c r="C21" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="D21" s="29" t="s">
+      <c r="D21" s="30" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="22" ht="33.75" customHeight="1">
-      <c r="A22" s="38"/>
-      <c r="B22" s="29" t="s">
+      <c r="A22" s="39"/>
+      <c r="B22" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="C22" s="29" t="s">
+      <c r="C22" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="D22" s="29"/>
+      <c r="D22" s="30"/>
     </row>
     <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="38"/>
-      <c r="B23" s="28" t="s">
+      <c r="A23" s="39"/>
+      <c r="B23" s="29" t="s">
         <v>73</v>
       </c>
-      <c r="C23" s="29" t="s">
+      <c r="C23" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="D23" s="29"/>
+      <c r="D23" s="30"/>
     </row>
     <row r="24" ht="27" customHeight="1">
-      <c r="A24" s="38"/>
-      <c r="B24" s="28" t="s">
+      <c r="A24" s="39"/>
+      <c r="B24" s="29" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="C24" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="29"/>
+      <c r="D24" s="30"/>
     </row>
     <row r="25" ht="27" customHeight="1">
-      <c r="A25" s="38"/>
-      <c r="B25" s="28" t="s">
+      <c r="A25" s="39"/>
+      <c r="B25" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="C25" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="D25" s="29"/>
+      <c r="D25" s="30"/>
     </row>
     <row r="26" ht="28.5">
-      <c r="A26" s="38"/>
-      <c r="B26" s="28" t="s">
+      <c r="A26" s="39"/>
+      <c r="B26" s="29" t="s">
         <v>79</v>
       </c>
-      <c r="C26" s="29" t="s">
+      <c r="C26" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="D26" s="29" t="s">
+      <c r="D26" s="30" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="27" ht="28.5">
-      <c r="A27" s="38"/>
-      <c r="B27" s="28" t="s">
+      <c r="A27" s="39"/>
+      <c r="B27" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="C27" s="29" t="s">
+      <c r="C27" s="30" t="s">
         <v>83</v>
       </c>
-      <c r="D27" s="29" t="s">
+      <c r="D27" s="30" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="28" ht="42.75">
-      <c r="A28" s="38"/>
-      <c r="B28" s="28" t="s">
+      <c r="A28" s="39"/>
+      <c r="B28" s="29" t="s">
         <v>84</v>
       </c>
-      <c r="C28" s="29" t="s">
+      <c r="C28" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="D28" s="29" t="s">
+      <c r="D28" s="30" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="29" ht="28.800000000000001" customHeight="1">
-      <c r="A29" s="38"/>
-      <c r="B29" s="28" t="s">
+      <c r="A29" s="39"/>
+      <c r="B29" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="C29" s="29" t="s">
+      <c r="C29" s="30" t="s">
         <v>88</v>
       </c>
-      <c r="D29" s="29"/>
+      <c r="D29" s="30"/>
     </row>
     <row r="30" ht="27.600000000000001" customHeight="1">
-      <c r="A30" s="38"/>
-      <c r="B30" s="28"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
+      <c r="A30" s="39"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="30"/>
+      <c r="D30" s="30"/>
     </row>
     <row r="31" ht="26.399999999999999" customHeight="1">
-      <c r="A31" s="38"/>
-      <c r="B31" s="28"/>
-      <c r="C31" s="29"/>
-      <c r="D31" s="29"/>
+      <c r="A31" s="39"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="30"/>
+      <c r="D31" s="30"/>
     </row>
     <row r="32" ht="27" customHeight="1">
-      <c r="A32" s="38"/>
-      <c r="B32" s="28"/>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
+      <c r="A32" s="39"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="30"/>
+      <c r="D32" s="30"/>
     </row>
     <row r="33" ht="17.399999999999999" customHeight="1">
       <c r="A33" s="5"/>
-      <c r="B33" s="31"/>
-      <c r="C33" s="32"/>
-      <c r="D33" s="32"/>
+      <c r="B33" s="32"/>
+      <c r="C33" s="33"/>
+      <c r="D33" s="33"/>
     </row>
     <row r="34" ht="27.75" customHeight="1">
-      <c r="A34" s="39" t="s">
+      <c r="A34" s="40" t="s">
         <v>89</v>
       </c>
-      <c r="B34" s="40" t="s">
+      <c r="B34" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="C34" s="41" t="s">
+      <c r="C34" s="30" t="s">
         <v>91</v>
       </c>
-      <c r="D34" s="29" t="s">
+      <c r="D34" s="30" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="35" ht="27.75" customHeight="1">
-      <c r="A35" s="39"/>
-      <c r="B35" s="28" t="s">
+      <c r="A35" s="40"/>
+      <c r="B35" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="C35" s="29" t="s">
+      <c r="C35" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="D35" s="29" t="s">
+      <c r="D35" s="30" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="36" ht="28.5">
-      <c r="A36" s="39"/>
-      <c r="B36" s="28" t="s">
+      <c r="A36" s="40"/>
+      <c r="B36" s="29" t="s">
         <v>96</v>
       </c>
-      <c r="C36" s="29" t="s">
+      <c r="C36" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="D36" s="29"/>
+      <c r="D36" s="30"/>
     </row>
     <row r="37" ht="28.5">
-      <c r="A37" s="39"/>
-      <c r="B37" s="28" t="s">
+      <c r="A37" s="40"/>
+      <c r="B37" s="29" t="s">
         <v>98</v>
       </c>
-      <c r="C37" s="29" t="s">
+      <c r="C37" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="D37" s="29"/>
+      <c r="D37" s="30"/>
     </row>
     <row r="38" ht="27.75" customHeight="1">
-      <c r="A38" s="39"/>
-      <c r="B38" s="28" t="s">
+      <c r="A38" s="40"/>
+      <c r="B38" s="29" t="s">
         <v>100</v>
       </c>
-      <c r="C38" s="29" t="s">
+      <c r="C38" s="30" t="s">
         <v>101</v>
       </c>
-      <c r="D38" s="29" t="s">
+      <c r="D38" s="30" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="39" ht="31.199999999999999" customHeight="1">
-      <c r="A39" s="39"/>
-      <c r="B39" s="28" t="s">
+      <c r="A39" s="40"/>
+      <c r="B39" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="C39" s="29" t="s">
+      <c r="C39" s="30" t="s">
         <v>104</v>
       </c>
-      <c r="D39" s="29"/>
+      <c r="D39" s="30"/>
     </row>
     <row r="40" ht="28.800000000000001" customHeight="1">
-      <c r="A40" s="39"/>
-      <c r="B40" s="28" t="s">
+      <c r="A40" s="40"/>
+      <c r="B40" s="29" t="s">
         <v>105</v>
       </c>
-      <c r="C40" s="29" t="s">
+      <c r="C40" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="D40" s="29" t="s">
+      <c r="D40" s="30" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="41" ht="29.399999999999999" customHeight="1">
-      <c r="A41" s="39"/>
-      <c r="B41" s="28" t="s">
+      <c r="A41" s="40"/>
+      <c r="B41" s="29" t="s">
         <v>108</v>
       </c>
-      <c r="C41" s="29" t="s">
+      <c r="C41" s="30" t="s">
         <v>109</v>
       </c>
-      <c r="D41" s="29" t="s">
+      <c r="D41" s="30" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="42" ht="42.75">
-      <c r="A42" s="39"/>
-      <c r="B42" s="28" t="s">
+      <c r="A42" s="40"/>
+      <c r="B42" s="29" t="s">
         <v>111</v>
       </c>
-      <c r="C42" s="29" t="s">
+      <c r="C42" s="30" t="s">
         <v>112</v>
       </c>
-      <c r="D42" s="29" t="s">
+      <c r="D42" s="30" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="43" ht="28.800000000000001" customHeight="1">
-      <c r="A43" s="39"/>
-      <c r="B43" s="29" t="s">
+      <c r="A43" s="40"/>
+      <c r="B43" s="30" t="s">
         <v>114</v>
       </c>
-      <c r="C43" s="29" t="s">
+      <c r="C43" s="30" t="s">
         <v>115</v>
       </c>
-      <c r="D43" s="29"/>
+      <c r="D43" s="30"/>
     </row>
     <row r="44" ht="28.800000000000001" customHeight="1">
-      <c r="A44" s="39"/>
-      <c r="B44" s="28" t="s">
+      <c r="A44" s="40"/>
+      <c r="B44" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="C44" s="29" t="s">
+      <c r="C44" s="30" t="s">
         <v>117</v>
       </c>
-      <c r="D44" s="29"/>
+      <c r="D44" s="30"/>
     </row>
     <row r="45" ht="28.5" customHeight="1">
-      <c r="A45" s="39"/>
-      <c r="B45" s="28"/>
-      <c r="C45" s="29"/>
-      <c r="D45" s="29"/>
+      <c r="A45" s="40"/>
+      <c r="B45" s="29"/>
+      <c r="C45" s="30"/>
+      <c r="D45" s="30"/>
     </row>
     <row r="46" ht="28.5" customHeight="1">
-      <c r="A46" s="39"/>
-      <c r="B46" s="28"/>
-      <c r="C46" s="29"/>
-      <c r="D46" s="29"/>
+      <c r="A46" s="40"/>
+      <c r="B46" s="29"/>
+      <c r="C46" s="30"/>
+      <c r="D46" s="30"/>
     </row>
     <row r="47" ht="28.5" customHeight="1">
-      <c r="A47" s="39"/>
-      <c r="B47" s="28"/>
-      <c r="C47" s="29"/>
-      <c r="D47" s="29"/>
+      <c r="A47" s="40"/>
+      <c r="B47" s="29"/>
+      <c r="C47" s="30"/>
+      <c r="D47" s="30"/>
     </row>
     <row r="48" ht="28.5" customHeight="1">
-      <c r="A48" s="39"/>
-      <c r="B48" s="28"/>
-      <c r="C48" s="29"/>
-      <c r="D48" s="29"/>
+      <c r="A48" s="40"/>
+      <c r="B48" s="29"/>
+      <c r="C48" s="30"/>
+      <c r="D48" s="30"/>
     </row>
     <row r="49" ht="28.5" customHeight="1">
-      <c r="A49" s="39"/>
-      <c r="B49" s="28"/>
-      <c r="C49" s="29"/>
-      <c r="D49" s="29"/>
+      <c r="A49" s="40"/>
+      <c r="B49" s="29"/>
+      <c r="C49" s="30"/>
+      <c r="D49" s="30"/>
     </row>
     <row r="50" ht="28.5" customHeight="1">
-      <c r="B50" s="23"/>
-      <c r="C50" s="24"/>
-      <c r="D50" s="24"/>
+      <c r="B50" s="24"/>
+      <c r="C50" s="25"/>
+      <c r="D50" s="25"/>
     </row>
     <row r="51" ht="28.5" customHeight="1">
-      <c r="B51" s="23"/>
-      <c r="C51" s="24"/>
-      <c r="D51" s="24"/>
+      <c r="B51" s="24"/>
+      <c r="C51" s="25"/>
+      <c r="D51" s="25"/>
     </row>
     <row r="52" ht="28.5" customHeight="1"/>
     <row r="53" ht="28.5" customHeight="1"/>
@@ -2364,7 +2368,7 @@
       <c r="A3" t="s">
         <v>125</v>
       </c>
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="41" t="s">
         <v>126</v>
       </c>
       <c r="C3" t="s">
@@ -2381,7 +2385,7 @@
       <c r="B4" t="s">
         <v>128</v>
       </c>
-      <c r="C4" s="43" t="s">
+      <c r="C4" s="42" t="s">
         <v>123</v>
       </c>
       <c r="D4" t="s">
@@ -2395,7 +2399,7 @@
       <c r="B5" t="s">
         <v>131</v>
       </c>
-      <c r="C5" s="43" t="s">
+      <c r="C5" s="42" t="s">
         <v>123</v>
       </c>
       <c r="D5" t="s">
@@ -2403,13 +2407,13 @@
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="42" t="s">
+      <c r="A6" s="41" t="s">
         <v>133</v>
       </c>
       <c r="B6" t="s">
         <v>134</v>
       </c>
-      <c r="C6" s="43" t="s">
+      <c r="C6" s="42" t="s">
         <v>123</v>
       </c>
       <c r="D6" t="s">
@@ -2417,13 +2421,13 @@
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="42" t="s">
+      <c r="A7" s="41" t="s">
         <v>136</v>
       </c>
       <c r="B7" t="s">
         <v>137</v>
       </c>
-      <c r="C7" s="43" t="s">
+      <c r="C7" s="42" t="s">
         <v>123</v>
       </c>
       <c r="D7" t="s">
@@ -3436,228 +3440,228 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.57421875"/>
-    <col customWidth="1" min="2" max="2" style="44" width="38.421875"/>
-    <col customWidth="1" min="3" max="3" width="55.421875"/>
-    <col customWidth="1" min="4" max="4" width="75.8515625"/>
+    <col customWidth="1" min="2" max="2" style="43" width="38.421875"/>
+    <col customWidth="1" min="3" max="3" style="43" width="49.00390625"/>
+    <col customWidth="1" min="4" max="4" style="43" width="92.7109375"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
       <c r="A1" t="s">
         <v>139</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="27" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" s="44" customFormat="1" ht="28.5">
-      <c r="A2" s="45"/>
-      <c r="B2" s="46" t="s">
+    <row r="2" s="43" customFormat="1" ht="28.5">
+      <c r="A2" s="44"/>
+      <c r="B2" s="45" t="s">
         <v>140</v>
       </c>
-      <c r="C2" s="47" t="s">
+      <c r="C2" s="46" t="s">
         <v>141</v>
       </c>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="46" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="3" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A3" s="45"/>
-      <c r="B3" s="46" t="s">
+    <row r="3" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A3" s="44"/>
+      <c r="B3" s="45" t="s">
         <v>143</v>
       </c>
-      <c r="C3" s="47" t="s">
+      <c r="C3" s="46" t="s">
         <v>144</v>
       </c>
-      <c r="D3" s="47"/>
-    </row>
-    <row r="4" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A4" s="45"/>
-      <c r="B4" s="46"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
-    </row>
-    <row r="5" s="44" customFormat="1" ht="57">
-      <c r="A5" s="45"/>
-      <c r="B5" s="47" t="s">
+      <c r="D3" s="46"/>
+    </row>
+    <row r="4" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A4" s="44"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+    </row>
+    <row r="5" s="43" customFormat="1" ht="42.75">
+      <c r="A5" s="44"/>
+      <c r="B5" s="46" t="s">
         <v>145</v>
       </c>
-      <c r="C5" s="47" t="s">
+      <c r="C5" s="47">
+        <v>2055</v>
+      </c>
+      <c r="D5" s="46" t="s">
         <v>146</v>
       </c>
-      <c r="D5" s="47" t="s">
+    </row>
+    <row r="6" s="43" customFormat="1" ht="36" customHeight="1">
+      <c r="A6" s="44"/>
+      <c r="B6" s="46" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="6" s="44" customFormat="1" ht="36" customHeight="1">
-      <c r="A6" s="45"/>
-      <c r="B6" s="47" t="s">
+      <c r="C6" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="C6" s="47" t="s">
+      <c r="D6" s="46" t="s">
         <v>149</v>
       </c>
-      <c r="D6" s="47" t="s">
+      <c r="G6" s="43"/>
+    </row>
+    <row r="7" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A7" s="44"/>
+      <c r="B7" s="45" t="s">
         <v>150</v>
       </c>
-      <c r="G6" s="44"/>
-    </row>
-    <row r="7" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A7" s="45"/>
-      <c r="B7" s="46" t="s">
+      <c r="C7" s="49" t="s">
         <v>151</v>
       </c>
-      <c r="C7" s="48" t="s">
+      <c r="D7" s="46" t="s">
         <v>152</v>
       </c>
-      <c r="D7" s="47" t="s">
+    </row>
+    <row r="8" s="43" customFormat="1" ht="28.5">
+      <c r="A8" s="44"/>
+      <c r="B8" s="45" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="8" s="44" customFormat="1" ht="28.5">
-      <c r="A8" s="45"/>
-      <c r="B8" s="46" t="s">
+      <c r="C8" s="46" t="s">
         <v>154</v>
       </c>
-      <c r="C8" s="47" t="s">
+      <c r="D8" s="46" t="s">
         <v>155</v>
-      </c>
-      <c r="D8" s="47" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="9" ht="14.25">
       <c r="A9" s="5"/>
-      <c r="B9" s="49"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
+      <c r="B9" s="50"/>
+      <c r="C9" s="51"/>
+      <c r="D9" s="51"/>
     </row>
     <row r="10" ht="41.25" customHeight="1">
-      <c r="A10" s="50" t="s">
+      <c r="A10" s="52" t="s">
+        <v>156</v>
+      </c>
+      <c r="B10" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="B10" s="28" t="s">
+      <c r="C10" s="53" t="s">
         <v>158</v>
       </c>
-      <c r="C10" s="51" t="s">
+      <c r="D10" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="D10" s="29" t="s">
+    </row>
+    <row r="11" ht="39.75" customHeight="1">
+      <c r="A11" s="54"/>
+      <c r="B11" s="29" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="52"/>
-      <c r="B11" s="28" t="s">
+      <c r="C11" s="30">
+        <v>60000</v>
+      </c>
+      <c r="D11" s="30" t="s">
         <v>161</v>
       </c>
-      <c r="C11" s="29">
-        <v>60000</v>
-      </c>
-      <c r="D11" s="29" t="s">
+    </row>
+    <row r="12" ht="36.75" customHeight="1">
+      <c r="A12" s="54"/>
+      <c r="B12" s="29" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="52"/>
-      <c r="B12" s="28" t="s">
+      <c r="C12" s="30">
+        <v>3000</v>
+      </c>
+      <c r="D12" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="C12" s="29">
-        <v>3000</v>
-      </c>
-      <c r="D12" s="29" t="s">
+    </row>
+    <row r="13" ht="36.75" customHeight="1">
+      <c r="A13" s="54"/>
+      <c r="B13" s="29" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="13" ht="36.75" customHeight="1">
-      <c r="A13" s="52"/>
-      <c r="B13" s="28" t="s">
+      <c r="C13" s="30" t="s">
         <v>165</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="D13" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="D13" s="29" t="s">
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="54"/>
+      <c r="B14" s="29" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="52"/>
-      <c r="B14" s="28" t="s">
+      <c r="C14" s="55" t="s">
         <v>168</v>
       </c>
-      <c r="C14" s="53" t="s">
+      <c r="D14" s="30" t="s">
         <v>169</v>
       </c>
-      <c r="D14" s="29" t="s">
+    </row>
+    <row r="15" ht="63.600000000000001" customHeight="1">
+      <c r="A15" s="54"/>
+      <c r="B15" s="29" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="15" ht="63.600000000000001" customHeight="1">
-      <c r="A15" s="52"/>
-      <c r="B15" s="28" t="s">
+      <c r="C15" s="56" t="s">
         <v>171</v>
       </c>
-      <c r="C15" s="53" t="s">
+      <c r="D15" s="30" t="s">
         <v>172</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="16" ht="14.25">
       <c r="A16" s="5"/>
-      <c r="B16" s="49"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
+      <c r="B16" s="50"/>
+      <c r="C16" s="50"/>
+      <c r="D16" s="50"/>
     </row>
     <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="54" t="s">
+      <c r="A17" s="57" t="s">
+        <v>173</v>
+      </c>
+      <c r="B17" s="58" t="s">
         <v>174</v>
       </c>
-      <c r="B17" s="55" t="s">
+      <c r="C17" s="59" t="s">
         <v>175</v>
       </c>
-      <c r="C17" s="56" t="s">
+      <c r="D17" s="60" t="s">
         <v>176</v>
       </c>
-      <c r="D17" s="57" t="s">
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="57"/>
+      <c r="B18" s="58" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="54"/>
-      <c r="B18" s="55" t="s">
+      <c r="C18" s="59">
+        <v>5000</v>
+      </c>
+      <c r="D18" s="59" t="s">
         <v>178</v>
       </c>
-      <c r="C18" s="56">
-        <v>5000</v>
-      </c>
-      <c r="D18" s="56" t="s">
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="57"/>
+      <c r="B19" s="58" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="54"/>
-      <c r="B19" s="55" t="s">
+      <c r="C19" s="59" t="s">
+        <v>165</v>
+      </c>
+      <c r="D19" s="59" t="s">
         <v>180</v>
       </c>
-      <c r="C19" s="56" t="s">
-        <v>166</v>
-      </c>
-      <c r="D19" s="56" t="s">
-        <v>181</v>
-      </c>
     </row>
     <row r="20" ht="28.199999999999999" customHeight="1">
-      <c r="B20" s="44"/>
+      <c r="B20" s="43"/>
     </row>
     <row r="21" ht="28.199999999999999" customHeight="1"/>
     <row r="22" ht="28.199999999999999" customHeight="1"/>

</xml_diff>

<commit_message>
Finalização da lógica das datas de getExpenses_dateStart e getExpenses_dateEnd
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="179">
   <si>
     <t>Name</t>
   </si>
@@ -614,16 +614,10 @@
     <t>getExpenses_dateStart</t>
   </si>
   <si>
-    <t>01/01/2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">Inicio do range de datas que abrange a data de vencimento das despesas que irão ser importadas. Deve estar no formato "dd/MM/yyyy" e só deve existir caso o getExpenses_dateEnd existir também.</t>
   </si>
   <si>
     <t>getExpenses_dateEnd</t>
-  </si>
-  <si>
-    <t>01/02/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Fim do range de datas que abrange a data de vencimento das despesas que irão ser importadas. Deve estar no formato "dd/MM/yyyy" e só deve existir caso o getExpenses_dateStart existir também. Deve ser posterior ao getExpenses_dateStart</t>
@@ -802,7 +796,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="58">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -842,7 +836,6 @@
     <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="5" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -923,9 +916,6 @@
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -943,9 +933,6 @@
     </xf>
     <xf fontId="2" fillId="7" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1591,7 +1578,7 @@
       <c r="B10" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="15" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="15" t="s">
@@ -1603,7 +1590,7 @@
       <c r="B11" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="17" t="s">
         <v>17</v>
       </c>
       <c r="D11" s="16" t="s">
@@ -1615,7 +1602,7 @@
       <c r="B12" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="18" t="s">
         <v>20</v>
       </c>
       <c r="D12" s="16" t="s">
@@ -1644,21 +1631,21 @@
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="14"/>
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="21"/>
-      <c r="D15" s="22" t="s">
+      <c r="C15" s="20"/>
+      <c r="D15" s="21" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="16" ht="34.799999999999997" customHeight="1">
       <c r="A16" s="14"/>
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="19" t="s">
         <v>26</v>
       </c>
       <c r="C16" s="15"/>
-      <c r="D16" s="22" t="s">
+      <c r="D16" s="21" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1669,7 +1656,7 @@
       <c r="D17" s="5"/>
     </row>
     <row r="18" ht="46.799999999999997" customHeight="1">
-      <c r="A18" s="23" t="s">
+      <c r="A18" s="22" t="s">
         <v>28</v>
       </c>
       <c r="B18" s="12" t="s">
@@ -1683,7 +1670,7 @@
       </c>
     </row>
     <row r="19" ht="46.799999999999997" customHeight="1">
-      <c r="A19" s="23"/>
+      <c r="A19" s="22"/>
       <c r="B19" s="15" t="s">
         <v>32</v>
       </c>
@@ -1693,11 +1680,11 @@
       <c r="D19" s="15"/>
     </row>
     <row r="20" ht="43.200000000000003" customHeight="1">
-      <c r="A20" s="23"/>
+      <c r="A20" s="22"/>
       <c r="B20" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="17" t="s">
         <v>35</v>
       </c>
       <c r="D20" s="16"/>
@@ -1756,20 +1743,20 @@
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="8.00390625"/>
-    <col customWidth="1" min="2" max="2" style="24" width="53.8515625"/>
-    <col bestFit="1" customWidth="1" min="3" max="3" style="25" width="63.11328125"/>
-    <col customWidth="1" min="4" max="4" style="25" width="84.140625"/>
+    <col customWidth="1" min="2" max="2" style="23" width="53.8515625"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" style="24" width="63.11328125"/>
+    <col customWidth="1" min="4" max="4" style="24" width="84.140625"/>
     <col customWidth="1" min="5" max="27" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="26" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="2"/>
@@ -1797,79 +1784,79 @@
       <c r="AA1" s="2"/>
     </row>
     <row r="2" ht="28.5">
-      <c r="A2" s="28"/>
-      <c r="B2" s="29" t="s">
+      <c r="A2" s="27"/>
+      <c r="B2" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="30">
+      <c r="C2" s="29">
         <v>1</v>
       </c>
-      <c r="D2" s="30" t="s">
+      <c r="D2" s="29" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="3" ht="28.5">
-      <c r="A3" s="28"/>
-      <c r="B3" s="29" t="s">
+      <c r="A3" s="27"/>
+      <c r="B3" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="30">
+      <c r="C3" s="29">
         <v>3</v>
       </c>
-      <c r="D3" s="30" t="s">
+      <c r="D3" s="29" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="28"/>
-      <c r="B4" s="29" t="s">
+      <c r="A4" s="27"/>
+      <c r="B4" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="D4" s="29" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="5" ht="28.5">
-      <c r="A5" s="28"/>
-      <c r="B5" s="29" t="s">
+      <c r="A5" s="27"/>
+      <c r="B5" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="29">
         <v>15</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="29" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" ht="28.5">
-      <c r="A6" s="28"/>
-      <c r="B6" s="29" t="s">
+      <c r="A6" s="27"/>
+      <c r="B6" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="30">
+      <c r="C6" s="29">
         <v>2</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="29" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="7" s="31" customFormat="1" ht="17.399999999999999" customHeight="1">
+    <row r="7" s="30" customFormat="1" ht="17.399999999999999" customHeight="1">
       <c r="A7" s="5"/>
-      <c r="B7" s="32"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
+      <c r="B7" s="31"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
     </row>
     <row r="8" ht="39.75" customHeight="1">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="33" t="s">
         <v>47</v>
       </c>
       <c r="B8" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="35">
+      <c r="C8" s="34">
         <v>30000</v>
       </c>
       <c r="D8" s="16" t="s">
@@ -1877,11 +1864,11 @@
       </c>
     </row>
     <row r="9" ht="39.75" customHeight="1">
-      <c r="A9" s="36"/>
+      <c r="A9" s="35"/>
       <c r="B9" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="35">
+      <c r="C9" s="34">
         <v>20000</v>
       </c>
       <c r="D9" s="16" t="s">
@@ -1889,11 +1876,11 @@
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
-      <c r="A10" s="36"/>
+      <c r="A10" s="35"/>
       <c r="B10" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="35">
+      <c r="C10" s="34">
         <v>0</v>
       </c>
       <c r="D10" s="16" t="s">
@@ -1901,11 +1888,11 @@
       </c>
     </row>
     <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="36"/>
+      <c r="A11" s="35"/>
       <c r="B11" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="35">
+      <c r="C11" s="34">
         <v>0</v>
       </c>
       <c r="D11" s="16" t="s">
@@ -1914,367 +1901,367 @@
     </row>
     <row r="12" ht="17.399999999999999" customHeight="1">
       <c r="A12" s="5"/>
-      <c r="B12" s="32"/>
-      <c r="C12" s="33"/>
-      <c r="D12" s="33"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
     </row>
     <row r="13" ht="22.800000000000001" customHeight="1">
-      <c r="A13" s="37" t="s">
+      <c r="A13" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="29" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="30" t="s">
+      <c r="D13" s="29" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="14" ht="28.199999999999999" customHeight="1">
-      <c r="A14" s="37"/>
-      <c r="B14" s="29" t="s">
+      <c r="A14" s="36"/>
+      <c r="B14" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="C14" s="30" t="s">
+      <c r="C14" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="30"/>
+      <c r="D14" s="29"/>
     </row>
     <row r="15" ht="28.199999999999999" customHeight="1">
-      <c r="A15" s="37"/>
-      <c r="B15" s="29" t="s">
+      <c r="A15" s="36"/>
+      <c r="B15" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="C15" s="30" t="s">
+      <c r="C15" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="D15" s="30"/>
+      <c r="D15" s="29"/>
     </row>
     <row r="16" ht="27" customHeight="1">
-      <c r="A16" s="37"/>
-      <c r="B16" s="29"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
+      <c r="A16" s="36"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
     </row>
     <row r="17" ht="27" customHeight="1">
-      <c r="A17" s="37"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
+      <c r="A17" s="36"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
     </row>
     <row r="18" ht="27" customHeight="1">
-      <c r="A18" s="37"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
+      <c r="A18" s="36"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
     </row>
     <row r="19" ht="17.399999999999999" customHeight="1">
-      <c r="A19" s="38"/>
-      <c r="B19" s="32"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="33"/>
+      <c r="A19" s="37"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
     </row>
     <row r="20" ht="27" customHeight="1">
-      <c r="A20" s="39" t="s">
+      <c r="A20" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="C20" s="30" t="s">
+      <c r="C20" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="D20" s="30" t="s">
+      <c r="D20" s="29" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="21" ht="27" customHeight="1">
-      <c r="A21" s="39"/>
-      <c r="B21" s="29" t="s">
+      <c r="A21" s="38"/>
+      <c r="B21" s="28" t="s">
         <v>68</v>
       </c>
-      <c r="C21" s="30" t="s">
+      <c r="C21" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="D21" s="30" t="s">
+      <c r="D21" s="29" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="22" ht="33.75" customHeight="1">
-      <c r="A22" s="39"/>
-      <c r="B22" s="30" t="s">
+      <c r="A22" s="38"/>
+      <c r="B22" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="C22" s="30" t="s">
+      <c r="C22" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="D22" s="30"/>
+      <c r="D22" s="29"/>
     </row>
     <row r="23" ht="27" customHeight="1">
-      <c r="A23" s="39"/>
-      <c r="B23" s="29" t="s">
+      <c r="A23" s="38"/>
+      <c r="B23" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="C23" s="30" t="s">
+      <c r="C23" s="29" t="s">
         <v>74</v>
       </c>
-      <c r="D23" s="30"/>
+      <c r="D23" s="29"/>
     </row>
     <row r="24" ht="27" customHeight="1">
-      <c r="A24" s="39"/>
-      <c r="B24" s="29" t="s">
+      <c r="A24" s="38"/>
+      <c r="B24" s="28" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="30" t="s">
+      <c r="C24" s="29" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="30"/>
+      <c r="D24" s="29"/>
     </row>
     <row r="25" ht="27" customHeight="1">
-      <c r="A25" s="39"/>
-      <c r="B25" s="29" t="s">
+      <c r="A25" s="38"/>
+      <c r="B25" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="C25" s="22" t="s">
+      <c r="C25" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="D25" s="30"/>
+      <c r="D25" s="29"/>
     </row>
     <row r="26" ht="28.5">
-      <c r="A26" s="39"/>
-      <c r="B26" s="29" t="s">
+      <c r="A26" s="38"/>
+      <c r="B26" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="C26" s="30" t="s">
+      <c r="C26" s="29" t="s">
         <v>80</v>
       </c>
-      <c r="D26" s="30" t="s">
+      <c r="D26" s="29" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="27" ht="28.5">
-      <c r="A27" s="39"/>
-      <c r="B27" s="29" t="s">
+      <c r="A27" s="38"/>
+      <c r="B27" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="C27" s="30" t="s">
+      <c r="C27" s="29" t="s">
         <v>83</v>
       </c>
-      <c r="D27" s="30" t="s">
+      <c r="D27" s="29" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="28" ht="42.75">
-      <c r="A28" s="39"/>
-      <c r="B28" s="29" t="s">
+      <c r="A28" s="38"/>
+      <c r="B28" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="C28" s="30" t="s">
+      <c r="C28" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="D28" s="30" t="s">
+      <c r="D28" s="29" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="29" ht="28.800000000000001" customHeight="1">
-      <c r="A29" s="39"/>
-      <c r="B29" s="29" t="s">
+      <c r="A29" s="38"/>
+      <c r="B29" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="C29" s="30" t="s">
+      <c r="C29" s="29" t="s">
         <v>88</v>
       </c>
-      <c r="D29" s="30"/>
+      <c r="D29" s="29"/>
     </row>
     <row r="30" ht="27.600000000000001" customHeight="1">
-      <c r="A30" s="39"/>
-      <c r="B30" s="29"/>
-      <c r="C30" s="30"/>
-      <c r="D30" s="30"/>
+      <c r="A30" s="38"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
     </row>
     <row r="31" ht="26.399999999999999" customHeight="1">
-      <c r="A31" s="39"/>
-      <c r="B31" s="29"/>
-      <c r="C31" s="30"/>
-      <c r="D31" s="30"/>
+      <c r="A31" s="38"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="29"/>
     </row>
     <row r="32" ht="27" customHeight="1">
-      <c r="A32" s="39"/>
-      <c r="B32" s="29"/>
-      <c r="C32" s="30"/>
-      <c r="D32" s="30"/>
+      <c r="A32" s="38"/>
+      <c r="B32" s="28"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="29"/>
     </row>
     <row r="33" ht="17.399999999999999" customHeight="1">
       <c r="A33" s="5"/>
-      <c r="B33" s="32"/>
-      <c r="C33" s="33"/>
-      <c r="D33" s="33"/>
+      <c r="B33" s="31"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
     </row>
     <row r="34" ht="27.75" customHeight="1">
-      <c r="A34" s="40" t="s">
+      <c r="A34" s="39" t="s">
         <v>89</v>
       </c>
-      <c r="B34" s="29" t="s">
+      <c r="B34" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="C34" s="30" t="s">
+      <c r="C34" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="D34" s="30" t="s">
+      <c r="D34" s="29" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="35" ht="27.75" customHeight="1">
-      <c r="A35" s="40"/>
-      <c r="B35" s="29" t="s">
+      <c r="A35" s="39"/>
+      <c r="B35" s="28" t="s">
         <v>93</v>
       </c>
-      <c r="C35" s="30" t="s">
+      <c r="C35" s="29" t="s">
         <v>94</v>
       </c>
-      <c r="D35" s="30" t="s">
+      <c r="D35" s="29" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="36" ht="28.5">
-      <c r="A36" s="40"/>
-      <c r="B36" s="29" t="s">
+      <c r="A36" s="39"/>
+      <c r="B36" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="C36" s="30" t="s">
+      <c r="C36" s="29" t="s">
         <v>97</v>
       </c>
-      <c r="D36" s="30"/>
+      <c r="D36" s="29"/>
     </row>
     <row r="37" ht="28.5">
-      <c r="A37" s="40"/>
-      <c r="B37" s="29" t="s">
+      <c r="A37" s="39"/>
+      <c r="B37" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="C37" s="30" t="s">
+      <c r="C37" s="29" t="s">
         <v>99</v>
       </c>
-      <c r="D37" s="30"/>
+      <c r="D37" s="29"/>
     </row>
     <row r="38" ht="27.75" customHeight="1">
-      <c r="A38" s="40"/>
-      <c r="B38" s="29" t="s">
+      <c r="A38" s="39"/>
+      <c r="B38" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="C38" s="30" t="s">
+      <c r="C38" s="29" t="s">
         <v>101</v>
       </c>
-      <c r="D38" s="30" t="s">
+      <c r="D38" s="29" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="39" ht="31.199999999999999" customHeight="1">
-      <c r="A39" s="40"/>
-      <c r="B39" s="29" t="s">
+      <c r="A39" s="39"/>
+      <c r="B39" s="28" t="s">
         <v>103</v>
       </c>
-      <c r="C39" s="30" t="s">
+      <c r="C39" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="D39" s="30"/>
+      <c r="D39" s="29"/>
     </row>
     <row r="40" ht="28.800000000000001" customHeight="1">
-      <c r="A40" s="40"/>
-      <c r="B40" s="29" t="s">
+      <c r="A40" s="39"/>
+      <c r="B40" s="28" t="s">
         <v>105</v>
       </c>
-      <c r="C40" s="30" t="s">
+      <c r="C40" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="D40" s="30" t="s">
+      <c r="D40" s="29" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="41" ht="29.399999999999999" customHeight="1">
-      <c r="A41" s="40"/>
-      <c r="B41" s="29" t="s">
+      <c r="A41" s="39"/>
+      <c r="B41" s="28" t="s">
         <v>108</v>
       </c>
-      <c r="C41" s="30" t="s">
+      <c r="C41" s="29" t="s">
         <v>109</v>
       </c>
-      <c r="D41" s="30" t="s">
+      <c r="D41" s="29" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="42" ht="42.75">
-      <c r="A42" s="40"/>
-      <c r="B42" s="29" t="s">
+      <c r="A42" s="39"/>
+      <c r="B42" s="28" t="s">
         <v>111</v>
       </c>
-      <c r="C42" s="30" t="s">
+      <c r="C42" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="D42" s="30" t="s">
+      <c r="D42" s="29" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="43" ht="28.800000000000001" customHeight="1">
-      <c r="A43" s="40"/>
-      <c r="B43" s="30" t="s">
+      <c r="A43" s="39"/>
+      <c r="B43" s="29" t="s">
         <v>114</v>
       </c>
-      <c r="C43" s="30" t="s">
+      <c r="C43" s="29" t="s">
         <v>115</v>
       </c>
-      <c r="D43" s="30"/>
+      <c r="D43" s="29"/>
     </row>
     <row r="44" ht="28.800000000000001" customHeight="1">
-      <c r="A44" s="40"/>
-      <c r="B44" s="29" t="s">
+      <c r="A44" s="39"/>
+      <c r="B44" s="28" t="s">
         <v>116</v>
       </c>
-      <c r="C44" s="30" t="s">
+      <c r="C44" s="29" t="s">
         <v>117</v>
       </c>
-      <c r="D44" s="30"/>
+      <c r="D44" s="29"/>
     </row>
     <row r="45" ht="28.5" customHeight="1">
-      <c r="A45" s="40"/>
-      <c r="B45" s="29"/>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
+      <c r="A45" s="39"/>
+      <c r="B45" s="28"/>
+      <c r="C45" s="29"/>
+      <c r="D45" s="29"/>
     </row>
     <row r="46" ht="28.5" customHeight="1">
-      <c r="A46" s="40"/>
-      <c r="B46" s="29"/>
-      <c r="C46" s="30"/>
-      <c r="D46" s="30"/>
+      <c r="A46" s="39"/>
+      <c r="B46" s="28"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="29"/>
     </row>
     <row r="47" ht="28.5" customHeight="1">
-      <c r="A47" s="40"/>
-      <c r="B47" s="29"/>
-      <c r="C47" s="30"/>
-      <c r="D47" s="30"/>
+      <c r="A47" s="39"/>
+      <c r="B47" s="28"/>
+      <c r="C47" s="29"/>
+      <c r="D47" s="29"/>
     </row>
     <row r="48" ht="28.5" customHeight="1">
-      <c r="A48" s="40"/>
-      <c r="B48" s="29"/>
-      <c r="C48" s="30"/>
-      <c r="D48" s="30"/>
+      <c r="A48" s="39"/>
+      <c r="B48" s="28"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="29"/>
     </row>
     <row r="49" ht="28.5" customHeight="1">
-      <c r="A49" s="40"/>
-      <c r="B49" s="29"/>
-      <c r="C49" s="30"/>
-      <c r="D49" s="30"/>
+      <c r="A49" s="39"/>
+      <c r="B49" s="28"/>
+      <c r="C49" s="29"/>
+      <c r="D49" s="29"/>
     </row>
     <row r="50" ht="28.5" customHeight="1">
-      <c r="B50" s="24"/>
-      <c r="C50" s="25"/>
-      <c r="D50" s="25"/>
+      <c r="B50" s="23"/>
+      <c r="C50" s="24"/>
+      <c r="D50" s="24"/>
     </row>
     <row r="51" ht="28.5" customHeight="1">
-      <c r="B51" s="24"/>
-      <c r="C51" s="25"/>
-      <c r="D51" s="25"/>
+      <c r="B51" s="23"/>
+      <c r="C51" s="24"/>
+      <c r="D51" s="24"/>
     </row>
     <row r="52" ht="28.5" customHeight="1"/>
     <row r="53" ht="28.5" customHeight="1"/>
@@ -2368,7 +2355,7 @@
       <c r="A3" t="s">
         <v>125</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="40" t="s">
         <v>126</v>
       </c>
       <c r="C3" t="s">
@@ -2385,7 +2372,7 @@
       <c r="B4" t="s">
         <v>128</v>
       </c>
-      <c r="C4" s="42" t="s">
+      <c r="C4" s="41" t="s">
         <v>123</v>
       </c>
       <c r="D4" t="s">
@@ -2399,7 +2386,7 @@
       <c r="B5" t="s">
         <v>131</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="C5" s="41" t="s">
         <v>123</v>
       </c>
       <c r="D5" t="s">
@@ -2407,13 +2394,13 @@
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="40" t="s">
         <v>133</v>
       </c>
       <c r="B6" t="s">
         <v>134</v>
       </c>
-      <c r="C6" s="42" t="s">
+      <c r="C6" s="41" t="s">
         <v>123</v>
       </c>
       <c r="D6" t="s">
@@ -2421,13 +2408,13 @@
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="41" t="s">
+      <c r="A7" s="40" t="s">
         <v>136</v>
       </c>
       <c r="B7" t="s">
         <v>137</v>
       </c>
-      <c r="C7" s="42" t="s">
+      <c r="C7" s="41" t="s">
         <v>123</v>
       </c>
       <c r="D7" t="s">
@@ -3440,228 +3427,224 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.57421875"/>
-    <col customWidth="1" min="2" max="2" style="43" width="38.421875"/>
-    <col customWidth="1" min="3" max="3" style="43" width="49.00390625"/>
-    <col customWidth="1" min="4" max="4" style="43" width="92.7109375"/>
+    <col customWidth="1" min="2" max="2" style="42" width="38.421875"/>
+    <col customWidth="1" min="3" max="3" style="42" width="49.00390625"/>
+    <col customWidth="1" min="4" max="4" style="42" width="92.7109375"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
       <c r="A1" t="s">
         <v>139</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="26" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" s="43" customFormat="1" ht="28.5">
-      <c r="A2" s="44"/>
-      <c r="B2" s="45" t="s">
+    <row r="2" s="42" customFormat="1" ht="28.5">
+      <c r="A2" s="43"/>
+      <c r="B2" s="44" t="s">
         <v>140</v>
       </c>
-      <c r="C2" s="46" t="s">
+      <c r="C2" s="45" t="s">
         <v>141</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="D2" s="45" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="3" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A3" s="44"/>
-      <c r="B3" s="45" t="s">
+    <row r="3" s="42" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A3" s="43"/>
+      <c r="B3" s="44" t="s">
         <v>143</v>
       </c>
-      <c r="C3" s="46" t="s">
+      <c r="C3" s="45" t="s">
         <v>144</v>
       </c>
-      <c r="D3" s="46"/>
-    </row>
-    <row r="4" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A4" s="44"/>
-      <c r="B4" s="45"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-    </row>
-    <row r="5" s="43" customFormat="1" ht="42.75">
-      <c r="A5" s="44"/>
-      <c r="B5" s="46" t="s">
+      <c r="D3" s="45"/>
+    </row>
+    <row r="4" s="42" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A4" s="43"/>
+      <c r="B4" s="44"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+    </row>
+    <row r="5" s="42" customFormat="1" ht="42.75">
+      <c r="A5" s="43"/>
+      <c r="B5" s="45" t="s">
         <v>145</v>
       </c>
-      <c r="C5" s="47">
+      <c r="C5" s="46">
         <v>2055</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="45" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="6" s="43" customFormat="1" ht="36" customHeight="1">
-      <c r="A6" s="44"/>
-      <c r="B6" s="46" t="s">
+    <row r="6" s="42" customFormat="1" ht="36" customHeight="1">
+      <c r="A6" s="43"/>
+      <c r="B6" s="45" t="s">
         <v>147</v>
       </c>
-      <c r="C6" s="48" t="s">
+      <c r="C6" s="45" t="s">
         <v>148</v>
       </c>
-      <c r="D6" s="46" t="s">
+      <c r="D6" s="45" t="s">
         <v>149</v>
       </c>
-      <c r="G6" s="43"/>
-    </row>
-    <row r="7" s="43" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A7" s="44"/>
-      <c r="B7" s="45" t="s">
+      <c r="G6" s="42"/>
+    </row>
+    <row r="7" s="42" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A7" s="43"/>
+      <c r="B7" s="44" t="s">
         <v>150</v>
       </c>
-      <c r="C7" s="49" t="s">
+      <c r="C7" s="47" t="s">
         <v>151</v>
       </c>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="45" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="8" s="43" customFormat="1" ht="28.5">
-      <c r="A8" s="44"/>
-      <c r="B8" s="45" t="s">
+    <row r="8" s="42" customFormat="1" ht="28.5">
+      <c r="A8" s="43"/>
+      <c r="B8" s="44" t="s">
         <v>153</v>
       </c>
-      <c r="C8" s="46" t="s">
+      <c r="C8" s="45" t="s">
         <v>154</v>
       </c>
-      <c r="D8" s="46" t="s">
+      <c r="D8" s="45" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="9" ht="14.25">
       <c r="A9" s="5"/>
-      <c r="B9" s="50"/>
-      <c r="C9" s="51"/>
-      <c r="D9" s="51"/>
+      <c r="B9" s="48"/>
+      <c r="C9" s="49"/>
+      <c r="D9" s="49"/>
     </row>
     <row r="10" ht="41.25" customHeight="1">
-      <c r="A10" s="52" t="s">
+      <c r="A10" s="50" t="s">
         <v>156</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="C10" s="53" t="s">
+      <c r="C10" s="51" t="s">
         <v>158</v>
       </c>
-      <c r="D10" s="30" t="s">
+      <c r="D10" s="29" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="54"/>
-      <c r="B11" s="29" t="s">
+      <c r="A11" s="52"/>
+      <c r="B11" s="28" t="s">
         <v>160</v>
       </c>
-      <c r="C11" s="30">
+      <c r="C11" s="29">
         <v>60000</v>
       </c>
-      <c r="D11" s="30" t="s">
+      <c r="D11" s="29" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="54"/>
-      <c r="B12" s="29" t="s">
+      <c r="A12" s="52"/>
+      <c r="B12" s="28" t="s">
         <v>162</v>
       </c>
-      <c r="C12" s="30">
+      <c r="C12" s="29">
         <v>3000</v>
       </c>
-      <c r="D12" s="30" t="s">
+      <c r="D12" s="29" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="13" ht="36.75" customHeight="1">
-      <c r="A13" s="54"/>
-      <c r="B13" s="29" t="s">
+      <c r="A13" s="52"/>
+      <c r="B13" s="28" t="s">
         <v>164</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="29" t="s">
         <v>165</v>
       </c>
-      <c r="D13" s="30" t="s">
+      <c r="D13" s="29" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="54"/>
-      <c r="B14" s="29" t="s">
+      <c r="A14" s="52"/>
+      <c r="B14" s="28" t="s">
         <v>167</v>
       </c>
-      <c r="C14" s="55" t="s">
+      <c r="C14" s="53"/>
+      <c r="D14" s="29" t="s">
         <v>168</v>
       </c>
-      <c r="D14" s="30" t="s">
+    </row>
+    <row r="15" ht="63.600000000000001" customHeight="1">
+      <c r="A15" s="52"/>
+      <c r="B15" s="28" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="15" ht="63.600000000000001" customHeight="1">
-      <c r="A15" s="54"/>
-      <c r="B15" s="29" t="s">
+      <c r="C15" s="53"/>
+      <c r="D15" s="29" t="s">
         <v>170</v>
-      </c>
-      <c r="C15" s="56" t="s">
-        <v>171</v>
-      </c>
-      <c r="D15" s="30" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="16" ht="14.25">
       <c r="A16" s="5"/>
-      <c r="B16" s="50"/>
-      <c r="C16" s="50"/>
-      <c r="D16" s="50"/>
+      <c r="B16" s="48"/>
+      <c r="C16" s="48"/>
+      <c r="D16" s="48"/>
     </row>
     <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="57" t="s">
+      <c r="A17" s="54" t="s">
+        <v>171</v>
+      </c>
+      <c r="B17" s="55" t="s">
+        <v>172</v>
+      </c>
+      <c r="C17" s="56" t="s">
         <v>173</v>
       </c>
-      <c r="B17" s="58" t="s">
+      <c r="D17" s="57" t="s">
         <v>174</v>
       </c>
-      <c r="C17" s="59" t="s">
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="54"/>
+      <c r="B18" s="55" t="s">
         <v>175</v>
       </c>
-      <c r="D17" s="60" t="s">
+      <c r="C18" s="56">
+        <v>5000</v>
+      </c>
+      <c r="D18" s="56" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="57"/>
-      <c r="B18" s="58" t="s">
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="54"/>
+      <c r="B19" s="55" t="s">
         <v>177</v>
       </c>
-      <c r="C18" s="59">
-        <v>5000</v>
-      </c>
-      <c r="D18" s="59" t="s">
+      <c r="C19" s="56" t="s">
+        <v>165</v>
+      </c>
+      <c r="D19" s="56" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="57"/>
-      <c r="B19" s="58" t="s">
-        <v>179</v>
-      </c>
-      <c r="C19" s="59" t="s">
-        <v>165</v>
-      </c>
-      <c r="D19" s="59" t="s">
-        <v>180</v>
-      </c>
-    </row>
     <row r="20" ht="28.199999999999999" customHeight="1">
-      <c r="B20" s="43"/>
+      <c r="B20" s="42"/>
     </row>
     <row r="21" ht="28.199999999999999" customHeight="1"/>
     <row r="22" ht="28.199999999999999" customHeight="1"/>

</xml_diff>

<commit_message>
Implementação de tratamento para situação de não haver despesas na empresa sem exceção
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -113,16 +113,10 @@
     <t>obligationDateStart</t>
   </si>
   <si>
-    <t>20/03/2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">Data inicial do range de datas que deve abranger a data de vencimento da obrigação em questão, se não estiver definida nenhuma data nessa variável, o processo define o primeiro e o ultimo dia do mês como as datas de inicio e fim do range.</t>
   </si>
   <si>
     <t>obligationDateEnd</t>
-  </si>
-  <si>
-    <t>05/04/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Data final do range de datas que deve abranger a data de vencimento da obrigação em questão, se não estiver definida nenhuma data nessa variável, o processo define o primeiro e o ultimo dia do mês como as datas de inicio e fim do range.</t>
@@ -462,6 +456,12 @@
   </si>
   <si>
     <t xml:space="preserve">O relatorio de importações do Domínio não foi apresentado.</t>
+  </si>
+  <si>
+    <t>ExceptionMessage_QueryDominioDatesLimitsError</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Houve um erro na consulta das datas de limite de importação no domínio. Data de fechamento, inicio e fim do periodo de trabalho.</t>
   </si>
   <si>
     <t>Asset</t>
@@ -796,7 +796,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="60">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -896,6 +896,12 @@
     </xf>
     <xf fontId="4" fillId="11" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
@@ -1590,39 +1596,35 @@
       <c r="B11" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="17"/>
+      <c r="D11" s="16" t="s">
         <v>17</v>
-      </c>
-      <c r="D11" s="16" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="12" ht="61.200000000000003" customHeight="1">
       <c r="A12" s="14"/>
       <c r="B12" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="18"/>
+      <c r="D12" s="16" t="s">
         <v>19</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="13" ht="28.800000000000001" customHeight="1">
       <c r="A13" s="14"/>
       <c r="B13" s="15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C13" s="15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13" s="15"/>
     </row>
     <row r="14" ht="28.800000000000001" customHeight="1">
       <c r="A14" s="14"/>
       <c r="B14" s="15" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C14" s="15" t="b">
         <v>0</v>
@@ -1632,21 +1634,21 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="14"/>
       <c r="B15" s="19" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C15" s="20"/>
       <c r="D15" s="21" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" ht="34.799999999999997" customHeight="1">
       <c r="A16" s="14"/>
       <c r="B16" s="19" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C16" s="15"/>
       <c r="D16" s="21" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" ht="17.399999999999999" customHeight="1">
@@ -1657,35 +1659,35 @@
     </row>
     <row r="18" ht="46.799999999999997" customHeight="1">
       <c r="A18" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="D18" s="16" t="s">
         <v>29</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="D18" s="16" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="19" ht="46.799999999999997" customHeight="1">
       <c r="A19" s="22"/>
       <c r="B19" s="15" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D19" s="15"/>
     </row>
     <row r="20" ht="43.200000000000003" customHeight="1">
       <c r="A20" s="22"/>
       <c r="B20" s="15" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D20" s="16"/>
     </row>
@@ -1786,61 +1788,61 @@
     <row r="2" ht="28.5">
       <c r="A2" s="27"/>
       <c r="B2" s="28" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C2" s="29">
         <v>1</v>
       </c>
       <c r="D2" s="29" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" ht="28.5">
       <c r="A3" s="27"/>
       <c r="B3" s="28" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C3" s="29">
         <v>3</v>
       </c>
       <c r="D3" s="29" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" ht="27" customHeight="1">
       <c r="A4" s="27"/>
       <c r="B4" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="29" t="s">
         <v>40</v>
-      </c>
-      <c r="C4" s="29" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" s="29" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="5" ht="28.5">
       <c r="A5" s="27"/>
       <c r="B5" s="28" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C5" s="29">
         <v>15</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" ht="28.5">
       <c r="A6" s="27"/>
       <c r="B6" s="28" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C6" s="29">
         <v>2</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" s="30" customFormat="1" ht="17.399999999999999" customHeight="1">
@@ -1851,52 +1853,52 @@
     </row>
     <row r="8" ht="39.75" customHeight="1">
       <c r="A8" s="33" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C8" s="34">
         <v>30000</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" ht="39.75" customHeight="1">
       <c r="A9" s="35"/>
       <c r="B9" s="15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C9" s="34">
         <v>20000</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" ht="39.75" customHeight="1">
       <c r="A10" s="35"/>
       <c r="B10" s="15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C10" s="34">
         <v>0</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" ht="39.75" customHeight="1">
       <c r="A11" s="35"/>
       <c r="B11" s="15" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C11" s="34">
         <v>0</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" ht="17.399999999999999" customHeight="1">
@@ -1907,35 +1909,35 @@
     </row>
     <row r="13" ht="22.800000000000001" customHeight="1">
       <c r="A13" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="29" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="28" t="s">
+      <c r="D13" s="29" t="s">
         <v>57</v>
-      </c>
-      <c r="C13" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="D13" s="29" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="14" ht="28.199999999999999" customHeight="1">
       <c r="A14" s="36"/>
       <c r="B14" s="28" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D14" s="29"/>
     </row>
     <row r="15" ht="28.199999999999999" customHeight="1">
       <c r="A15" s="36"/>
       <c r="B15" s="28" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C15" s="29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D15" s="29"/>
     </row>
@@ -1965,113 +1967,113 @@
     </row>
     <row r="20" ht="27" customHeight="1">
       <c r="A20" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="B20" s="28" t="s">
+      <c r="D20" s="29" t="s">
         <v>65</v>
-      </c>
-      <c r="C20" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="D20" s="29" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="21" ht="27" customHeight="1">
       <c r="A21" s="38"/>
       <c r="B21" s="28" t="s">
+        <v>66</v>
+      </c>
+      <c r="C21" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="D21" s="29" t="s">
         <v>68</v>
-      </c>
-      <c r="C21" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="D21" s="29" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="22" ht="33.75" customHeight="1">
       <c r="A22" s="38"/>
       <c r="B22" s="29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D22" s="29"/>
     </row>
     <row r="23" ht="27" customHeight="1">
       <c r="A23" s="38"/>
       <c r="B23" s="28" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C23" s="29" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D23" s="29"/>
     </row>
     <row r="24" ht="27" customHeight="1">
       <c r="A24" s="38"/>
       <c r="B24" s="28" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D24" s="29"/>
     </row>
     <row r="25" ht="27" customHeight="1">
       <c r="A25" s="38"/>
       <c r="B25" s="28" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D25" s="29"/>
     </row>
     <row r="26" ht="28.5">
       <c r="A26" s="38"/>
       <c r="B26" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="29" t="s">
+        <v>78</v>
+      </c>
+      <c r="D26" s="29" t="s">
         <v>79</v>
-      </c>
-      <c r="C26" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="D26" s="29" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="27" ht="28.5">
       <c r="A27" s="38"/>
       <c r="B27" s="28" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C27" s="29" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D27" s="29" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="28" ht="42.75">
       <c r="A28" s="38"/>
       <c r="B28" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="C28" s="29" t="s">
+        <v>83</v>
+      </c>
+      <c r="D28" s="29" t="s">
         <v>84</v>
-      </c>
-      <c r="C28" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="D28" s="29" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="29" ht="28.800000000000001" customHeight="1">
       <c r="A29" s="38"/>
       <c r="B29" s="28" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C29" s="29" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D29" s="29"/>
     </row>
@@ -2101,132 +2103,136 @@
     </row>
     <row r="34" ht="27.75" customHeight="1">
       <c r="A34" s="39" t="s">
+        <v>87</v>
+      </c>
+      <c r="B34" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="C34" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="B34" s="28" t="s">
+      <c r="D34" s="29" t="s">
         <v>90</v>
-      </c>
-      <c r="C34" s="29" t="s">
-        <v>91</v>
-      </c>
-      <c r="D34" s="29" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="35" ht="27.75" customHeight="1">
       <c r="A35" s="39"/>
       <c r="B35" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="C35" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="D35" s="29" t="s">
         <v>93</v>
-      </c>
-      <c r="C35" s="29" t="s">
-        <v>94</v>
-      </c>
-      <c r="D35" s="29" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="36" ht="28.5">
       <c r="A36" s="39"/>
       <c r="B36" s="28" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C36" s="29" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D36" s="29"/>
     </row>
     <row r="37" ht="28.5">
       <c r="A37" s="39"/>
       <c r="B37" s="28" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C37" s="29" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D37" s="29"/>
     </row>
     <row r="38" ht="27.75" customHeight="1">
       <c r="A38" s="39"/>
       <c r="B38" s="28" t="s">
+        <v>98</v>
+      </c>
+      <c r="C38" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="D38" s="29" t="s">
         <v>100</v>
-      </c>
-      <c r="C38" s="29" t="s">
-        <v>101</v>
-      </c>
-      <c r="D38" s="29" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="39" ht="31.199999999999999" customHeight="1">
       <c r="A39" s="39"/>
       <c r="B39" s="28" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C39" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D39" s="29"/>
     </row>
     <row r="40" ht="28.800000000000001" customHeight="1">
       <c r="A40" s="39"/>
       <c r="B40" s="28" t="s">
+        <v>103</v>
+      </c>
+      <c r="C40" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="D40" s="29" t="s">
         <v>105</v>
-      </c>
-      <c r="C40" s="29" t="s">
-        <v>106</v>
-      </c>
-      <c r="D40" s="29" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="41" ht="29.399999999999999" customHeight="1">
       <c r="A41" s="39"/>
       <c r="B41" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="C41" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="D41" s="29" t="s">
         <v>108</v>
-      </c>
-      <c r="C41" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="D41" s="29" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="42" ht="42.75">
       <c r="A42" s="39"/>
       <c r="B42" s="28" t="s">
+        <v>109</v>
+      </c>
+      <c r="C42" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D42" s="29" t="s">
         <v>111</v>
-      </c>
-      <c r="C42" s="29" t="s">
-        <v>112</v>
-      </c>
-      <c r="D42" s="29" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="43" ht="28.800000000000001" customHeight="1">
       <c r="A43" s="39"/>
       <c r="B43" s="29" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C43" s="29" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D43" s="29"/>
     </row>
     <row r="44" ht="28.800000000000001" customHeight="1">
       <c r="A44" s="39"/>
       <c r="B44" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="C44" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="D44" s="29"/>
+    </row>
+    <row r="45" ht="28.5">
+      <c r="A45" s="39"/>
+      <c r="B45" s="40" t="s">
         <v>116</v>
       </c>
-      <c r="C44" s="29" t="s">
+      <c r="C45" s="41" t="s">
         <v>117</v>
       </c>
-      <c r="D44" s="29"/>
-    </row>
-    <row r="45" ht="28.5" customHeight="1">
-      <c r="A45" s="39"/>
-      <c r="B45" s="28"/>
-      <c r="C45" s="29"/>
       <c r="D45" s="29"/>
     </row>
     <row r="46" ht="28.5" customHeight="1">
@@ -2355,7 +2361,7 @@
       <c r="A3" t="s">
         <v>125</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="42" t="s">
         <v>126</v>
       </c>
       <c r="C3" t="s">
@@ -2372,7 +2378,7 @@
       <c r="B4" t="s">
         <v>128</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="C4" s="43" t="s">
         <v>123</v>
       </c>
       <c r="D4" t="s">
@@ -2386,7 +2392,7 @@
       <c r="B5" t="s">
         <v>131</v>
       </c>
-      <c r="C5" s="41" t="s">
+      <c r="C5" s="43" t="s">
         <v>123</v>
       </c>
       <c r="D5" t="s">
@@ -2394,13 +2400,13 @@
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="40" t="s">
+      <c r="A6" s="42" t="s">
         <v>133</v>
       </c>
       <c r="B6" t="s">
         <v>134</v>
       </c>
-      <c r="C6" s="41" t="s">
+      <c r="C6" s="43" t="s">
         <v>123</v>
       </c>
       <c r="D6" t="s">
@@ -2408,13 +2414,13 @@
       </c>
     </row>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="40" t="s">
+      <c r="A7" s="42" t="s">
         <v>136</v>
       </c>
       <c r="B7" t="s">
         <v>137</v>
       </c>
-      <c r="C7" s="41" t="s">
+      <c r="C7" s="43" t="s">
         <v>123</v>
       </c>
       <c r="D7" t="s">
@@ -3427,9 +3433,9 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.57421875"/>
-    <col customWidth="1" min="2" max="2" style="42" width="38.421875"/>
-    <col customWidth="1" min="3" max="3" style="42" width="49.00390625"/>
-    <col customWidth="1" min="4" max="4" style="42" width="92.7109375"/>
+    <col customWidth="1" min="2" max="2" style="44" width="38.421875"/>
+    <col customWidth="1" min="3" max="3" style="44" width="49.00390625"/>
+    <col customWidth="1" min="4" max="4" style="44" width="92.7109375"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75">
@@ -3446,97 +3452,97 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" s="42" customFormat="1" ht="28.5">
-      <c r="A2" s="43"/>
-      <c r="B2" s="44" t="s">
+    <row r="2" s="44" customFormat="1" ht="28.5">
+      <c r="A2" s="45"/>
+      <c r="B2" s="46" t="s">
         <v>140</v>
       </c>
-      <c r="C2" s="45" t="s">
+      <c r="C2" s="47" t="s">
         <v>141</v>
       </c>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="47" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="3" s="42" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A3" s="43"/>
-      <c r="B3" s="44" t="s">
+    <row r="3" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A3" s="45"/>
+      <c r="B3" s="46" t="s">
         <v>143</v>
       </c>
-      <c r="C3" s="45" t="s">
+      <c r="C3" s="47" t="s">
         <v>144</v>
       </c>
-      <c r="D3" s="45"/>
-    </row>
-    <row r="4" s="42" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A4" s="43"/>
-      <c r="B4" s="44"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-    </row>
-    <row r="5" s="42" customFormat="1" ht="42.75">
-      <c r="A5" s="43"/>
-      <c r="B5" s="45" t="s">
+      <c r="D3" s="47"/>
+    </row>
+    <row r="4" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A4" s="45"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+    </row>
+    <row r="5" s="44" customFormat="1" ht="42.75">
+      <c r="A5" s="45"/>
+      <c r="B5" s="47" t="s">
         <v>145</v>
       </c>
-      <c r="C5" s="46">
+      <c r="C5" s="48">
         <v>2055</v>
       </c>
-      <c r="D5" s="45" t="s">
+      <c r="D5" s="47" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="6" s="42" customFormat="1" ht="36" customHeight="1">
-      <c r="A6" s="43"/>
-      <c r="B6" s="45" t="s">
+    <row r="6" s="44" customFormat="1" ht="36" customHeight="1">
+      <c r="A6" s="45"/>
+      <c r="B6" s="47" t="s">
         <v>147</v>
       </c>
-      <c r="C6" s="45" t="s">
+      <c r="C6" s="47" t="s">
         <v>148</v>
       </c>
-      <c r="D6" s="45" t="s">
+      <c r="D6" s="47" t="s">
         <v>149</v>
       </c>
-      <c r="G6" s="42"/>
-    </row>
-    <row r="7" s="42" customFormat="1" ht="21.600000000000001" customHeight="1">
-      <c r="A7" s="43"/>
-      <c r="B7" s="44" t="s">
+      <c r="G6" s="44"/>
+    </row>
+    <row r="7" s="44" customFormat="1" ht="21.600000000000001" customHeight="1">
+      <c r="A7" s="45"/>
+      <c r="B7" s="46" t="s">
         <v>150</v>
       </c>
-      <c r="C7" s="47" t="s">
+      <c r="C7" s="49" t="s">
         <v>151</v>
       </c>
-      <c r="D7" s="45" t="s">
+      <c r="D7" s="47" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="8" s="42" customFormat="1" ht="28.5">
-      <c r="A8" s="43"/>
-      <c r="B8" s="44" t="s">
+    <row r="8" s="44" customFormat="1" ht="28.5">
+      <c r="A8" s="45"/>
+      <c r="B8" s="46" t="s">
         <v>153</v>
       </c>
-      <c r="C8" s="45" t="s">
+      <c r="C8" s="47" t="s">
         <v>154</v>
       </c>
-      <c r="D8" s="45" t="s">
+      <c r="D8" s="47" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="9" ht="14.25">
       <c r="A9" s="5"/>
-      <c r="B9" s="48"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="49"/>
+      <c r="B9" s="50"/>
+      <c r="C9" s="51"/>
+      <c r="D9" s="51"/>
     </row>
     <row r="10" ht="41.25" customHeight="1">
-      <c r="A10" s="50" t="s">
+      <c r="A10" s="52" t="s">
         <v>156</v>
       </c>
       <c r="B10" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="C10" s="51" t="s">
+      <c r="C10" s="53" t="s">
         <v>158</v>
       </c>
       <c r="D10" s="29" t="s">
@@ -3544,7 +3550,7 @@
       </c>
     </row>
     <row r="11" ht="39.75" customHeight="1">
-      <c r="A11" s="52"/>
+      <c r="A11" s="54"/>
       <c r="B11" s="28" t="s">
         <v>160</v>
       </c>
@@ -3556,7 +3562,7 @@
       </c>
     </row>
     <row r="12" ht="36.75" customHeight="1">
-      <c r="A12" s="52"/>
+      <c r="A12" s="54"/>
       <c r="B12" s="28" t="s">
         <v>162</v>
       </c>
@@ -3568,7 +3574,7 @@
       </c>
     </row>
     <row r="13" ht="36.75" customHeight="1">
-      <c r="A13" s="52"/>
+      <c r="A13" s="54"/>
       <c r="B13" s="28" t="s">
         <v>164</v>
       </c>
@@ -3580,71 +3586,71 @@
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="52"/>
+      <c r="A14" s="54"/>
       <c r="B14" s="28" t="s">
         <v>167</v>
       </c>
-      <c r="C14" s="53"/>
+      <c r="C14" s="55"/>
       <c r="D14" s="29" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="15" ht="63.600000000000001" customHeight="1">
-      <c r="A15" s="52"/>
+      <c r="A15" s="54"/>
       <c r="B15" s="28" t="s">
         <v>169</v>
       </c>
-      <c r="C15" s="53"/>
+      <c r="C15" s="55"/>
       <c r="D15" s="29" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="16" ht="14.25">
       <c r="A16" s="5"/>
-      <c r="B16" s="48"/>
-      <c r="C16" s="48"/>
-      <c r="D16" s="48"/>
+      <c r="B16" s="50"/>
+      <c r="C16" s="50"/>
+      <c r="D16" s="50"/>
     </row>
     <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="54" t="s">
+      <c r="A17" s="56" t="s">
         <v>171</v>
       </c>
-      <c r="B17" s="55" t="s">
+      <c r="B17" s="57" t="s">
         <v>172</v>
       </c>
-      <c r="C17" s="56" t="s">
+      <c r="C17" s="58" t="s">
         <v>173</v>
       </c>
-      <c r="D17" s="57" t="s">
+      <c r="D17" s="59" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="54"/>
-      <c r="B18" s="55" t="s">
+      <c r="A18" s="56"/>
+      <c r="B18" s="57" t="s">
         <v>175</v>
       </c>
-      <c r="C18" s="56">
+      <c r="C18" s="58">
         <v>5000</v>
       </c>
-      <c r="D18" s="56" t="s">
+      <c r="D18" s="58" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="54"/>
-      <c r="B19" s="55" t="s">
+      <c r="A19" s="56"/>
+      <c r="B19" s="57" t="s">
         <v>177</v>
       </c>
-      <c r="C19" s="56" t="s">
+      <c r="C19" s="58" t="s">
         <v>165</v>
       </c>
-      <c r="D19" s="56" t="s">
+      <c r="D19" s="58" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="20" ht="28.199999999999999" customHeight="1">
-      <c r="B20" s="42"/>
+      <c r="B20" s="44"/>
     </row>
     <row r="21" ht="28.199999999999999" customHeight="1"/>
     <row r="22" ht="28.199999999999999" customHeight="1"/>

</xml_diff>